<commit_message>
Publish current dashboard data and add one-command release
</commit_message>
<xml_diff>
--- a/tongji_target.xlsx
+++ b/tongji_target.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$117</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="34">
   <si>
     <t>期次</t>
   </si>
@@ -129,6 +129,9 @@
   </si>
   <si>
     <t>暑_9</t>
+  </si>
+  <si>
+    <t>暑_12</t>
   </si>
 </sst>
 </file>
@@ -904,7 +907,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1021,14 +1024,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
@@ -1038,46 +1033,6 @@
       </extLst>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
@@ -1619,7 +1574,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H102"/>
+  <dimension ref="A1:H117"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.3076923076923" style="1" customWidth="1"/>
@@ -3414,7 +3369,7 @@
       <c r="E69" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F69" s="22">
+      <c r="F69" s="8">
         <v>130</v>
       </c>
       <c r="G69" s="9">
@@ -3440,7 +3395,7 @@
       <c r="E70" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F70" s="22">
+      <c r="F70" s="8">
         <v>120</v>
       </c>
       <c r="G70" s="9">
@@ -3466,7 +3421,7 @@
       <c r="E71" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F71" s="22">
+      <c r="F71" s="8">
         <v>130</v>
       </c>
       <c r="G71" s="9">
@@ -3492,7 +3447,7 @@
       <c r="E72" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F72" s="23">
+      <c r="F72" s="22">
         <v>800</v>
       </c>
       <c r="G72" s="9">
@@ -3518,7 +3473,7 @@
       <c r="E73" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F73" s="23">
+      <c r="F73" s="22">
         <v>1000</v>
       </c>
       <c r="G73" s="9">
@@ -3544,7 +3499,7 @@
       <c r="E74" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F74" s="23">
+      <c r="F74" s="22">
         <v>1000</v>
       </c>
       <c r="G74" s="9">
@@ -3570,7 +3525,7 @@
       <c r="E75" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F75" s="23">
+      <c r="F75" s="22">
         <v>100</v>
       </c>
       <c r="G75" s="9">
@@ -3596,7 +3551,7 @@
       <c r="E76" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F76" s="23">
+      <c r="F76" s="22">
         <v>700</v>
       </c>
       <c r="G76" s="9">
@@ -3622,7 +3577,7 @@
       <c r="E77" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F77" s="23">
+      <c r="F77" s="22">
         <v>700</v>
       </c>
       <c r="G77" s="9">
@@ -3648,7 +3603,7 @@
       <c r="E78" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F78" s="24">
+      <c r="F78" s="23">
         <v>220</v>
       </c>
       <c r="G78" s="9">
@@ -3674,7 +3629,7 @@
       <c r="E79" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F79" s="24">
+      <c r="F79" s="23">
         <v>350</v>
       </c>
       <c r="G79" s="9">
@@ -3700,7 +3655,7 @@
       <c r="E80" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F80" s="24">
+      <c r="F80" s="23">
         <v>300</v>
       </c>
       <c r="G80" s="9">
@@ -3726,7 +3681,7 @@
       <c r="E81" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F81" s="25">
+      <c r="F81" s="13">
         <v>650</v>
       </c>
       <c r="G81" s="9">
@@ -3752,7 +3707,7 @@
       <c r="E82" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F82" s="25">
+      <c r="F82" s="13">
         <v>650</v>
       </c>
       <c r="G82" s="9">
@@ -3778,7 +3733,7 @@
       <c r="E83" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F83" s="25">
+      <c r="F83" s="13">
         <v>750</v>
       </c>
       <c r="G83" s="9">
@@ -3804,7 +3759,7 @@
       <c r="E84" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F84" s="25">
+      <c r="F84" s="13">
         <v>950</v>
       </c>
       <c r="G84" s="9">
@@ -3830,7 +3785,7 @@
       <c r="E85" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F85" s="26">
+      <c r="F85" s="11">
         <v>900</v>
       </c>
       <c r="G85" s="9">
@@ -3856,7 +3811,7 @@
       <c r="E86" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F86" s="27">
+      <c r="F86" s="10">
         <v>100</v>
       </c>
       <c r="G86" s="9">
@@ -3882,7 +3837,7 @@
       <c r="E87" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="F87" s="28">
+      <c r="F87" s="15">
         <v>230</v>
       </c>
       <c r="G87" s="9">
@@ -3908,7 +3863,7 @@
       <c r="E88" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F88" s="28">
+      <c r="F88" s="15">
         <v>330</v>
       </c>
       <c r="G88" s="9">
@@ -3934,7 +3889,7 @@
       <c r="E89" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F89" s="28">
+      <c r="F89" s="15">
         <v>330</v>
       </c>
       <c r="G89" s="9">
@@ -3960,7 +3915,7 @@
       <c r="E90" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F90" s="28">
+      <c r="F90" s="15">
         <v>420</v>
       </c>
       <c r="G90" s="9">
@@ -3986,7 +3941,7 @@
       <c r="E91" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="F91" s="28">
+      <c r="F91" s="15">
         <v>150</v>
       </c>
       <c r="G91" s="9">
@@ -4012,7 +3967,7 @@
       <c r="E92" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F92" s="28">
+      <c r="F92" s="15">
         <v>350</v>
       </c>
       <c r="G92" s="9">
@@ -4038,7 +3993,7 @@
       <c r="E93" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F93" s="28">
+      <c r="F93" s="15">
         <v>250</v>
       </c>
       <c r="G93" s="9">
@@ -4064,7 +4019,7 @@
       <c r="E94" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F94" s="28">
+      <c r="F94" s="15">
         <v>250</v>
       </c>
       <c r="G94" s="9">
@@ -4090,7 +4045,7 @@
       <c r="E95" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="F95" s="27">
+      <c r="F95" s="10">
         <v>20</v>
       </c>
       <c r="G95" s="9">
@@ -4116,7 +4071,7 @@
       <c r="E96" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F96" s="27">
+      <c r="F96" s="10">
         <v>110</v>
       </c>
       <c r="G96" s="9">
@@ -4142,7 +4097,7 @@
       <c r="E97" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F97" s="27">
+      <c r="F97" s="10">
         <v>110</v>
       </c>
       <c r="G97" s="9">
@@ -4168,7 +4123,7 @@
       <c r="E98" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F98" s="27">
+      <c r="F98" s="10">
         <v>110</v>
       </c>
       <c r="G98" s="9">
@@ -4194,7 +4149,7 @@
       <c r="E99" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="F99" s="29">
+      <c r="F99" s="16">
         <v>2520</v>
       </c>
       <c r="G99" s="9">
@@ -4220,7 +4175,7 @@
       <c r="E100" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F100" s="29">
+      <c r="F100" s="16">
         <v>2720</v>
       </c>
       <c r="G100" s="9">
@@ -4246,7 +4201,7 @@
       <c r="E101" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F101" s="29">
+      <c r="F101" s="16">
         <v>2530</v>
       </c>
       <c r="G101" s="9">
@@ -4272,7 +4227,7 @@
       <c r="E102" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F102" s="29">
+      <c r="F102" s="16">
         <v>2050</v>
       </c>
       <c r="G102" s="9">
@@ -4282,12 +4237,402 @@
         <v>46205</v>
       </c>
     </row>
+    <row r="103" ht="17" hidden="1" spans="1:8">
+      <c r="A103" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B103" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C103" s="7">
+        <v>0</v>
+      </c>
+      <c r="D103" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E103" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F103" s="18">
+        <v>70</v>
+      </c>
+      <c r="G103" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H103" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="104" ht="17" hidden="1" spans="1:8">
+      <c r="A104" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B104" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C104" s="7">
+        <v>0</v>
+      </c>
+      <c r="D104" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E104" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F104" s="17">
+        <v>140</v>
+      </c>
+      <c r="G104" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H104" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="105" ht="17" hidden="1" spans="1:8">
+      <c r="A105" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B105" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C105" s="7">
+        <v>0</v>
+      </c>
+      <c r="D105" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E105" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F105" s="17">
+        <v>140</v>
+      </c>
+      <c r="G105" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H105" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="106" ht="17" hidden="1" spans="1:8">
+      <c r="A106" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B106" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C106" s="7">
+        <v>100</v>
+      </c>
+      <c r="D106" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E106" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F106" s="18">
+        <v>335</v>
+      </c>
+      <c r="G106" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H106" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="107" ht="17" hidden="1" spans="1:8">
+      <c r="A107" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B107" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C107" s="7">
+        <v>100</v>
+      </c>
+      <c r="D107" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E107" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F107" s="16">
+        <v>980</v>
+      </c>
+      <c r="G107" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H107" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="108" ht="17" hidden="1" spans="1:8">
+      <c r="A108" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B108" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C108" s="7">
+        <v>100</v>
+      </c>
+      <c r="D108" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E108" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F108" s="18">
+        <v>1240</v>
+      </c>
+      <c r="G108" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H108" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="109" ht="17" hidden="1" spans="1:8">
+      <c r="A109" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C109" s="7">
+        <v>2880</v>
+      </c>
+      <c r="D109" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E109" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F109" s="10">
+        <v>0</v>
+      </c>
+      <c r="G109" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H109" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="110" ht="17" hidden="1" spans="1:8">
+      <c r="A110" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B110" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C110" s="7">
+        <v>2880</v>
+      </c>
+      <c r="D110" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E110" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F110" s="10">
+        <v>150</v>
+      </c>
+      <c r="G110" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H110" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="111" ht="17" hidden="1" spans="1:8">
+      <c r="A111" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B111" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C111" s="7">
+        <v>2880</v>
+      </c>
+      <c r="D111" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E111" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F111" s="10">
+        <v>485</v>
+      </c>
+      <c r="G111" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H111" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="112" ht="17" hidden="1" spans="1:8">
+      <c r="A112" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B112" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C112" s="7">
+        <v>2880</v>
+      </c>
+      <c r="D112" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E112" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F112" s="18">
+        <v>0</v>
+      </c>
+      <c r="G112" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H112" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="113" ht="17" hidden="1" spans="1:8">
+      <c r="A113" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B113" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C113" s="7">
+        <v>2880</v>
+      </c>
+      <c r="D113" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E113" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F113" s="16">
+        <v>300</v>
+      </c>
+      <c r="G113" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H113" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="114" ht="17" hidden="1" spans="1:8">
+      <c r="A114" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B114" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C114" s="7">
+        <v>2880</v>
+      </c>
+      <c r="D114" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E114" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F114" s="16">
+        <v>500</v>
+      </c>
+      <c r="G114" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H114" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="115" ht="17" hidden="1" spans="1:8">
+      <c r="A115" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B115" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C115" s="19">
+        <v>990</v>
+      </c>
+      <c r="D115" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E115" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F115" s="20">
+        <v>100</v>
+      </c>
+      <c r="G115" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H115" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="116" ht="17" hidden="1" spans="1:8">
+      <c r="A116" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B116" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C116" s="19">
+        <v>990</v>
+      </c>
+      <c r="D116" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E116" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F116" s="17">
+        <v>800</v>
+      </c>
+      <c r="G116" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H116" s="9">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="117" ht="17" hidden="1" spans="1:8">
+      <c r="A117" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B117" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C117" s="19">
+        <v>990</v>
+      </c>
+      <c r="D117" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E117" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F117" s="20">
+        <v>700</v>
+      </c>
+      <c r="G117" s="9">
+        <v>46212</v>
+      </c>
+      <c r="H117" s="9">
+        <v>46205</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H85" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H117" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="3">
-      <filters>
-        <filter val="小学"/>
-      </filters>
+      <customFilters>
+        <customFilter operator="equal" val="小学"/>
+      </customFilters>
     </filterColumn>
     <extLst/>
   </autoFilter>

</xml_diff>

<commit_message>
Publish dashboard sync retry and latest data
</commit_message>
<xml_diff>
--- a/tongji_target.xlsx
+++ b/tongji_target.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$220</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="36">
   <si>
     <t>期次</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>暑_13</t>
+  </si>
+  <si>
+    <t>暑_14</t>
   </si>
 </sst>
 </file>
@@ -933,7 +936,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1153,6 +1156,22 @@
       </extLst>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
@@ -1700,7 +1719,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H220"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.3076923076923" style="2" customWidth="1"/>
@@ -6495,7 +6514,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="185" ht="17.75" spans="1:8">
+    <row r="185" ht="17" hidden="1" spans="1:8">
       <c r="A185" s="16" t="s">
         <v>25</v>
       </c>
@@ -6511,8 +6530,8 @@
       <c r="E185" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F185" s="12">
-        <v>150</v>
+      <c r="F185" s="37">
+        <v>130</v>
       </c>
       <c r="G185" s="11">
         <v>46225</v>
@@ -6521,7 +6540,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="186" ht="17" spans="1:8">
+    <row r="186" ht="17" hidden="1" spans="1:8">
       <c r="A186" s="16" t="s">
         <v>25</v>
       </c>
@@ -6537,8 +6556,8 @@
       <c r="E186" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F186" s="17">
-        <v>350</v>
+      <c r="F186" s="33">
+        <v>250</v>
       </c>
       <c r="G186" s="11">
         <v>46225</v>
@@ -6547,7 +6566,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="187" ht="17" spans="1:8">
+    <row r="187" ht="17" hidden="1" spans="1:8">
       <c r="A187" s="16" t="s">
         <v>25</v>
       </c>
@@ -6563,7 +6582,7 @@
       <c r="E187" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F187" s="17">
+      <c r="F187" s="33">
         <v>400</v>
       </c>
       <c r="G187" s="11">
@@ -6573,7 +6592,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="188" ht="17" spans="1:8">
+    <row r="188" ht="17" hidden="1" spans="1:8">
       <c r="A188" s="16" t="s">
         <v>25</v>
       </c>
@@ -6589,8 +6608,8 @@
       <c r="E188" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F188" s="17">
-        <v>400</v>
+      <c r="F188" s="33">
+        <v>470</v>
       </c>
       <c r="G188" s="11">
         <v>46225</v>
@@ -6599,7 +6618,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="189" ht="17" spans="1:8">
+    <row r="189" ht="17" hidden="1" spans="1:8">
       <c r="A189" s="16" t="s">
         <v>25</v>
       </c>
@@ -6615,7 +6634,7 @@
       <c r="E189" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F189" s="17">
+      <c r="F189" s="33">
         <v>600</v>
       </c>
       <c r="G189" s="11">
@@ -6625,7 +6644,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="190" ht="17" spans="1:8">
+    <row r="190" ht="17" hidden="1" spans="1:8">
       <c r="A190" s="16" t="s">
         <v>25</v>
       </c>
@@ -6641,7 +6660,7 @@
       <c r="E190" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F190" s="17">
+      <c r="F190" s="33">
         <v>150</v>
       </c>
       <c r="G190" s="11">
@@ -6651,7 +6670,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="191" ht="17" spans="1:8">
+    <row r="191" ht="17" hidden="1" spans="1:8">
       <c r="A191" s="16" t="s">
         <v>25</v>
       </c>
@@ -6667,7 +6686,7 @@
       <c r="E191" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F191" s="17">
+      <c r="F191" s="33">
         <v>350</v>
       </c>
       <c r="G191" s="11">
@@ -6677,7 +6696,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="192" ht="17" spans="1:8">
+    <row r="192" ht="17" hidden="1" spans="1:8">
       <c r="A192" s="16" t="s">
         <v>25</v>
       </c>
@@ -6693,7 +6712,7 @@
       <c r="E192" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F192" s="17">
+      <c r="F192" s="33">
         <v>250</v>
       </c>
       <c r="G192" s="11">
@@ -6703,7 +6722,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="193" ht="17" spans="1:8">
+    <row r="193" ht="17" hidden="1" spans="1:8">
       <c r="A193" s="16" t="s">
         <v>25</v>
       </c>
@@ -6719,7 +6738,7 @@
       <c r="E193" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F193" s="17">
+      <c r="F193" s="33">
         <v>250</v>
       </c>
       <c r="G193" s="11">
@@ -6729,7 +6748,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="194" ht="17" spans="1:8">
+    <row r="194" ht="17" hidden="1" spans="1:8">
       <c r="A194" s="16" t="s">
         <v>25</v>
       </c>
@@ -6745,8 +6764,8 @@
       <c r="E194" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F194" s="12">
-        <v>20</v>
+      <c r="F194" s="37">
+        <v>30</v>
       </c>
       <c r="G194" s="11">
         <v>46225</v>
@@ -6755,7 +6774,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="195" ht="17" spans="1:8">
+    <row r="195" ht="17" hidden="1" spans="1:8">
       <c r="A195" s="16" t="s">
         <v>25</v>
       </c>
@@ -6771,8 +6790,8 @@
       <c r="E195" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F195" s="12">
-        <v>110</v>
+      <c r="F195" s="37">
+        <v>140</v>
       </c>
       <c r="G195" s="11">
         <v>46225</v>
@@ -6781,7 +6800,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="196" ht="17" spans="1:8">
+    <row r="196" ht="17" hidden="1" spans="1:8">
       <c r="A196" s="16" t="s">
         <v>25</v>
       </c>
@@ -6797,8 +6816,8 @@
       <c r="E196" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F196" s="12">
-        <v>110</v>
+      <c r="F196" s="37">
+        <v>140</v>
       </c>
       <c r="G196" s="11">
         <v>46225</v>
@@ -6807,7 +6826,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="197" ht="17" spans="1:8">
+    <row r="197" ht="17" hidden="1" spans="1:8">
       <c r="A197" s="16" t="s">
         <v>25</v>
       </c>
@@ -6823,8 +6842,8 @@
       <c r="E197" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F197" s="12">
-        <v>110</v>
+      <c r="F197" s="37">
+        <v>140</v>
       </c>
       <c r="G197" s="11">
         <v>46225</v>
@@ -6833,7 +6852,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="198" ht="17" spans="1:8">
+    <row r="198" ht="17" hidden="1" spans="1:8">
       <c r="A198" s="16" t="s">
         <v>25</v>
       </c>
@@ -6849,8 +6868,8 @@
       <c r="E198" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F198" s="18">
-        <v>3120</v>
+      <c r="F198" s="33">
+        <v>1400</v>
       </c>
       <c r="G198" s="11">
         <v>46225</v>
@@ -6859,7 +6878,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="199" ht="17" spans="1:8">
+    <row r="199" ht="17" hidden="1" spans="1:8">
       <c r="A199" s="16" t="s">
         <v>25</v>
       </c>
@@ -6875,8 +6894,8 @@
       <c r="E199" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F199" s="18">
-        <v>3020</v>
+      <c r="F199" s="33">
+        <v>1550</v>
       </c>
       <c r="G199" s="11">
         <v>46225</v>
@@ -6885,7 +6904,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="200" ht="17" spans="1:8">
+    <row r="200" ht="17" hidden="1" spans="1:8">
       <c r="A200" s="16" t="s">
         <v>25</v>
       </c>
@@ -6901,8 +6920,8 @@
       <c r="E200" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F200" s="18">
-        <v>2930</v>
+      <c r="F200" s="33">
+        <v>1650</v>
       </c>
       <c r="G200" s="11">
         <v>46225</v>
@@ -6911,7 +6930,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="201" ht="17" spans="1:8">
+    <row r="201" ht="17" hidden="1" spans="1:8">
       <c r="A201" s="16" t="s">
         <v>25</v>
       </c>
@@ -6927,8 +6946,8 @@
       <c r="E201" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F201" s="18">
-        <v>2930</v>
+      <c r="F201" s="33">
+        <v>1300</v>
       </c>
       <c r="G201" s="11">
         <v>46225</v>
@@ -6937,17 +6956,511 @@
         <v>46219</v>
       </c>
     </row>
+    <row r="202" ht="17" hidden="1" spans="1:8">
+      <c r="A202" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B202" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C202" s="9">
+        <v>990</v>
+      </c>
+      <c r="D202" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E202" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F202" s="33">
+        <v>150</v>
+      </c>
+      <c r="G202" s="11">
+        <v>46225</v>
+      </c>
+      <c r="H202" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="203" ht="17" hidden="1" spans="1:8">
+      <c r="A203" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B203" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C203" s="9">
+        <v>990</v>
+      </c>
+      <c r="D203" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E203" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F203" s="33">
+        <v>150</v>
+      </c>
+      <c r="G203" s="11">
+        <v>46225</v>
+      </c>
+      <c r="H203" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="204" ht="17" hidden="1" spans="1:8">
+      <c r="A204" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B204" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C204" s="9">
+        <v>990</v>
+      </c>
+      <c r="D204" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E204" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F204" s="33">
+        <v>150</v>
+      </c>
+      <c r="G204" s="11">
+        <v>46225</v>
+      </c>
+      <c r="H204" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="205" ht="17" hidden="1" spans="1:8">
+      <c r="A205" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B205" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C205" s="9">
+        <v>990</v>
+      </c>
+      <c r="D205" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E205" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F205" s="33">
+        <v>150</v>
+      </c>
+      <c r="G205" s="11">
+        <v>46225</v>
+      </c>
+      <c r="H205" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="206" ht="17" spans="1:8">
+      <c r="A206" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B206" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C206" s="9">
+        <v>0</v>
+      </c>
+      <c r="D206" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E206" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F206" s="37">
+        <v>100</v>
+      </c>
+      <c r="G206" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H206" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="207" ht="17" spans="1:8">
+      <c r="A207" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B207" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C207" s="9">
+        <v>0</v>
+      </c>
+      <c r="D207" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E207" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F207" s="37">
+        <v>200</v>
+      </c>
+      <c r="G207" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H207" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="208" ht="17" spans="1:8">
+      <c r="A208" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B208" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C208" s="9">
+        <v>0</v>
+      </c>
+      <c r="D208" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E208" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F208" s="37">
+        <v>200</v>
+      </c>
+      <c r="G208" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H208" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="209" ht="17" spans="1:8">
+      <c r="A209" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B209" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C209" s="9">
+        <v>100</v>
+      </c>
+      <c r="D209" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E209" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F209" s="38">
+        <v>200</v>
+      </c>
+      <c r="G209" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H209" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="210" ht="17" spans="1:8">
+      <c r="A210" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B210" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C210" s="9">
+        <v>100</v>
+      </c>
+      <c r="D210" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E210" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F210" s="38">
+        <v>1300</v>
+      </c>
+      <c r="G210" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H210" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="211" ht="17" spans="1:8">
+      <c r="A211" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B211" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C211" s="9">
+        <v>100</v>
+      </c>
+      <c r="D211" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E211" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F211" s="38">
+        <v>1300</v>
+      </c>
+      <c r="G211" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H211" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="212" ht="17" spans="1:8">
+      <c r="A212" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B212" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C212" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D212" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E212" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F212" s="12">
+        <v>0</v>
+      </c>
+      <c r="G212" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H212" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="213" ht="17" spans="1:8">
+      <c r="A213" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B213" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C213" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D213" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E213" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F213" s="37">
+        <v>450</v>
+      </c>
+      <c r="G213" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H213" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="214" ht="17" spans="1:8">
+      <c r="A214" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B214" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C214" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D214" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E214" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F214" s="37">
+        <v>450</v>
+      </c>
+      <c r="G214" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H214" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="215" ht="17" spans="1:8">
+      <c r="A215" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B215" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C215" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D215" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E215" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F215" s="20">
+        <v>0</v>
+      </c>
+      <c r="G215" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H215" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="216" ht="17" spans="1:8">
+      <c r="A216" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B216" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C216" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D216" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E216" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F216" s="37">
+        <v>650</v>
+      </c>
+      <c r="G216" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H216" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="217" ht="17" spans="1:8">
+      <c r="A217" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B217" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C217" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D217" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E217" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F217" s="37">
+        <v>750</v>
+      </c>
+      <c r="G217" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H217" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="218" ht="17" spans="1:8">
+      <c r="A218" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B218" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C218" s="21">
+        <v>990</v>
+      </c>
+      <c r="D218" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E218" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F218" s="22">
+        <v>100</v>
+      </c>
+      <c r="G218" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H218" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="219" ht="17" spans="1:8">
+      <c r="A219" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B219" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C219" s="21">
+        <v>990</v>
+      </c>
+      <c r="D219" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E219" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F219" s="19">
+        <v>600</v>
+      </c>
+      <c r="G219" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H219" s="11">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="220" ht="17" spans="1:8">
+      <c r="A220" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B220" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C220" s="21">
+        <v>990</v>
+      </c>
+      <c r="D220" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E220" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F220" s="22">
+        <v>980</v>
+      </c>
+      <c r="G220" s="11">
+        <v>46219</v>
+      </c>
+      <c r="H220" s="11">
+        <v>46212</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H201" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H220" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
       <filters>
-        <filter val="暑_11"/>
+        <filter val="暑_14"/>
       </filters>
     </filterColumn>
     <filterColumn colId="3">
-      <filters>
-        <filter val="小学"/>
-      </filters>
+      <customFilters>
+        <customFilter operator="equal" val="高中"/>
+      </customFilters>
     </filterColumn>
     <extLst/>
   </autoFilter>

</xml_diff>

<commit_message>
Stabilize online dashboard sync
</commit_message>
<xml_diff>
--- a/tongji_target.xlsx
+++ b/tongji_target.xlsx
@@ -1756,7 +1756,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" hidden="1" spans="1:8">
+    <row r="2" ht="17.55" hidden="1" spans="1:8">
       <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
@@ -7060,7 +7060,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="206" ht="17" spans="1:8">
+    <row r="206" ht="17.75" spans="1:8">
       <c r="A206" s="16" t="s">
         <v>35</v>
       </c>
@@ -7080,10 +7080,10 @@
         <v>100</v>
       </c>
       <c r="G206" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H206" s="11">
         <v>46219</v>
-      </c>
-      <c r="H206" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="207" ht="17" spans="1:8">
@@ -7106,10 +7106,10 @@
         <v>200</v>
       </c>
       <c r="G207" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H207" s="11">
         <v>46219</v>
-      </c>
-      <c r="H207" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="208" ht="17" spans="1:8">
@@ -7132,10 +7132,10 @@
         <v>200</v>
       </c>
       <c r="G208" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H208" s="11">
         <v>46219</v>
-      </c>
-      <c r="H208" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="209" ht="17" spans="1:8">
@@ -7158,10 +7158,10 @@
         <v>200</v>
       </c>
       <c r="G209" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H209" s="11">
         <v>46219</v>
-      </c>
-      <c r="H209" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="210" ht="17" spans="1:8">
@@ -7184,10 +7184,10 @@
         <v>1300</v>
       </c>
       <c r="G210" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H210" s="11">
         <v>46219</v>
-      </c>
-      <c r="H210" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="211" ht="17" spans="1:8">
@@ -7210,10 +7210,10 @@
         <v>1300</v>
       </c>
       <c r="G211" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H211" s="11">
         <v>46219</v>
-      </c>
-      <c r="H211" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="212" ht="17" spans="1:8">
@@ -7236,10 +7236,10 @@
         <v>0</v>
       </c>
       <c r="G212" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H212" s="11">
         <v>46219</v>
-      </c>
-      <c r="H212" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="213" ht="17" spans="1:8">
@@ -7262,10 +7262,10 @@
         <v>450</v>
       </c>
       <c r="G213" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H213" s="11">
         <v>46219</v>
-      </c>
-      <c r="H213" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="214" ht="17" spans="1:8">
@@ -7288,10 +7288,10 @@
         <v>450</v>
       </c>
       <c r="G214" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H214" s="11">
         <v>46219</v>
-      </c>
-      <c r="H214" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="215" ht="17" spans="1:8">
@@ -7314,10 +7314,10 @@
         <v>0</v>
       </c>
       <c r="G215" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H215" s="11">
         <v>46219</v>
-      </c>
-      <c r="H215" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="216" ht="17" spans="1:8">
@@ -7340,10 +7340,10 @@
         <v>650</v>
       </c>
       <c r="G216" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H216" s="11">
         <v>46219</v>
-      </c>
-      <c r="H216" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="217" ht="17" spans="1:8">
@@ -7366,10 +7366,10 @@
         <v>750</v>
       </c>
       <c r="G217" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H217" s="11">
         <v>46219</v>
-      </c>
-      <c r="H217" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="218" ht="17" spans="1:8">
@@ -7392,10 +7392,10 @@
         <v>100</v>
       </c>
       <c r="G218" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H218" s="11">
         <v>46219</v>
-      </c>
-      <c r="H218" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="219" ht="17" spans="1:8">
@@ -7418,10 +7418,10 @@
         <v>600</v>
       </c>
       <c r="G219" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H219" s="11">
         <v>46219</v>
-      </c>
-      <c r="H219" s="11">
-        <v>46212</v>
       </c>
     </row>
     <row r="220" ht="17" spans="1:8">
@@ -7444,18 +7444,18 @@
         <v>980</v>
       </c>
       <c r="G220" s="11">
+        <v>46226</v>
+      </c>
+      <c r="H220" s="11">
         <v>46219</v>
-      </c>
-      <c r="H220" s="11">
-        <v>46212</v>
       </c>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H220" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
-      <filters>
-        <filter val="暑_14"/>
-      </filters>
+      <customFilters>
+        <customFilter operator="equal" val="暑_14"/>
+      </customFilters>
     </filterColumn>
     <filterColumn colId="3">
       <customFilters>

</xml_diff>

<commit_message>
Show self-study current intake in detail table
</commit_message>
<xml_diff>
--- a/tongji_target.xlsx
+++ b/tongji_target.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$220</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$236</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="37">
   <si>
     <t>期次</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>暑_14</t>
+  </si>
+  <si>
+    <t>秋_1</t>
   </si>
 </sst>
 </file>
@@ -936,7 +939,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1131,6 +1134,14 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
@@ -1172,6 +1183,30 @@
       </extLst>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
@@ -1719,7 +1754,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H220"/>
+  <dimension ref="A1:H236"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.3076923076923" style="2" customWidth="1"/>
@@ -1756,7 +1791,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="17.55" hidden="1" spans="1:8">
+    <row r="2" ht="17.55" spans="1:8">
       <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
@@ -1782,7 +1817,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="3" hidden="1" spans="1:8">
+    <row r="3" spans="1:8">
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
@@ -1808,7 +1843,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="4" hidden="1" spans="1:8">
+    <row r="4" spans="1:8">
       <c r="A4" s="7" t="s">
         <v>8</v>
       </c>
@@ -1834,7 +1869,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="5" ht="17" hidden="1" spans="1:8">
+    <row r="5" ht="17" spans="1:8">
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
@@ -1860,7 +1895,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="6" ht="17" hidden="1" spans="1:8">
+    <row r="6" ht="17" spans="1:8">
       <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
@@ -1886,7 +1921,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="7" ht="17" hidden="1" spans="1:8">
+    <row r="7" ht="17" spans="1:8">
       <c r="A7" s="7" t="s">
         <v>8</v>
       </c>
@@ -1912,7 +1947,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="8" hidden="1" spans="1:8">
+    <row r="8" spans="1:8">
       <c r="A8" s="7" t="s">
         <v>8</v>
       </c>
@@ -1938,7 +1973,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="9" hidden="1" spans="1:8">
+    <row r="9" spans="1:8">
       <c r="A9" s="7" t="s">
         <v>8</v>
       </c>
@@ -1964,7 +1999,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="10" hidden="1" spans="1:8">
+    <row r="10" spans="1:8">
       <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
@@ -1990,7 +2025,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="11" hidden="1" spans="1:8">
+    <row r="11" spans="1:8">
       <c r="A11" s="7" t="s">
         <v>8</v>
       </c>
@@ -2016,7 +2051,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="12" hidden="1" spans="1:8">
+    <row r="12" spans="1:8">
       <c r="A12" s="7" t="s">
         <v>8</v>
       </c>
@@ -2042,7 +2077,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="13" hidden="1" spans="1:8">
+    <row r="13" spans="1:8">
       <c r="A13" s="7" t="s">
         <v>8</v>
       </c>
@@ -2068,7 +2103,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="14" ht="17" hidden="1" spans="1:8">
+    <row r="14" ht="17" spans="1:8">
       <c r="A14" s="7" t="s">
         <v>8</v>
       </c>
@@ -2094,7 +2129,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="15" ht="17" hidden="1" spans="1:8">
+    <row r="15" ht="17" spans="1:8">
       <c r="A15" s="7" t="s">
         <v>8</v>
       </c>
@@ -2120,7 +2155,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="16" ht="17" hidden="1" spans="1:8">
+    <row r="16" ht="17" spans="1:8">
       <c r="A16" s="7" t="s">
         <v>8</v>
       </c>
@@ -2146,7 +2181,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="17" hidden="1" spans="1:8">
+    <row r="17" spans="1:8">
       <c r="A17" s="7" t="s">
         <v>8</v>
       </c>
@@ -2172,7 +2207,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="18" hidden="1" spans="1:8">
+    <row r="18" spans="1:8">
       <c r="A18" s="7" t="s">
         <v>8</v>
       </c>
@@ -2198,7 +2233,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="19" hidden="1" spans="1:8">
+    <row r="19" spans="1:8">
       <c r="A19" s="7" t="s">
         <v>8</v>
       </c>
@@ -2224,7 +2259,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="20" hidden="1" spans="1:8">
+    <row r="20" spans="1:8">
       <c r="A20" s="7" t="s">
         <v>8</v>
       </c>
@@ -2250,7 +2285,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="21" hidden="1" spans="1:8">
+    <row r="21" spans="1:8">
       <c r="A21" s="7" t="s">
         <v>8</v>
       </c>
@@ -3498,7 +3533,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="69" hidden="1" spans="1:8">
+    <row r="69" spans="1:8">
       <c r="A69" s="7" t="s">
         <v>25</v>
       </c>
@@ -3524,7 +3559,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="70" hidden="1" spans="1:8">
+    <row r="70" spans="1:8">
       <c r="A70" s="7" t="s">
         <v>25</v>
       </c>
@@ -3550,7 +3585,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="71" hidden="1" spans="1:8">
+    <row r="71" spans="1:8">
       <c r="A71" s="7" t="s">
         <v>25</v>
       </c>
@@ -3576,7 +3611,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="72" hidden="1" spans="1:8">
+    <row r="72" spans="1:8">
       <c r="A72" s="7" t="s">
         <v>25</v>
       </c>
@@ -3602,7 +3637,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="73" hidden="1" spans="1:8">
+    <row r="73" spans="1:8">
       <c r="A73" s="7" t="s">
         <v>25</v>
       </c>
@@ -3628,7 +3663,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="74" hidden="1" spans="1:8">
+    <row r="74" spans="1:8">
       <c r="A74" s="7" t="s">
         <v>25</v>
       </c>
@@ -3654,7 +3689,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="75" hidden="1" spans="1:8">
+    <row r="75" spans="1:8">
       <c r="A75" s="7" t="s">
         <v>25</v>
       </c>
@@ -3680,7 +3715,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="76" hidden="1" spans="1:8">
+    <row r="76" spans="1:8">
       <c r="A76" s="7" t="s">
         <v>25</v>
       </c>
@@ -3706,7 +3741,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="77" hidden="1" spans="1:8">
+    <row r="77" spans="1:8">
       <c r="A77" s="7" t="s">
         <v>25</v>
       </c>
@@ -3732,7 +3767,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="78" ht="17" hidden="1" spans="1:8">
+    <row r="78" ht="17" spans="1:8">
       <c r="A78" s="7" t="s">
         <v>25</v>
       </c>
@@ -3758,7 +3793,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="79" ht="17" hidden="1" spans="1:8">
+    <row r="79" ht="17" spans="1:8">
       <c r="A79" s="7" t="s">
         <v>25</v>
       </c>
@@ -3784,7 +3819,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="80" ht="17" hidden="1" spans="1:8">
+    <row r="80" ht="17" spans="1:8">
       <c r="A80" s="7" t="s">
         <v>25</v>
       </c>
@@ -3810,7 +3845,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="81" hidden="1" spans="1:8">
+    <row r="81" spans="1:8">
       <c r="A81" s="7" t="s">
         <v>25</v>
       </c>
@@ -3836,7 +3871,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="82" hidden="1" spans="1:8">
+    <row r="82" spans="1:8">
       <c r="A82" s="7" t="s">
         <v>25</v>
       </c>
@@ -3862,7 +3897,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="83" hidden="1" spans="1:8">
+    <row r="83" spans="1:8">
       <c r="A83" s="7" t="s">
         <v>25</v>
       </c>
@@ -3888,7 +3923,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="84" hidden="1" spans="1:8">
+    <row r="84" spans="1:8">
       <c r="A84" s="7" t="s">
         <v>25</v>
       </c>
@@ -3914,7 +3949,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="85" hidden="1" spans="1:8">
+    <row r="85" spans="1:8">
       <c r="A85" s="7" t="s">
         <v>25</v>
       </c>
@@ -5214,7 +5249,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="135" hidden="1" spans="1:8">
+    <row r="135" spans="1:8">
       <c r="A135" s="7" t="s">
         <v>33</v>
       </c>
@@ -5240,7 +5275,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="136" hidden="1" spans="1:8">
+    <row r="136" spans="1:8">
       <c r="A136" s="7" t="s">
         <v>33</v>
       </c>
@@ -5266,7 +5301,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="137" hidden="1" spans="1:8">
+    <row r="137" spans="1:8">
       <c r="A137" s="7" t="s">
         <v>33</v>
       </c>
@@ -5292,7 +5327,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="138" s="1" customFormat="1" hidden="1" spans="1:8">
+    <row r="138" s="1" customFormat="1" spans="1:8">
       <c r="A138" s="7" t="s">
         <v>33</v>
       </c>
@@ -5318,7 +5353,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="139" s="1" customFormat="1" hidden="1" spans="1:8">
+    <row r="139" s="1" customFormat="1" spans="1:8">
       <c r="A139" s="7" t="s">
         <v>33</v>
       </c>
@@ -5344,7 +5379,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="140" s="1" customFormat="1" hidden="1" spans="1:8">
+    <row r="140" s="1" customFormat="1" spans="1:8">
       <c r="A140" s="7" t="s">
         <v>33</v>
       </c>
@@ -5370,7 +5405,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="141" s="1" customFormat="1" hidden="1" spans="1:8">
+    <row r="141" s="1" customFormat="1" spans="1:8">
       <c r="A141" s="7" t="s">
         <v>33</v>
       </c>
@@ -5396,7 +5431,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="142" s="1" customFormat="1" hidden="1" spans="1:8">
+    <row r="142" s="1" customFormat="1" spans="1:8">
       <c r="A142" s="7" t="s">
         <v>33</v>
       </c>
@@ -5422,7 +5457,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="143" s="1" customFormat="1" hidden="1" spans="1:8">
+    <row r="143" s="1" customFormat="1" spans="1:8">
       <c r="A143" s="7" t="s">
         <v>33</v>
       </c>
@@ -5448,7 +5483,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="144" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
+    <row r="144" s="1" customFormat="1" ht="17" spans="1:8">
       <c r="A144" s="7" t="s">
         <v>33</v>
       </c>
@@ -5474,7 +5509,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="145" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
+    <row r="145" s="1" customFormat="1" ht="17" spans="1:8">
       <c r="A145" s="7" t="s">
         <v>33</v>
       </c>
@@ -5500,7 +5535,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="146" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
+    <row r="146" s="1" customFormat="1" ht="17" spans="1:8">
       <c r="A146" s="7" t="s">
         <v>33</v>
       </c>
@@ -5526,7 +5561,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="147" s="1" customFormat="1" hidden="1" spans="1:8">
+    <row r="147" s="1" customFormat="1" spans="1:8">
       <c r="A147" s="7" t="s">
         <v>33</v>
       </c>
@@ -5552,7 +5587,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="148" hidden="1" spans="1:8">
+    <row r="148" spans="1:8">
       <c r="A148" s="7" t="s">
         <v>33</v>
       </c>
@@ -5578,7 +5613,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="149" hidden="1" spans="1:8">
+    <row r="149" spans="1:8">
       <c r="A149" s="7" t="s">
         <v>33</v>
       </c>
@@ -5604,7 +5639,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="150" hidden="1" spans="1:8">
+    <row r="150" spans="1:8">
       <c r="A150" s="7" t="s">
         <v>33</v>
       </c>
@@ -5630,7 +5665,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="151" hidden="1" spans="1:8">
+    <row r="151" spans="1:8">
       <c r="A151" s="7" t="s">
         <v>33</v>
       </c>
@@ -6046,7 +6081,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="167" hidden="1" spans="1:8">
+    <row r="167" spans="1:8">
       <c r="A167" s="7" t="s">
         <v>34</v>
       </c>
@@ -6072,7 +6107,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="168" hidden="1" spans="1:8">
+    <row r="168" spans="1:8">
       <c r="A168" s="7" t="s">
         <v>34</v>
       </c>
@@ -6098,7 +6133,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="169" hidden="1" spans="1:8">
+    <row r="169" spans="1:8">
       <c r="A169" s="7" t="s">
         <v>34</v>
       </c>
@@ -6124,7 +6159,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="170" hidden="1" spans="1:8">
+    <row r="170" spans="1:8">
       <c r="A170" s="7" t="s">
         <v>34</v>
       </c>
@@ -6132,7 +6167,7 @@
         <v>14</v>
       </c>
       <c r="C170" s="9">
-        <v>990</v>
+        <v>1880</v>
       </c>
       <c r="D170" s="8" t="s">
         <v>10</v>
@@ -6141,7 +6176,7 @@
         <v>11</v>
       </c>
       <c r="F170" s="32">
-        <v>60</v>
+        <v>600</v>
       </c>
       <c r="G170" s="11">
         <v>46224</v>
@@ -6150,7 +6185,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="171" hidden="1" spans="1:8">
+    <row r="171" spans="1:8">
       <c r="A171" s="7" t="s">
         <v>34</v>
       </c>
@@ -6158,16 +6193,16 @@
         <v>14</v>
       </c>
       <c r="C171" s="9">
-        <v>1880</v>
+        <v>990</v>
       </c>
       <c r="D171" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E171" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F171" s="32">
-        <v>540</v>
+        <v>1200</v>
       </c>
       <c r="G171" s="11">
         <v>46224</v>
@@ -6176,7 +6211,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="172" hidden="1" spans="1:8">
+    <row r="172" spans="1:8">
       <c r="A172" s="7" t="s">
         <v>34</v>
       </c>
@@ -6190,7 +6225,7 @@
         <v>10</v>
       </c>
       <c r="E172" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F172" s="32">
         <v>1200</v>
@@ -6202,12 +6237,12 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="173" hidden="1" spans="1:8">
+    <row r="173" spans="1:8">
       <c r="A173" s="7" t="s">
         <v>34</v>
       </c>
       <c r="B173" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C173" s="9">
         <v>990</v>
@@ -6216,10 +6251,10 @@
         <v>10</v>
       </c>
       <c r="E173" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F173" s="32">
-        <v>1200</v>
+        <v>11</v>
+      </c>
+      <c r="F173" s="33">
+        <v>150</v>
       </c>
       <c r="G173" s="11">
         <v>46224</v>
@@ -6228,7 +6263,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="174" hidden="1" spans="1:8">
+    <row r="174" spans="1:8">
       <c r="A174" s="7" t="s">
         <v>34</v>
       </c>
@@ -6242,10 +6277,10 @@
         <v>10</v>
       </c>
       <c r="E174" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F174" s="32">
-        <v>150</v>
+        <v>12</v>
+      </c>
+      <c r="F174" s="33">
+        <v>850</v>
       </c>
       <c r="G174" s="11">
         <v>46224</v>
@@ -6254,7 +6289,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="175" hidden="1" spans="1:8">
+    <row r="175" spans="1:8">
       <c r="A175" s="7" t="s">
         <v>34</v>
       </c>
@@ -6268,9 +6303,9 @@
         <v>10</v>
       </c>
       <c r="E175" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F175" s="32">
+        <v>13</v>
+      </c>
+      <c r="F175" s="33">
         <v>850</v>
       </c>
       <c r="G175" s="11">
@@ -6280,12 +6315,12 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="176" hidden="1" spans="1:8">
+    <row r="176" ht="17" spans="1:8">
       <c r="A176" s="7" t="s">
         <v>34</v>
       </c>
       <c r="B176" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C176" s="9">
         <v>990</v>
@@ -6294,10 +6329,10 @@
         <v>10</v>
       </c>
       <c r="E176" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F176" s="32">
-        <v>850</v>
+        <v>11</v>
+      </c>
+      <c r="F176" s="34">
+        <v>210</v>
       </c>
       <c r="G176" s="11">
         <v>46224</v>
@@ -6306,7 +6341,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="177" ht="17" hidden="1" spans="1:8">
+    <row r="177" ht="17" spans="1:8">
       <c r="A177" s="7" t="s">
         <v>34</v>
       </c>
@@ -6314,16 +6349,16 @@
         <v>16</v>
       </c>
       <c r="C177" s="9">
-        <v>990</v>
+        <v>2880</v>
       </c>
       <c r="D177" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E177" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F177" s="33">
-        <v>210</v>
+        <v>12</v>
+      </c>
+      <c r="F177" s="34">
+        <v>230</v>
       </c>
       <c r="G177" s="11">
         <v>46224</v>
@@ -6332,7 +6367,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="178" ht="17" hidden="1" spans="1:8">
+    <row r="178" ht="17" spans="1:8">
       <c r="A178" s="7" t="s">
         <v>34</v>
       </c>
@@ -6346,10 +6381,10 @@
         <v>10</v>
       </c>
       <c r="E178" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F178" s="33">
-        <v>230</v>
+        <v>13</v>
+      </c>
+      <c r="F178" s="34">
+        <v>360</v>
       </c>
       <c r="G178" s="11">
         <v>46224</v>
@@ -6358,24 +6393,24 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="179" ht="17" hidden="1" spans="1:8">
+    <row r="179" spans="1:8">
       <c r="A179" s="7" t="s">
         <v>34</v>
       </c>
       <c r="B179" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C179" s="9">
-        <v>2880</v>
+        <v>100</v>
       </c>
       <c r="D179" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E179" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F179" s="33">
-        <v>360</v>
+        <v>12</v>
+      </c>
+      <c r="F179" s="35">
+        <v>800</v>
       </c>
       <c r="G179" s="11">
         <v>46224</v>
@@ -6384,7 +6419,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="180" hidden="1" spans="1:8">
+    <row r="180" spans="1:8">
       <c r="A180" s="7" t="s">
         <v>34</v>
       </c>
@@ -6400,8 +6435,8 @@
       <c r="E180" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F180" s="34">
-        <v>800</v>
+      <c r="F180" s="35">
+        <v>900</v>
       </c>
       <c r="G180" s="11">
         <v>46224</v>
@@ -6410,7 +6445,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="181" hidden="1" spans="1:8">
+    <row r="181" spans="1:8">
       <c r="A181" s="7" t="s">
         <v>34</v>
       </c>
@@ -6418,16 +6453,16 @@
         <v>17</v>
       </c>
       <c r="C181" s="9">
-        <v>100</v>
+        <v>1880</v>
       </c>
       <c r="D181" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E181" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F181" s="34">
-        <v>900</v>
+        <v>11</v>
+      </c>
+      <c r="F181" s="36">
+        <v>680</v>
       </c>
       <c r="G181" s="11">
         <v>46224</v>
@@ -6436,7 +6471,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="182" hidden="1" spans="1:8">
+    <row r="182" spans="1:8">
       <c r="A182" s="7" t="s">
         <v>34</v>
       </c>
@@ -6444,16 +6479,16 @@
         <v>17</v>
       </c>
       <c r="C182" s="9">
-        <v>1880</v>
+        <v>2880</v>
       </c>
       <c r="D182" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E182" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F182" s="35">
-        <v>680</v>
+        <v>12</v>
+      </c>
+      <c r="F182" s="36">
+        <v>600</v>
       </c>
       <c r="G182" s="11">
         <v>46224</v>
@@ -6462,7 +6497,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="183" hidden="1" spans="1:8">
+    <row r="183" spans="1:8">
       <c r="A183" s="7" t="s">
         <v>34</v>
       </c>
@@ -6478,7 +6513,7 @@
       <c r="E183" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F183" s="35">
+      <c r="F183" s="37">
         <v>600</v>
       </c>
       <c r="G183" s="11">
@@ -6488,9 +6523,9 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="184" hidden="1" spans="1:8">
-      <c r="A184" s="7" t="s">
-        <v>34</v>
+    <row r="184" ht="17" hidden="1" spans="1:8">
+      <c r="A184" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="B184" s="9" t="s">
         <v>17</v>
@@ -6498,20 +6533,20 @@
       <c r="C184" s="9">
         <v>2880</v>
       </c>
-      <c r="D184" s="8" t="s">
-        <v>10</v>
+      <c r="D184" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="E184" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F184" s="36">
-        <v>600</v>
+        <v>20</v>
+      </c>
+      <c r="F184" s="38">
+        <v>130</v>
       </c>
       <c r="G184" s="11">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="H184" s="11">
-        <v>46218</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="185" ht="17" hidden="1" spans="1:8">
@@ -6528,10 +6563,10 @@
         <v>19</v>
       </c>
       <c r="E185" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F185" s="37">
-        <v>130</v>
+        <v>21</v>
+      </c>
+      <c r="F185" s="34">
+        <v>250</v>
       </c>
       <c r="G185" s="11">
         <v>46225</v>
@@ -6554,10 +6589,10 @@
         <v>19</v>
       </c>
       <c r="E186" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F186" s="33">
-        <v>250</v>
+        <v>22</v>
+      </c>
+      <c r="F186" s="34">
+        <v>400</v>
       </c>
       <c r="G186" s="11">
         <v>46225</v>
@@ -6580,10 +6615,10 @@
         <v>19</v>
       </c>
       <c r="E187" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F187" s="33">
-        <v>400</v>
+        <v>23</v>
+      </c>
+      <c r="F187" s="34">
+        <v>470</v>
       </c>
       <c r="G187" s="11">
         <v>46225</v>
@@ -6606,10 +6641,10 @@
         <v>19</v>
       </c>
       <c r="E188" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F188" s="33">
-        <v>470</v>
+        <v>24</v>
+      </c>
+      <c r="F188" s="34">
+        <v>600</v>
       </c>
       <c r="G188" s="11">
         <v>46225</v>
@@ -6623,19 +6658,19 @@
         <v>25</v>
       </c>
       <c r="B189" s="9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C189" s="9">
-        <v>2880</v>
+        <v>990</v>
       </c>
       <c r="D189" s="9" t="s">
         <v>19</v>
       </c>
       <c r="E189" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="F189" s="33">
-        <v>600</v>
+        <v>21</v>
+      </c>
+      <c r="F189" s="34">
+        <v>150</v>
       </c>
       <c r="G189" s="11">
         <v>46225</v>
@@ -6658,10 +6693,10 @@
         <v>19</v>
       </c>
       <c r="E190" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F190" s="33">
-        <v>150</v>
+        <v>22</v>
+      </c>
+      <c r="F190" s="34">
+        <v>350</v>
       </c>
       <c r="G190" s="11">
         <v>46225</v>
@@ -6684,10 +6719,10 @@
         <v>19</v>
       </c>
       <c r="E191" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F191" s="33">
-        <v>350</v>
+        <v>23</v>
+      </c>
+      <c r="F191" s="34">
+        <v>250</v>
       </c>
       <c r="G191" s="11">
         <v>46225</v>
@@ -6710,9 +6745,9 @@
         <v>19</v>
       </c>
       <c r="E192" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F192" s="33">
+        <v>24</v>
+      </c>
+      <c r="F192" s="34">
         <v>250</v>
       </c>
       <c r="G192" s="11">
@@ -6726,20 +6761,20 @@
       <c r="A193" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B193" s="9" t="s">
-        <v>15</v>
+      <c r="B193" s="8" t="s">
+        <v>9</v>
       </c>
       <c r="C193" s="9">
-        <v>990</v>
+        <v>0</v>
       </c>
       <c r="D193" s="9" t="s">
         <v>19</v>
       </c>
       <c r="E193" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="F193" s="33">
-        <v>250</v>
+        <v>21</v>
+      </c>
+      <c r="F193" s="38">
+        <v>30</v>
       </c>
       <c r="G193" s="11">
         <v>46225</v>
@@ -6752,7 +6787,7 @@
       <c r="A194" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B194" s="8" t="s">
+      <c r="B194" s="9" t="s">
         <v>9</v>
       </c>
       <c r="C194" s="9">
@@ -6762,10 +6797,10 @@
         <v>19</v>
       </c>
       <c r="E194" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F194" s="37">
-        <v>30</v>
+        <v>22</v>
+      </c>
+      <c r="F194" s="38">
+        <v>140</v>
       </c>
       <c r="G194" s="11">
         <v>46225</v>
@@ -6788,9 +6823,9 @@
         <v>19</v>
       </c>
       <c r="E195" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F195" s="37">
+        <v>23</v>
+      </c>
+      <c r="F195" s="38">
         <v>140</v>
       </c>
       <c r="G195" s="11">
@@ -6804,7 +6839,7 @@
       <c r="A196" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B196" s="9" t="s">
+      <c r="B196" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C196" s="9">
@@ -6814,9 +6849,9 @@
         <v>19</v>
       </c>
       <c r="E196" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F196" s="37">
+        <v>24</v>
+      </c>
+      <c r="F196" s="38">
         <v>140</v>
       </c>
       <c r="G196" s="11">
@@ -6830,20 +6865,20 @@
       <c r="A197" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B197" s="8" t="s">
-        <v>9</v>
+      <c r="B197" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C197" s="9">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D197" s="9" t="s">
         <v>19</v>
       </c>
       <c r="E197" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="F197" s="37">
-        <v>140</v>
+        <v>21</v>
+      </c>
+      <c r="F197" s="34">
+        <v>1400</v>
       </c>
       <c r="G197" s="11">
         <v>46225</v>
@@ -6866,10 +6901,10 @@
         <v>19</v>
       </c>
       <c r="E198" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F198" s="33">
-        <v>1400</v>
+        <v>22</v>
+      </c>
+      <c r="F198" s="34">
+        <v>1550</v>
       </c>
       <c r="G198" s="11">
         <v>46225</v>
@@ -6892,10 +6927,10 @@
         <v>19</v>
       </c>
       <c r="E199" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F199" s="33">
-        <v>1550</v>
+        <v>23</v>
+      </c>
+      <c r="F199" s="34">
+        <v>1650</v>
       </c>
       <c r="G199" s="11">
         <v>46225</v>
@@ -6918,10 +6953,10 @@
         <v>19</v>
       </c>
       <c r="E200" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F200" s="33">
-        <v>1650</v>
+        <v>24</v>
+      </c>
+      <c r="F200" s="34">
+        <v>1300</v>
       </c>
       <c r="G200" s="11">
         <v>46225</v>
@@ -6938,16 +6973,16 @@
         <v>14</v>
       </c>
       <c r="C201" s="9">
-        <v>100</v>
+        <v>990</v>
       </c>
       <c r="D201" s="9" t="s">
         <v>19</v>
       </c>
       <c r="E201" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="F201" s="33">
-        <v>1300</v>
+        <v>21</v>
+      </c>
+      <c r="F201" s="34">
+        <v>150</v>
       </c>
       <c r="G201" s="11">
         <v>46225</v>
@@ -6970,9 +7005,9 @@
         <v>19</v>
       </c>
       <c r="E202" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F202" s="33">
+        <v>22</v>
+      </c>
+      <c r="F202" s="34">
         <v>150</v>
       </c>
       <c r="G202" s="11">
@@ -6996,9 +7031,9 @@
         <v>19</v>
       </c>
       <c r="E203" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F203" s="33">
+        <v>23</v>
+      </c>
+      <c r="F203" s="34">
         <v>150</v>
       </c>
       <c r="G203" s="11">
@@ -7022,9 +7057,9 @@
         <v>19</v>
       </c>
       <c r="E204" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F204" s="33">
+        <v>24</v>
+      </c>
+      <c r="F204" s="34">
         <v>150</v>
       </c>
       <c r="G204" s="11">
@@ -7036,31 +7071,31 @@
     </row>
     <row r="205" ht="17" hidden="1" spans="1:8">
       <c r="A205" s="16" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B205" s="9" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C205" s="9">
-        <v>990</v>
+        <v>0</v>
       </c>
       <c r="D205" s="9" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E205" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="F205" s="33">
-        <v>150</v>
+        <v>27</v>
+      </c>
+      <c r="F205" s="38">
+        <v>100</v>
       </c>
       <c r="G205" s="11">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="H205" s="11">
         <v>46219</v>
       </c>
     </row>
-    <row r="206" ht="17.75" spans="1:8">
+    <row r="206" ht="17" hidden="1" spans="1:8">
       <c r="A206" s="16" t="s">
         <v>35</v>
       </c>
@@ -7074,10 +7109,10 @@
         <v>26</v>
       </c>
       <c r="E206" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F206" s="37">
-        <v>100</v>
+        <v>28</v>
+      </c>
+      <c r="F206" s="38">
+        <v>200</v>
       </c>
       <c r="G206" s="11">
         <v>46226</v>
@@ -7086,7 +7121,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="207" ht="17" spans="1:8">
+    <row r="207" ht="17" hidden="1" spans="1:8">
       <c r="A207" s="16" t="s">
         <v>35</v>
       </c>
@@ -7100,9 +7135,9 @@
         <v>26</v>
       </c>
       <c r="E207" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F207" s="37">
+        <v>29</v>
+      </c>
+      <c r="F207" s="38">
         <v>200</v>
       </c>
       <c r="G207" s="11">
@@ -7112,23 +7147,23 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="208" ht="17" spans="1:8">
+    <row r="208" ht="17" hidden="1" spans="1:8">
       <c r="A208" s="16" t="s">
         <v>35</v>
       </c>
       <c r="B208" s="9" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C208" s="9">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D208" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E208" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F208" s="37">
+        <v>27</v>
+      </c>
+      <c r="F208" s="39">
         <v>200</v>
       </c>
       <c r="G208" s="11">
@@ -7138,7 +7173,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="209" ht="17" spans="1:8">
+    <row r="209" ht="17" hidden="1" spans="1:8">
       <c r="A209" s="16" t="s">
         <v>35</v>
       </c>
@@ -7152,10 +7187,10 @@
         <v>26</v>
       </c>
       <c r="E209" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F209" s="38">
-        <v>200</v>
+        <v>28</v>
+      </c>
+      <c r="F209" s="39">
+        <v>1300</v>
       </c>
       <c r="G209" s="11">
         <v>46226</v>
@@ -7164,7 +7199,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="210" ht="17" spans="1:8">
+    <row r="210" ht="17" hidden="1" spans="1:8">
       <c r="A210" s="16" t="s">
         <v>35</v>
       </c>
@@ -7178,9 +7213,9 @@
         <v>26</v>
       </c>
       <c r="E210" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F210" s="38">
+        <v>29</v>
+      </c>
+      <c r="F210" s="39">
         <v>1300</v>
       </c>
       <c r="G210" s="11">
@@ -7190,24 +7225,24 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="211" ht="17" spans="1:8">
+    <row r="211" ht="17" hidden="1" spans="1:8">
       <c r="A211" s="16" t="s">
         <v>35</v>
       </c>
       <c r="B211" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C211" s="9">
-        <v>100</v>
+        <v>1880</v>
       </c>
       <c r="D211" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E211" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F211" s="38">
-        <v>1300</v>
+        <v>27</v>
+      </c>
+      <c r="F211" s="12">
+        <v>0</v>
       </c>
       <c r="G211" s="11">
         <v>46226</v>
@@ -7216,7 +7251,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="212" ht="17" spans="1:8">
+    <row r="212" ht="17" hidden="1" spans="1:8">
       <c r="A212" s="16" t="s">
         <v>35</v>
       </c>
@@ -7230,10 +7265,10 @@
         <v>26</v>
       </c>
       <c r="E212" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F212" s="12">
-        <v>0</v>
+        <v>28</v>
+      </c>
+      <c r="F212" s="38">
+        <v>450</v>
       </c>
       <c r="G212" s="11">
         <v>46226</v>
@@ -7242,7 +7277,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="213" ht="17" spans="1:8">
+    <row r="213" ht="17" hidden="1" spans="1:8">
       <c r="A213" s="16" t="s">
         <v>35</v>
       </c>
@@ -7256,9 +7291,9 @@
         <v>26</v>
       </c>
       <c r="E213" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F213" s="37">
+        <v>29</v>
+      </c>
+      <c r="F213" s="38">
         <v>450</v>
       </c>
       <c r="G213" s="11">
@@ -7268,12 +7303,12 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="214" ht="17" spans="1:8">
+    <row r="214" ht="17" hidden="1" spans="1:8">
       <c r="A214" s="16" t="s">
         <v>35</v>
       </c>
       <c r="B214" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C214" s="9">
         <v>1880</v>
@@ -7282,10 +7317,10 @@
         <v>26</v>
       </c>
       <c r="E214" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F214" s="37">
-        <v>450</v>
+        <v>27</v>
+      </c>
+      <c r="F214" s="20">
+        <v>0</v>
       </c>
       <c r="G214" s="11">
         <v>46226</v>
@@ -7294,7 +7329,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="215" ht="17" spans="1:8">
+    <row r="215" ht="17" hidden="1" spans="1:8">
       <c r="A215" s="16" t="s">
         <v>35</v>
       </c>
@@ -7308,10 +7343,10 @@
         <v>26</v>
       </c>
       <c r="E215" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F215" s="20">
-        <v>0</v>
+        <v>28</v>
+      </c>
+      <c r="F215" s="38">
+        <v>650</v>
       </c>
       <c r="G215" s="11">
         <v>46226</v>
@@ -7320,7 +7355,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="216" ht="17" spans="1:8">
+    <row r="216" ht="17" hidden="1" spans="1:8">
       <c r="A216" s="16" t="s">
         <v>35</v>
       </c>
@@ -7334,10 +7369,10 @@
         <v>26</v>
       </c>
       <c r="E216" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F216" s="37">
-        <v>650</v>
+        <v>29</v>
+      </c>
+      <c r="F216" s="38">
+        <v>750</v>
       </c>
       <c r="G216" s="11">
         <v>46226</v>
@@ -7346,24 +7381,24 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="217" ht="17" spans="1:8">
+    <row r="217" ht="17" hidden="1" spans="1:8">
       <c r="A217" s="16" t="s">
         <v>35</v>
       </c>
       <c r="B217" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C217" s="9">
-        <v>1880</v>
+        <v>15</v>
+      </c>
+      <c r="C217" s="21">
+        <v>990</v>
       </c>
       <c r="D217" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E217" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F217" s="37">
-        <v>750</v>
+        <v>27</v>
+      </c>
+      <c r="F217" s="22">
+        <v>100</v>
       </c>
       <c r="G217" s="11">
         <v>46226</v>
@@ -7372,7 +7407,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="218" ht="17" spans="1:8">
+    <row r="218" ht="17" hidden="1" spans="1:8">
       <c r="A218" s="16" t="s">
         <v>35</v>
       </c>
@@ -7386,10 +7421,10 @@
         <v>26</v>
       </c>
       <c r="E218" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F218" s="22">
-        <v>100</v>
+        <v>28</v>
+      </c>
+      <c r="F218" s="19">
+        <v>600</v>
       </c>
       <c r="G218" s="11">
         <v>46226</v>
@@ -7398,7 +7433,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="219" ht="17" spans="1:8">
+    <row r="219" ht="17" hidden="1" spans="1:8">
       <c r="A219" s="16" t="s">
         <v>35</v>
       </c>
@@ -7412,10 +7447,10 @@
         <v>26</v>
       </c>
       <c r="E219" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F219" s="19">
-        <v>600</v>
+        <v>29</v>
+      </c>
+      <c r="F219" s="22">
+        <v>980</v>
       </c>
       <c r="G219" s="11">
         <v>46226</v>
@@ -7424,43 +7459,454 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="220" ht="17" spans="1:8">
-      <c r="A220" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="B220" s="9" t="s">
+    <row r="220" spans="1:8">
+      <c r="A220" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B220" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C220" s="8">
+        <v>0</v>
+      </c>
+      <c r="D220" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E220" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F220" s="40">
+        <v>300</v>
+      </c>
+      <c r="G220" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H220" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="221" spans="1:8">
+      <c r="A221" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B221" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C221" s="9">
+        <v>0</v>
+      </c>
+      <c r="D221" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E221" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F221" s="40">
+        <v>600</v>
+      </c>
+      <c r="G221" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H221" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="222" spans="1:8">
+      <c r="A222" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B222" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C222" s="9">
+        <v>0</v>
+      </c>
+      <c r="D222" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E222" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F222" s="40">
+        <v>600</v>
+      </c>
+      <c r="G222" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H222" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="223" spans="1:8">
+      <c r="A223" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B223" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C223" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D223" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E223" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F223" s="32">
+        <v>500</v>
+      </c>
+      <c r="G223" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H223" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="224" spans="1:8">
+      <c r="A224" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B224" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C224" s="9">
+        <v>990</v>
+      </c>
+      <c r="D224" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E224" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F224" s="32">
+        <v>1200</v>
+      </c>
+      <c r="G224" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H224" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="225" spans="1:8">
+      <c r="A225" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B225" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C225" s="9">
+        <v>990</v>
+      </c>
+      <c r="D225" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E225" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F225" s="32">
+        <v>1250</v>
+      </c>
+      <c r="G225" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H225" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="226" spans="1:8">
+      <c r="A226" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B226" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C220" s="21">
+      <c r="C226" s="9">
         <v>990</v>
       </c>
-      <c r="D220" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E220" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F220" s="22">
-        <v>980</v>
-      </c>
-      <c r="G220" s="11">
-        <v>46226</v>
-      </c>
-      <c r="H220" s="11">
-        <v>46219</v>
+      <c r="D226" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E226" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F226" s="32">
+        <v>100</v>
+      </c>
+      <c r="G226" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H226" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="227" spans="1:8">
+      <c r="A227" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B227" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C227" s="9">
+        <v>990</v>
+      </c>
+      <c r="D227" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E227" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F227" s="32">
+        <v>700</v>
+      </c>
+      <c r="G227" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H227" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="228" spans="1:8">
+      <c r="A228" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B228" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C228" s="9">
+        <v>990</v>
+      </c>
+      <c r="D228" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E228" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F228" s="32">
+        <v>700</v>
+      </c>
+      <c r="G228" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H228" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="229" ht="17" spans="1:8">
+      <c r="A229" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B229" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C229" s="9">
+        <v>990</v>
+      </c>
+      <c r="D229" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E229" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F229" s="41">
+        <v>60</v>
+      </c>
+      <c r="G229" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H229" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="230" ht="17" spans="1:8">
+      <c r="A230" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B230" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C230" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D230" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E230" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F230" s="41">
+        <v>320</v>
+      </c>
+      <c r="G230" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H230" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="231" ht="17" spans="1:8">
+      <c r="A231" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B231" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C231" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D231" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E231" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F231" s="41">
+        <v>470</v>
+      </c>
+      <c r="G231" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H231" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="232" spans="1:8">
+      <c r="A232" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B232" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C232" s="9">
+        <v>100</v>
+      </c>
+      <c r="D232" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E232" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F232" s="42">
+        <v>750</v>
+      </c>
+      <c r="G232" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H232" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8">
+      <c r="A233" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B233" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C233" s="9">
+        <v>100</v>
+      </c>
+      <c r="D233" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E233" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F233" s="42">
+        <v>850</v>
+      </c>
+      <c r="G233" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H233" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="234" spans="1:8">
+      <c r="A234" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B234" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C234" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D234" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E234" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F234" s="42">
+        <v>650</v>
+      </c>
+      <c r="G234" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H234" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="235" spans="1:8">
+      <c r="A235" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B235" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C235" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D235" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E235" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F235" s="42">
+        <v>600</v>
+      </c>
+      <c r="G235" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H235" s="11">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="236" spans="1:8">
+      <c r="A236" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B236" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C236" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D236" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E236" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F236" s="32">
+        <v>750</v>
+      </c>
+      <c r="G236" s="11">
+        <v>46231</v>
+      </c>
+      <c r="H236" s="11">
+        <v>46225</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H220" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="0">
-      <customFilters>
-        <customFilter operator="equal" val="暑_14"/>
-      </customFilters>
-    </filterColumn>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H236" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="3">
-      <customFilters>
-        <customFilter operator="equal" val="高中"/>
-      </customFilters>
+      <filters>
+        <filter val="初中"/>
+      </filters>
     </filterColumn>
     <extLst/>
   </autoFilter>

</xml_diff>

<commit_message>
Publish dashboard data 20260727-113755
</commit_message>
<xml_diff>
--- a/tongji_target.xlsx
+++ b/tongji_target.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$236</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$272</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="38">
   <si>
     <t>期次</t>
   </si>
@@ -141,6 +141,9 @@
   </si>
   <si>
     <t>秋_1</t>
+  </si>
+  <si>
+    <t>暑_15</t>
   </si>
 </sst>
 </file>
@@ -939,7 +942,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1134,14 +1137,6 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
@@ -1198,6 +1193,14 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
@@ -1206,7 +1209,15 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
@@ -1753,15 +1764,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:H236"/>
+  <sheetPr/>
+  <dimension ref="A1:H272"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.3076923076923" style="2" customWidth="1"/>
     <col min="2" max="2" width="20.6634615384615" style="2" customWidth="1"/>
     <col min="3" max="5" width="17.3076923076923" style="2" customWidth="1"/>
     <col min="6" max="6" width="17.3076923076923" style="3" customWidth="1"/>
-    <col min="7" max="7" width="17.7884615384615" style="4" customWidth="1"/>
+    <col min="7" max="7" width="21.4711538461538" style="4" customWidth="1"/>
     <col min="8" max="8" width="11.375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2311,7 +2322,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="22" ht="17" hidden="1" spans="1:8">
+    <row r="22" ht="17" spans="1:8">
       <c r="A22" s="16" t="s">
         <v>18</v>
       </c>
@@ -2337,7 +2348,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="23" ht="17" hidden="1" spans="1:8">
+    <row r="23" ht="17" spans="1:8">
       <c r="A23" s="16" t="s">
         <v>18</v>
       </c>
@@ -2363,7 +2374,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="24" ht="17" hidden="1" spans="1:8">
+    <row r="24" ht="17" spans="1:8">
       <c r="A24" s="16" t="s">
         <v>18</v>
       </c>
@@ -2389,7 +2400,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="25" ht="17" hidden="1" spans="1:8">
+    <row r="25" ht="17" spans="1:8">
       <c r="A25" s="16" t="s">
         <v>18</v>
       </c>
@@ -2415,7 +2426,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="26" ht="17" hidden="1" spans="1:8">
+    <row r="26" ht="17" spans="1:8">
       <c r="A26" s="16" t="s">
         <v>18</v>
       </c>
@@ -2441,7 +2452,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="27" ht="17" hidden="1" spans="1:8">
+    <row r="27" ht="17" spans="1:8">
       <c r="A27" s="16" t="s">
         <v>18</v>
       </c>
@@ -2467,7 +2478,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="28" ht="17" hidden="1" spans="1:8">
+    <row r="28" ht="17" spans="1:8">
       <c r="A28" s="16" t="s">
         <v>18</v>
       </c>
@@ -2493,7 +2504,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="29" ht="17" hidden="1" spans="1:8">
+    <row r="29" ht="17" spans="1:8">
       <c r="A29" s="16" t="s">
         <v>18</v>
       </c>
@@ -2519,7 +2530,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="30" ht="17" hidden="1" spans="1:8">
+    <row r="30" ht="17" spans="1:8">
       <c r="A30" s="16" t="s">
         <v>18</v>
       </c>
@@ -2545,7 +2556,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="31" ht="17" hidden="1" spans="1:8">
+    <row r="31" ht="17" spans="1:8">
       <c r="A31" s="16" t="s">
         <v>18</v>
       </c>
@@ -2571,7 +2582,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="32" ht="17" hidden="1" spans="1:8">
+    <row r="32" ht="17" spans="1:8">
       <c r="A32" s="16" t="s">
         <v>18</v>
       </c>
@@ -2597,7 +2608,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="33" ht="17" hidden="1" spans="1:8">
+    <row r="33" ht="17" spans="1:8">
       <c r="A33" s="16" t="s">
         <v>18</v>
       </c>
@@ -2623,7 +2634,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="34" ht="17" hidden="1" spans="1:8">
+    <row r="34" ht="17" spans="1:8">
       <c r="A34" s="16" t="s">
         <v>18</v>
       </c>
@@ -2649,7 +2660,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="35" ht="17" hidden="1" spans="1:8">
+    <row r="35" ht="17" spans="1:8">
       <c r="A35" s="16" t="s">
         <v>18</v>
       </c>
@@ -2675,7 +2686,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="36" ht="17" hidden="1" spans="1:8">
+    <row r="36" ht="17" spans="1:8">
       <c r="A36" s="16" t="s">
         <v>18</v>
       </c>
@@ -2701,7 +2712,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="37" ht="17" hidden="1" spans="1:8">
+    <row r="37" ht="17" spans="1:8">
       <c r="A37" s="16" t="s">
         <v>18</v>
       </c>
@@ -2727,7 +2738,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="38" ht="17" hidden="1" spans="1:8">
+    <row r="38" ht="17" spans="1:8">
       <c r="A38" s="16" t="s">
         <v>18</v>
       </c>
@@ -2753,7 +2764,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="39" ht="17" hidden="1" spans="1:8">
+    <row r="39" ht="17" spans="1:8">
       <c r="A39" s="16" t="s">
         <v>18</v>
       </c>
@@ -2779,7 +2790,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="40" ht="17" hidden="1" spans="1:8">
+    <row r="40" ht="17" spans="1:8">
       <c r="A40" s="16" t="s">
         <v>18</v>
       </c>
@@ -2805,7 +2816,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="41" ht="17" hidden="1" spans="1:8">
+    <row r="41" ht="17" spans="1:8">
       <c r="A41" s="16" t="s">
         <v>18</v>
       </c>
@@ -2831,7 +2842,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="42" ht="17" hidden="1" spans="1:8">
+    <row r="42" ht="17" spans="1:8">
       <c r="A42" s="16" t="s">
         <v>18</v>
       </c>
@@ -2857,7 +2868,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="43" ht="17" hidden="1" spans="1:8">
+    <row r="43" ht="17" spans="1:8">
       <c r="A43" s="16" t="s">
         <v>18</v>
       </c>
@@ -2883,7 +2894,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="44" ht="17" hidden="1" spans="1:8">
+    <row r="44" ht="17" spans="1:8">
       <c r="A44" s="16" t="s">
         <v>18</v>
       </c>
@@ -2909,7 +2920,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="45" ht="17" hidden="1" spans="1:8">
+    <row r="45" ht="17" spans="1:8">
       <c r="A45" s="16" t="s">
         <v>18</v>
       </c>
@@ -2935,7 +2946,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="46" ht="17" hidden="1" spans="1:8">
+    <row r="46" ht="17" spans="1:8">
       <c r="A46" s="16" t="s">
         <v>18</v>
       </c>
@@ -2961,7 +2972,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="47" ht="17" hidden="1" spans="1:8">
+    <row r="47" ht="17" spans="1:8">
       <c r="A47" s="16" t="s">
         <v>18</v>
       </c>
@@ -2987,7 +2998,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="48" ht="17" hidden="1" spans="1:8">
+    <row r="48" ht="17" spans="1:8">
       <c r="A48" s="16" t="s">
         <v>25</v>
       </c>
@@ -3013,7 +3024,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="49" ht="17" hidden="1" spans="1:8">
+    <row r="49" ht="17" spans="1:8">
       <c r="A49" s="16" t="s">
         <v>25</v>
       </c>
@@ -3039,7 +3050,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="50" ht="17" hidden="1" spans="1:8">
+    <row r="50" ht="17" spans="1:8">
       <c r="A50" s="16" t="s">
         <v>25</v>
       </c>
@@ -3065,7 +3076,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="51" ht="17" hidden="1" spans="1:8">
+    <row r="51" ht="17" spans="1:8">
       <c r="A51" s="16" t="s">
         <v>25</v>
       </c>
@@ -3091,7 +3102,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="52" ht="17" hidden="1" spans="1:8">
+    <row r="52" ht="17" spans="1:8">
       <c r="A52" s="16" t="s">
         <v>25</v>
       </c>
@@ -3117,7 +3128,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="53" ht="17" hidden="1" spans="1:8">
+    <row r="53" ht="17" spans="1:8">
       <c r="A53" s="16" t="s">
         <v>25</v>
       </c>
@@ -3143,7 +3154,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="54" ht="17" hidden="1" spans="1:8">
+    <row r="54" ht="17" spans="1:8">
       <c r="A54" s="16" t="s">
         <v>25</v>
       </c>
@@ -3169,7 +3180,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="55" ht="17" hidden="1" spans="1:8">
+    <row r="55" ht="17" spans="1:8">
       <c r="A55" s="16" t="s">
         <v>25</v>
       </c>
@@ -3195,7 +3206,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="56" ht="17" hidden="1" spans="1:8">
+    <row r="56" ht="17" spans="1:8">
       <c r="A56" s="16" t="s">
         <v>25</v>
       </c>
@@ -3221,7 +3232,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="57" ht="17" hidden="1" spans="1:8">
+    <row r="57" ht="17" spans="1:8">
       <c r="A57" s="16" t="s">
         <v>25</v>
       </c>
@@ -3247,7 +3258,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="58" ht="17" hidden="1" spans="1:8">
+    <row r="58" ht="17" spans="1:8">
       <c r="A58" s="16" t="s">
         <v>25</v>
       </c>
@@ -3273,7 +3284,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="59" ht="17" hidden="1" spans="1:8">
+    <row r="59" ht="17" spans="1:8">
       <c r="A59" s="16" t="s">
         <v>25</v>
       </c>
@@ -3299,7 +3310,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="60" ht="17" hidden="1" spans="1:8">
+    <row r="60" ht="17" spans="1:8">
       <c r="A60" s="16" t="s">
         <v>25</v>
       </c>
@@ -3325,7 +3336,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="61" ht="17" hidden="1" spans="1:8">
+    <row r="61" ht="17" spans="1:8">
       <c r="A61" s="16" t="s">
         <v>25</v>
       </c>
@@ -3351,7 +3362,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="62" ht="17" hidden="1" spans="1:8">
+    <row r="62" ht="17" spans="1:8">
       <c r="A62" s="16" t="s">
         <v>25</v>
       </c>
@@ -3377,7 +3388,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="63" ht="17" hidden="1" spans="1:8">
+    <row r="63" ht="17" spans="1:8">
       <c r="A63" s="16" t="s">
         <v>25</v>
       </c>
@@ -3403,7 +3414,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="64" ht="17" hidden="1" spans="1:8">
+    <row r="64" ht="17" spans="1:8">
       <c r="A64" s="16" t="s">
         <v>25</v>
       </c>
@@ -3429,7 +3440,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="65" ht="17" hidden="1" spans="1:8">
+    <row r="65" ht="17" spans="1:8">
       <c r="A65" s="16" t="s">
         <v>25</v>
       </c>
@@ -3455,7 +3466,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="66" ht="17" hidden="1" spans="1:8">
+    <row r="66" ht="17" spans="1:8">
       <c r="A66" s="16" t="s">
         <v>25</v>
       </c>
@@ -3481,7 +3492,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="67" ht="17" hidden="1" spans="1:8">
+    <row r="67" ht="17" spans="1:8">
       <c r="A67" s="16" t="s">
         <v>25</v>
       </c>
@@ -3507,7 +3518,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="68" ht="17" hidden="1" spans="1:8">
+    <row r="68" ht="17" spans="1:8">
       <c r="A68" s="16" t="s">
         <v>25</v>
       </c>
@@ -3975,7 +3986,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="86" ht="17" hidden="1" spans="1:8">
+    <row r="86" ht="17" spans="1:8">
       <c r="A86" s="16" t="s">
         <v>32</v>
       </c>
@@ -4001,7 +4012,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="87" ht="17" hidden="1" spans="1:8">
+    <row r="87" ht="17" spans="1:8">
       <c r="A87" s="16" t="s">
         <v>32</v>
       </c>
@@ -4027,7 +4038,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="88" ht="17" hidden="1" spans="1:8">
+    <row r="88" ht="17" spans="1:8">
       <c r="A88" s="16" t="s">
         <v>32</v>
       </c>
@@ -4053,7 +4064,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="89" ht="17" hidden="1" spans="1:8">
+    <row r="89" ht="17" spans="1:8">
       <c r="A89" s="16" t="s">
         <v>32</v>
       </c>
@@ -4079,7 +4090,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="90" ht="17" hidden="1" spans="1:8">
+    <row r="90" ht="17" spans="1:8">
       <c r="A90" s="16" t="s">
         <v>32</v>
       </c>
@@ -4105,7 +4116,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="91" ht="17" hidden="1" spans="1:8">
+    <row r="91" ht="17" spans="1:8">
       <c r="A91" s="16" t="s">
         <v>32</v>
       </c>
@@ -4131,7 +4142,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="92" ht="17" hidden="1" spans="1:8">
+    <row r="92" ht="17" spans="1:8">
       <c r="A92" s="16" t="s">
         <v>32</v>
       </c>
@@ -4157,7 +4168,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="93" ht="17" hidden="1" spans="1:8">
+    <row r="93" ht="17" spans="1:8">
       <c r="A93" s="16" t="s">
         <v>32</v>
       </c>
@@ -4183,7 +4194,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="94" ht="17" hidden="1" spans="1:8">
+    <row r="94" ht="17" spans="1:8">
       <c r="A94" s="16" t="s">
         <v>32</v>
       </c>
@@ -4209,7 +4220,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="95" ht="17" hidden="1" spans="1:8">
+    <row r="95" ht="17" spans="1:8">
       <c r="A95" s="16" t="s">
         <v>32</v>
       </c>
@@ -4235,7 +4246,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="96" ht="17" hidden="1" spans="1:8">
+    <row r="96" ht="17" spans="1:8">
       <c r="A96" s="16" t="s">
         <v>32</v>
       </c>
@@ -4261,7 +4272,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="97" ht="17" hidden="1" spans="1:8">
+    <row r="97" ht="17" spans="1:8">
       <c r="A97" s="16" t="s">
         <v>32</v>
       </c>
@@ -4287,7 +4298,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="98" ht="17" hidden="1" spans="1:8">
+    <row r="98" ht="17" spans="1:8">
       <c r="A98" s="16" t="s">
         <v>32</v>
       </c>
@@ -4313,7 +4324,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="99" ht="17" hidden="1" spans="1:8">
+    <row r="99" ht="17" spans="1:8">
       <c r="A99" s="16" t="s">
         <v>32</v>
       </c>
@@ -4339,7 +4350,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="100" ht="17" hidden="1" spans="1:8">
+    <row r="100" ht="17" spans="1:8">
       <c r="A100" s="16" t="s">
         <v>32</v>
       </c>
@@ -4365,7 +4376,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="101" ht="17" hidden="1" spans="1:8">
+    <row r="101" ht="17" spans="1:8">
       <c r="A101" s="16" t="s">
         <v>32</v>
       </c>
@@ -4391,7 +4402,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="102" ht="17" hidden="1" spans="1:8">
+    <row r="102" ht="17" spans="1:8">
       <c r="A102" s="16" t="s">
         <v>32</v>
       </c>
@@ -4417,7 +4428,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="103" ht="17" hidden="1" spans="1:8">
+    <row r="103" ht="17" spans="1:8">
       <c r="A103" s="16" t="s">
         <v>33</v>
       </c>
@@ -4443,7 +4454,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="104" ht="17" hidden="1" spans="1:8">
+    <row r="104" ht="17" spans="1:8">
       <c r="A104" s="16" t="s">
         <v>33</v>
       </c>
@@ -4469,7 +4480,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="105" ht="17" hidden="1" spans="1:8">
+    <row r="105" ht="17" spans="1:8">
       <c r="A105" s="16" t="s">
         <v>33</v>
       </c>
@@ -4495,7 +4506,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="106" ht="17" hidden="1" spans="1:8">
+    <row r="106" ht="17" spans="1:8">
       <c r="A106" s="16" t="s">
         <v>33</v>
       </c>
@@ -4521,7 +4532,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="107" ht="17" hidden="1" spans="1:8">
+    <row r="107" ht="17" spans="1:8">
       <c r="A107" s="16" t="s">
         <v>33</v>
       </c>
@@ -4547,7 +4558,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="108" ht="17" hidden="1" spans="1:8">
+    <row r="108" ht="17" spans="1:8">
       <c r="A108" s="16" t="s">
         <v>33</v>
       </c>
@@ -4573,7 +4584,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="109" ht="17" hidden="1" spans="1:8">
+    <row r="109" ht="17" spans="1:8">
       <c r="A109" s="16" t="s">
         <v>33</v>
       </c>
@@ -4599,7 +4610,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="110" ht="17" hidden="1" spans="1:8">
+    <row r="110" ht="17" spans="1:8">
       <c r="A110" s="16" t="s">
         <v>33</v>
       </c>
@@ -4625,7 +4636,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="111" ht="17" hidden="1" spans="1:8">
+    <row r="111" ht="17" spans="1:8">
       <c r="A111" s="16" t="s">
         <v>33</v>
       </c>
@@ -4651,7 +4662,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="112" ht="17" hidden="1" spans="1:8">
+    <row r="112" ht="17" spans="1:8">
       <c r="A112" s="16" t="s">
         <v>33</v>
       </c>
@@ -4677,7 +4688,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="113" ht="17" hidden="1" spans="1:8">
+    <row r="113" ht="17" spans="1:8">
       <c r="A113" s="16" t="s">
         <v>33</v>
       </c>
@@ -4703,7 +4714,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="114" ht="17" hidden="1" spans="1:8">
+    <row r="114" ht="17" spans="1:8">
       <c r="A114" s="16" t="s">
         <v>33</v>
       </c>
@@ -4729,7 +4740,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="115" ht="17" hidden="1" spans="1:8">
+    <row r="115" ht="17" spans="1:8">
       <c r="A115" s="16" t="s">
         <v>33</v>
       </c>
@@ -4755,7 +4766,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="116" ht="17" hidden="1" spans="1:8">
+    <row r="116" ht="17" spans="1:8">
       <c r="A116" s="16" t="s">
         <v>33</v>
       </c>
@@ -4781,7 +4792,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="117" ht="17" hidden="1" spans="1:8">
+    <row r="117" ht="17" spans="1:8">
       <c r="A117" s="16" t="s">
         <v>33</v>
       </c>
@@ -4807,7 +4818,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="118" ht="17" hidden="1" spans="1:8">
+    <row r="118" ht="17" spans="1:8">
       <c r="A118" s="16" t="s">
         <v>8</v>
       </c>
@@ -4833,7 +4844,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="119" ht="17" hidden="1" spans="1:8">
+    <row r="119" ht="17" spans="1:8">
       <c r="A119" s="16" t="s">
         <v>8</v>
       </c>
@@ -4859,7 +4870,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="120" ht="17" hidden="1" spans="1:8">
+    <row r="120" ht="17" spans="1:8">
       <c r="A120" s="16" t="s">
         <v>8</v>
       </c>
@@ -4885,7 +4896,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="121" ht="17" hidden="1" spans="1:8">
+    <row r="121" ht="17" spans="1:8">
       <c r="A121" s="16" t="s">
         <v>8</v>
       </c>
@@ -4911,7 +4922,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="122" ht="17" hidden="1" spans="1:8">
+    <row r="122" ht="17" spans="1:8">
       <c r="A122" s="16" t="s">
         <v>8</v>
       </c>
@@ -4937,7 +4948,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="123" ht="17" hidden="1" spans="1:8">
+    <row r="123" ht="17" spans="1:8">
       <c r="A123" s="16" t="s">
         <v>8</v>
       </c>
@@ -4963,7 +4974,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="124" ht="17" hidden="1" spans="1:8">
+    <row r="124" ht="17" spans="1:8">
       <c r="A124" s="16" t="s">
         <v>8</v>
       </c>
@@ -4989,7 +5000,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="125" ht="17" hidden="1" spans="1:8">
+    <row r="125" ht="17" spans="1:8">
       <c r="A125" s="16" t="s">
         <v>8</v>
       </c>
@@ -5015,7 +5026,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="126" ht="17" hidden="1" spans="1:8">
+    <row r="126" ht="17" spans="1:8">
       <c r="A126" s="16" t="s">
         <v>8</v>
       </c>
@@ -5041,7 +5052,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="127" ht="17" hidden="1" spans="1:8">
+    <row r="127" ht="17" spans="1:8">
       <c r="A127" s="16" t="s">
         <v>8</v>
       </c>
@@ -5067,7 +5078,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="128" ht="17" hidden="1" spans="1:8">
+    <row r="128" ht="17" spans="1:8">
       <c r="A128" s="16" t="s">
         <v>8</v>
       </c>
@@ -5093,7 +5104,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="129" ht="17" hidden="1" spans="1:8">
+    <row r="129" ht="17" spans="1:8">
       <c r="A129" s="16" t="s">
         <v>8</v>
       </c>
@@ -5119,7 +5130,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="130" ht="17" hidden="1" spans="1:8">
+    <row r="130" ht="17" spans="1:8">
       <c r="A130" s="16" t="s">
         <v>8</v>
       </c>
@@ -5145,7 +5156,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="131" ht="17" hidden="1" spans="1:8">
+    <row r="131" ht="17" spans="1:8">
       <c r="A131" s="16" t="s">
         <v>8</v>
       </c>
@@ -5171,7 +5182,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="132" ht="17" hidden="1" spans="1:8">
+    <row r="132" ht="17" spans="1:8">
       <c r="A132" s="16" t="s">
         <v>8</v>
       </c>
@@ -5197,7 +5208,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="133" ht="17" hidden="1" spans="1:8">
+    <row r="133" ht="17" spans="1:8">
       <c r="A133" s="16" t="s">
         <v>8</v>
       </c>
@@ -5223,7 +5234,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="134" ht="17" hidden="1" spans="1:8">
+    <row r="134" ht="17" spans="1:8">
       <c r="A134" s="16" t="s">
         <v>8</v>
       </c>
@@ -5691,7 +5702,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="152" ht="17" hidden="1" spans="1:8">
+    <row r="152" ht="17" spans="1:8">
       <c r="A152" s="16" t="s">
         <v>34</v>
       </c>
@@ -5717,7 +5728,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="153" ht="17" hidden="1" spans="1:8">
+    <row r="153" ht="17" spans="1:8">
       <c r="A153" s="16" t="s">
         <v>34</v>
       </c>
@@ -5743,7 +5754,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="154" ht="17" hidden="1" spans="1:8">
+    <row r="154" ht="17" spans="1:8">
       <c r="A154" s="16" t="s">
         <v>34</v>
       </c>
@@ -5769,7 +5780,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="155" ht="17" hidden="1" spans="1:8">
+    <row r="155" ht="17" spans="1:8">
       <c r="A155" s="16" t="s">
         <v>34</v>
       </c>
@@ -5795,7 +5806,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="156" ht="17" hidden="1" spans="1:8">
+    <row r="156" ht="17" spans="1:8">
       <c r="A156" s="16" t="s">
         <v>34</v>
       </c>
@@ -5821,7 +5832,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="157" ht="17" hidden="1" spans="1:8">
+    <row r="157" ht="17" spans="1:8">
       <c r="A157" s="16" t="s">
         <v>34</v>
       </c>
@@ -5847,7 +5858,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="158" ht="17" hidden="1" spans="1:8">
+    <row r="158" ht="17" spans="1:8">
       <c r="A158" s="16" t="s">
         <v>34</v>
       </c>
@@ -5873,7 +5884,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="159" ht="17" hidden="1" spans="1:8">
+    <row r="159" ht="17" spans="1:8">
       <c r="A159" s="16" t="s">
         <v>34</v>
       </c>
@@ -5899,7 +5910,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="160" ht="17" hidden="1" spans="1:8">
+    <row r="160" ht="17" spans="1:8">
       <c r="A160" s="16" t="s">
         <v>34</v>
       </c>
@@ -5925,7 +5936,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="161" ht="17" hidden="1" spans="1:8">
+    <row r="161" ht="17" spans="1:8">
       <c r="A161" s="16" t="s">
         <v>34</v>
       </c>
@@ -5951,7 +5962,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="162" ht="17" hidden="1" spans="1:8">
+    <row r="162" ht="17" spans="1:8">
       <c r="A162" s="16" t="s">
         <v>34</v>
       </c>
@@ -5977,7 +5988,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="163" ht="17" hidden="1" spans="1:8">
+    <row r="163" ht="17" spans="1:8">
       <c r="A163" s="16" t="s">
         <v>34</v>
       </c>
@@ -6003,7 +6014,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="164" ht="17" hidden="1" spans="1:8">
+    <row r="164" ht="17" spans="1:8">
       <c r="A164" s="16" t="s">
         <v>34</v>
       </c>
@@ -6029,7 +6040,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="165" ht="17" hidden="1" spans="1:8">
+    <row r="165" ht="17" spans="1:8">
       <c r="A165" s="16" t="s">
         <v>34</v>
       </c>
@@ -6055,7 +6066,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="166" ht="17" hidden="1" spans="1:8">
+    <row r="166" ht="17" spans="1:8">
       <c r="A166" s="16" t="s">
         <v>34</v>
       </c>
@@ -6253,7 +6264,7 @@
       <c r="E173" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F173" s="33">
+      <c r="F173" s="32">
         <v>150</v>
       </c>
       <c r="G173" s="11">
@@ -6279,7 +6290,7 @@
       <c r="E174" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F174" s="33">
+      <c r="F174" s="32">
         <v>850</v>
       </c>
       <c r="G174" s="11">
@@ -6305,7 +6316,7 @@
       <c r="E175" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F175" s="33">
+      <c r="F175" s="32">
         <v>850</v>
       </c>
       <c r="G175" s="11">
@@ -6331,7 +6342,7 @@
       <c r="E176" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F176" s="34">
+      <c r="F176" s="33">
         <v>210</v>
       </c>
       <c r="G176" s="11">
@@ -6357,7 +6368,7 @@
       <c r="E177" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F177" s="34">
+      <c r="F177" s="33">
         <v>230</v>
       </c>
       <c r="G177" s="11">
@@ -6383,7 +6394,7 @@
       <c r="E178" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F178" s="34">
+      <c r="F178" s="33">
         <v>360</v>
       </c>
       <c r="G178" s="11">
@@ -6409,7 +6420,7 @@
       <c r="E179" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F179" s="35">
+      <c r="F179" s="34">
         <v>800</v>
       </c>
       <c r="G179" s="11">
@@ -6435,7 +6446,7 @@
       <c r="E180" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F180" s="35">
+      <c r="F180" s="34">
         <v>900</v>
       </c>
       <c r="G180" s="11">
@@ -6461,7 +6472,7 @@
       <c r="E181" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F181" s="36">
+      <c r="F181" s="35">
         <v>680</v>
       </c>
       <c r="G181" s="11">
@@ -6487,7 +6498,7 @@
       <c r="E182" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F182" s="36">
+      <c r="F182" s="35">
         <v>600</v>
       </c>
       <c r="G182" s="11">
@@ -6513,7 +6524,7 @@
       <c r="E183" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F183" s="37">
+      <c r="F183" s="36">
         <v>600</v>
       </c>
       <c r="G183" s="11">
@@ -6523,7 +6534,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="184" ht="17" hidden="1" spans="1:8">
+    <row r="184" ht="17" spans="1:8">
       <c r="A184" s="16" t="s">
         <v>25</v>
       </c>
@@ -6539,7 +6550,7 @@
       <c r="E184" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F184" s="38">
+      <c r="F184" s="37">
         <v>130</v>
       </c>
       <c r="G184" s="11">
@@ -6549,7 +6560,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="185" ht="17" hidden="1" spans="1:8">
+    <row r="185" ht="17" spans="1:8">
       <c r="A185" s="16" t="s">
         <v>25</v>
       </c>
@@ -6565,7 +6576,7 @@
       <c r="E185" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F185" s="34">
+      <c r="F185" s="33">
         <v>250</v>
       </c>
       <c r="G185" s="11">
@@ -6575,7 +6586,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="186" ht="17" hidden="1" spans="1:8">
+    <row r="186" ht="17" spans="1:8">
       <c r="A186" s="16" t="s">
         <v>25</v>
       </c>
@@ -6591,7 +6602,7 @@
       <c r="E186" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F186" s="34">
+      <c r="F186" s="33">
         <v>400</v>
       </c>
       <c r="G186" s="11">
@@ -6601,7 +6612,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="187" ht="17" hidden="1" spans="1:8">
+    <row r="187" ht="17" spans="1:8">
       <c r="A187" s="16" t="s">
         <v>25</v>
       </c>
@@ -6617,7 +6628,7 @@
       <c r="E187" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F187" s="34">
+      <c r="F187" s="33">
         <v>470</v>
       </c>
       <c r="G187" s="11">
@@ -6627,7 +6638,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="188" ht="17" hidden="1" spans="1:8">
+    <row r="188" ht="17" spans="1:8">
       <c r="A188" s="16" t="s">
         <v>25</v>
       </c>
@@ -6643,7 +6654,7 @@
       <c r="E188" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F188" s="34">
+      <c r="F188" s="33">
         <v>600</v>
       </c>
       <c r="G188" s="11">
@@ -6653,7 +6664,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="189" ht="17" hidden="1" spans="1:8">
+    <row r="189" ht="17" spans="1:8">
       <c r="A189" s="16" t="s">
         <v>25</v>
       </c>
@@ -6669,7 +6680,7 @@
       <c r="E189" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F189" s="34">
+      <c r="F189" s="33">
         <v>150</v>
       </c>
       <c r="G189" s="11">
@@ -6679,7 +6690,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="190" ht="17" hidden="1" spans="1:8">
+    <row r="190" ht="17" spans="1:8">
       <c r="A190" s="16" t="s">
         <v>25</v>
       </c>
@@ -6695,7 +6706,7 @@
       <c r="E190" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F190" s="34">
+      <c r="F190" s="33">
         <v>350</v>
       </c>
       <c r="G190" s="11">
@@ -6705,7 +6716,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="191" ht="17" hidden="1" spans="1:8">
+    <row r="191" ht="17" spans="1:8">
       <c r="A191" s="16" t="s">
         <v>25</v>
       </c>
@@ -6721,7 +6732,7 @@
       <c r="E191" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F191" s="34">
+      <c r="F191" s="33">
         <v>250</v>
       </c>
       <c r="G191" s="11">
@@ -6731,7 +6742,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="192" ht="17" hidden="1" spans="1:8">
+    <row r="192" ht="17" spans="1:8">
       <c r="A192" s="16" t="s">
         <v>25</v>
       </c>
@@ -6747,7 +6758,7 @@
       <c r="E192" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F192" s="34">
+      <c r="F192" s="33">
         <v>250</v>
       </c>
       <c r="G192" s="11">
@@ -6757,7 +6768,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="193" ht="17" hidden="1" spans="1:8">
+    <row r="193" ht="17" spans="1:8">
       <c r="A193" s="16" t="s">
         <v>25</v>
       </c>
@@ -6773,7 +6784,7 @@
       <c r="E193" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F193" s="38">
+      <c r="F193" s="37">
         <v>30</v>
       </c>
       <c r="G193" s="11">
@@ -6783,7 +6794,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="194" ht="17" hidden="1" spans="1:8">
+    <row r="194" ht="17" spans="1:8">
       <c r="A194" s="16" t="s">
         <v>25</v>
       </c>
@@ -6799,7 +6810,7 @@
       <c r="E194" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F194" s="38">
+      <c r="F194" s="37">
         <v>140</v>
       </c>
       <c r="G194" s="11">
@@ -6809,7 +6820,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="195" ht="17" hidden="1" spans="1:8">
+    <row r="195" ht="17" spans="1:8">
       <c r="A195" s="16" t="s">
         <v>25</v>
       </c>
@@ -6825,7 +6836,7 @@
       <c r="E195" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F195" s="38">
+      <c r="F195" s="37">
         <v>140</v>
       </c>
       <c r="G195" s="11">
@@ -6835,7 +6846,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="196" ht="17" hidden="1" spans="1:8">
+    <row r="196" ht="17" spans="1:8">
       <c r="A196" s="16" t="s">
         <v>25</v>
       </c>
@@ -6851,7 +6862,7 @@
       <c r="E196" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F196" s="38">
+      <c r="F196" s="37">
         <v>140</v>
       </c>
       <c r="G196" s="11">
@@ -6861,7 +6872,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="197" ht="17" hidden="1" spans="1:8">
+    <row r="197" ht="17" spans="1:8">
       <c r="A197" s="16" t="s">
         <v>25</v>
       </c>
@@ -6877,7 +6888,7 @@
       <c r="E197" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F197" s="34">
+      <c r="F197" s="33">
         <v>1400</v>
       </c>
       <c r="G197" s="11">
@@ -6887,7 +6898,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="198" ht="17" hidden="1" spans="1:8">
+    <row r="198" ht="17" spans="1:8">
       <c r="A198" s="16" t="s">
         <v>25</v>
       </c>
@@ -6903,7 +6914,7 @@
       <c r="E198" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F198" s="34">
+      <c r="F198" s="33">
         <v>1550</v>
       </c>
       <c r="G198" s="11">
@@ -6913,7 +6924,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="199" ht="17" hidden="1" spans="1:8">
+    <row r="199" ht="17" spans="1:8">
       <c r="A199" s="16" t="s">
         <v>25</v>
       </c>
@@ -6929,7 +6940,7 @@
       <c r="E199" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F199" s="34">
+      <c r="F199" s="33">
         <v>1650</v>
       </c>
       <c r="G199" s="11">
@@ -6939,7 +6950,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="200" ht="17" hidden="1" spans="1:8">
+    <row r="200" ht="17" spans="1:8">
       <c r="A200" s="16" t="s">
         <v>25</v>
       </c>
@@ -6955,7 +6966,7 @@
       <c r="E200" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F200" s="34">
+      <c r="F200" s="33">
         <v>1300</v>
       </c>
       <c r="G200" s="11">
@@ -6965,7 +6976,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="201" ht="17" hidden="1" spans="1:8">
+    <row r="201" ht="17" spans="1:8">
       <c r="A201" s="16" t="s">
         <v>25</v>
       </c>
@@ -6981,7 +6992,7 @@
       <c r="E201" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F201" s="34">
+      <c r="F201" s="33">
         <v>150</v>
       </c>
       <c r="G201" s="11">
@@ -6991,7 +7002,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="202" ht="17" hidden="1" spans="1:8">
+    <row r="202" ht="17" spans="1:8">
       <c r="A202" s="16" t="s">
         <v>25</v>
       </c>
@@ -7007,7 +7018,7 @@
       <c r="E202" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F202" s="34">
+      <c r="F202" s="33">
         <v>150</v>
       </c>
       <c r="G202" s="11">
@@ -7017,7 +7028,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="203" ht="17" hidden="1" spans="1:8">
+    <row r="203" ht="17" spans="1:8">
       <c r="A203" s="16" t="s">
         <v>25</v>
       </c>
@@ -7033,7 +7044,7 @@
       <c r="E203" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F203" s="34">
+      <c r="F203" s="33">
         <v>150</v>
       </c>
       <c r="G203" s="11">
@@ -7043,7 +7054,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="204" ht="17" hidden="1" spans="1:8">
+    <row r="204" ht="17" spans="1:8">
       <c r="A204" s="16" t="s">
         <v>25</v>
       </c>
@@ -7059,7 +7070,7 @@
       <c r="E204" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F204" s="34">
+      <c r="F204" s="33">
         <v>150</v>
       </c>
       <c r="G204" s="11">
@@ -7069,7 +7080,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="205" ht="17" hidden="1" spans="1:8">
+    <row r="205" ht="17" spans="1:8">
       <c r="A205" s="16" t="s">
         <v>35</v>
       </c>
@@ -7085,7 +7096,7 @@
       <c r="E205" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F205" s="38">
+      <c r="F205" s="37">
         <v>100</v>
       </c>
       <c r="G205" s="11">
@@ -7095,7 +7106,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="206" ht="17" hidden="1" spans="1:8">
+    <row r="206" ht="17" spans="1:8">
       <c r="A206" s="16" t="s">
         <v>35</v>
       </c>
@@ -7111,7 +7122,7 @@
       <c r="E206" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F206" s="38">
+      <c r="F206" s="37">
         <v>200</v>
       </c>
       <c r="G206" s="11">
@@ -7121,7 +7132,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="207" ht="17" hidden="1" spans="1:8">
+    <row r="207" ht="17" spans="1:8">
       <c r="A207" s="16" t="s">
         <v>35</v>
       </c>
@@ -7137,7 +7148,7 @@
       <c r="E207" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F207" s="38">
+      <c r="F207" s="37">
         <v>200</v>
       </c>
       <c r="G207" s="11">
@@ -7147,7 +7158,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="208" ht="17" hidden="1" spans="1:8">
+    <row r="208" ht="17" spans="1:8">
       <c r="A208" s="16" t="s">
         <v>35</v>
       </c>
@@ -7163,7 +7174,7 @@
       <c r="E208" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F208" s="39">
+      <c r="F208" s="38">
         <v>200</v>
       </c>
       <c r="G208" s="11">
@@ -7173,7 +7184,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="209" ht="17" hidden="1" spans="1:8">
+    <row r="209" ht="17" spans="1:8">
       <c r="A209" s="16" t="s">
         <v>35</v>
       </c>
@@ -7189,7 +7200,7 @@
       <c r="E209" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F209" s="39">
+      <c r="F209" s="38">
         <v>1300</v>
       </c>
       <c r="G209" s="11">
@@ -7199,7 +7210,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="210" ht="17" hidden="1" spans="1:8">
+    <row r="210" ht="17" spans="1:8">
       <c r="A210" s="16" t="s">
         <v>35</v>
       </c>
@@ -7215,7 +7226,7 @@
       <c r="E210" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F210" s="39">
+      <c r="F210" s="38">
         <v>1300</v>
       </c>
       <c r="G210" s="11">
@@ -7225,7 +7236,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="211" ht="17" hidden="1" spans="1:8">
+    <row r="211" ht="17" spans="1:8">
       <c r="A211" s="16" t="s">
         <v>35</v>
       </c>
@@ -7251,7 +7262,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="212" ht="17" hidden="1" spans="1:8">
+    <row r="212" ht="17" spans="1:8">
       <c r="A212" s="16" t="s">
         <v>35</v>
       </c>
@@ -7267,7 +7278,7 @@
       <c r="E212" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F212" s="38">
+      <c r="F212" s="37">
         <v>450</v>
       </c>
       <c r="G212" s="11">
@@ -7277,7 +7288,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="213" ht="17" hidden="1" spans="1:8">
+    <row r="213" ht="17" spans="1:8">
       <c r="A213" s="16" t="s">
         <v>35</v>
       </c>
@@ -7293,7 +7304,7 @@
       <c r="E213" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F213" s="38">
+      <c r="F213" s="37">
         <v>450</v>
       </c>
       <c r="G213" s="11">
@@ -7303,7 +7314,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="214" ht="17" hidden="1" spans="1:8">
+    <row r="214" ht="17" spans="1:8">
       <c r="A214" s="16" t="s">
         <v>35</v>
       </c>
@@ -7329,7 +7340,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="215" ht="17" hidden="1" spans="1:8">
+    <row r="215" ht="17" spans="1:8">
       <c r="A215" s="16" t="s">
         <v>35</v>
       </c>
@@ -7345,7 +7356,7 @@
       <c r="E215" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F215" s="38">
+      <c r="F215" s="37">
         <v>650</v>
       </c>
       <c r="G215" s="11">
@@ -7355,7 +7366,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="216" ht="17" hidden="1" spans="1:8">
+    <row r="216" ht="17" spans="1:8">
       <c r="A216" s="16" t="s">
         <v>35</v>
       </c>
@@ -7371,7 +7382,7 @@
       <c r="E216" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F216" s="38">
+      <c r="F216" s="37">
         <v>750</v>
       </c>
       <c r="G216" s="11">
@@ -7381,7 +7392,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="217" ht="17" hidden="1" spans="1:8">
+    <row r="217" ht="17" spans="1:8">
       <c r="A217" s="16" t="s">
         <v>35</v>
       </c>
@@ -7407,7 +7418,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="218" ht="17" hidden="1" spans="1:8">
+    <row r="218" ht="17" spans="1:8">
       <c r="A218" s="16" t="s">
         <v>35</v>
       </c>
@@ -7433,7 +7444,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="219" ht="17" hidden="1" spans="1:8">
+    <row r="219" ht="17" spans="1:8">
       <c r="A219" s="16" t="s">
         <v>35</v>
       </c>
@@ -7475,7 +7486,7 @@
       <c r="E220" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F220" s="40">
+      <c r="F220" s="39">
         <v>300</v>
       </c>
       <c r="G220" s="11">
@@ -7501,7 +7512,7 @@
       <c r="E221" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F221" s="40">
+      <c r="F221" s="39">
         <v>600</v>
       </c>
       <c r="G221" s="11">
@@ -7527,7 +7538,7 @@
       <c r="E222" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F222" s="40">
+      <c r="F222" s="39">
         <v>600</v>
       </c>
       <c r="G222" s="11">
@@ -7709,7 +7720,7 @@
       <c r="E229" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F229" s="41">
+      <c r="F229" s="33">
         <v>60</v>
       </c>
       <c r="G229" s="11">
@@ -7735,7 +7746,7 @@
       <c r="E230" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F230" s="41">
+      <c r="F230" s="33">
         <v>320</v>
       </c>
       <c r="G230" s="11">
@@ -7761,7 +7772,7 @@
       <c r="E231" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F231" s="41">
+      <c r="F231" s="33">
         <v>470</v>
       </c>
       <c r="G231" s="11">
@@ -7787,7 +7798,7 @@
       <c r="E232" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F232" s="42">
+      <c r="F232" s="34">
         <v>750</v>
       </c>
       <c r="G232" s="11">
@@ -7813,7 +7824,7 @@
       <c r="E233" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F233" s="42">
+      <c r="F233" s="34">
         <v>850</v>
       </c>
       <c r="G233" s="11">
@@ -7839,7 +7850,7 @@
       <c r="E234" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F234" s="42">
+      <c r="F234" s="34">
         <v>650</v>
       </c>
       <c r="G234" s="11">
@@ -7865,7 +7876,7 @@
       <c r="E235" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F235" s="42">
+      <c r="F235" s="34">
         <v>600</v>
       </c>
       <c r="G235" s="11">
@@ -7901,13 +7912,944 @@
         <v>46225</v>
       </c>
     </row>
+    <row r="237" ht="17" spans="1:8">
+      <c r="A237" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B237" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C237" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D237" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E237" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F237" s="40">
+        <v>120</v>
+      </c>
+      <c r="G237" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H237" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="238" ht="17" spans="1:8">
+      <c r="A238" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B238" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C238" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D238" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E238" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F238" s="41">
+        <v>200</v>
+      </c>
+      <c r="G238" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H238" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="239" ht="17" spans="1:8">
+      <c r="A239" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B239" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C239" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D239" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E239" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F239" s="41">
+        <v>350</v>
+      </c>
+      <c r="G239" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H239" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="240" ht="17" spans="1:8">
+      <c r="A240" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B240" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C240" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D240" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E240" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F240" s="41">
+        <v>400</v>
+      </c>
+      <c r="G240" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H240" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="241" ht="17" spans="1:8">
+      <c r="A241" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B241" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C241" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D241" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E241" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F241" s="41">
+        <v>550</v>
+      </c>
+      <c r="G241" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H241" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="242" ht="17" spans="1:8">
+      <c r="A242" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B242" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C242" s="9">
+        <v>990</v>
+      </c>
+      <c r="D242" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E242" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F242" s="41">
+        <v>100</v>
+      </c>
+      <c r="G242" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H242" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="243" ht="17" spans="1:8">
+      <c r="A243" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B243" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C243" s="9">
+        <v>990</v>
+      </c>
+      <c r="D243" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E243" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F243" s="41">
+        <v>320</v>
+      </c>
+      <c r="G243" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H243" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="244" ht="17" spans="1:8">
+      <c r="A244" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B244" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C244" s="9">
+        <v>990</v>
+      </c>
+      <c r="D244" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E244" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F244" s="41">
+        <v>240</v>
+      </c>
+      <c r="G244" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H244" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="245" ht="17" spans="1:8">
+      <c r="A245" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B245" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C245" s="9">
+        <v>990</v>
+      </c>
+      <c r="D245" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E245" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F245" s="41">
+        <v>240</v>
+      </c>
+      <c r="G245" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H245" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="246" ht="17" spans="1:8">
+      <c r="A246" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B246" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C246" s="9">
+        <v>0</v>
+      </c>
+      <c r="D246" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E246" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F246" s="40">
+        <v>50</v>
+      </c>
+      <c r="G246" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H246" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="247" ht="17" spans="1:8">
+      <c r="A247" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B247" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C247" s="9">
+        <v>0</v>
+      </c>
+      <c r="D247" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E247" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F247" s="40">
+        <v>200</v>
+      </c>
+      <c r="G247" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H247" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="248" ht="17" spans="1:8">
+      <c r="A248" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B248" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C248" s="9">
+        <v>0</v>
+      </c>
+      <c r="D248" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E248" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F248" s="40">
+        <v>200</v>
+      </c>
+      <c r="G248" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H248" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="249" ht="17" spans="1:8">
+      <c r="A249" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B249" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C249" s="9">
+        <v>0</v>
+      </c>
+      <c r="D249" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E249" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F249" s="40">
+        <v>200</v>
+      </c>
+      <c r="G249" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H249" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="250" ht="17" spans="1:8">
+      <c r="A250" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B250" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C250" s="9">
+        <v>100</v>
+      </c>
+      <c r="D250" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E250" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F250" s="41">
+        <v>2050</v>
+      </c>
+      <c r="G250" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H250" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="251" ht="17" spans="1:8">
+      <c r="A251" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B251" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C251" s="9">
+        <v>100</v>
+      </c>
+      <c r="D251" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E251" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F251" s="41">
+        <v>2050</v>
+      </c>
+      <c r="G251" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H251" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="252" ht="17" spans="1:8">
+      <c r="A252" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B252" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C252" s="9">
+        <v>100</v>
+      </c>
+      <c r="D252" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E252" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F252" s="41">
+        <v>2050</v>
+      </c>
+      <c r="G252" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H252" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="253" ht="17" spans="1:8">
+      <c r="A253" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B253" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C253" s="9">
+        <v>100</v>
+      </c>
+      <c r="D253" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E253" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F253" s="41">
+        <v>2050</v>
+      </c>
+      <c r="G253" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H253" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="254" ht="17" spans="1:8">
+      <c r="A254" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B254" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C254" s="9">
+        <v>990</v>
+      </c>
+      <c r="D254" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E254" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F254" s="42">
+        <v>200</v>
+      </c>
+      <c r="G254" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H254" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="255" ht="17" spans="1:8">
+      <c r="A255" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B255" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C255" s="9">
+        <v>990</v>
+      </c>
+      <c r="D255" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E255" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F255" s="42">
+        <v>200</v>
+      </c>
+      <c r="G255" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H255" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="256" ht="17" spans="1:8">
+      <c r="A256" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B256" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C256" s="9">
+        <v>990</v>
+      </c>
+      <c r="D256" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E256" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F256" s="42">
+        <v>200</v>
+      </c>
+      <c r="G256" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H256" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="257" ht="17" spans="1:8">
+      <c r="A257" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B257" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C257" s="9">
+        <v>990</v>
+      </c>
+      <c r="D257" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E257" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F257" s="42">
+        <v>200</v>
+      </c>
+      <c r="G257" s="11">
+        <v>46232</v>
+      </c>
+      <c r="H257" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="258" ht="17" spans="1:8">
+      <c r="A258" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B258" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C258" s="9">
+        <v>0</v>
+      </c>
+      <c r="D258" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E258" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F258" s="40">
+        <v>150</v>
+      </c>
+      <c r="G258" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H258" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="259" ht="17" spans="1:8">
+      <c r="A259" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B259" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C259" s="9">
+        <v>0</v>
+      </c>
+      <c r="D259" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E259" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F259" s="40">
+        <v>300</v>
+      </c>
+      <c r="G259" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H259" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="260" ht="17" spans="1:8">
+      <c r="A260" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B260" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C260" s="9">
+        <v>0</v>
+      </c>
+      <c r="D260" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E260" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F260" s="40">
+        <v>300</v>
+      </c>
+      <c r="G260" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H260" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="261" ht="17" spans="1:8">
+      <c r="A261" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B261" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C261" s="9">
+        <v>100</v>
+      </c>
+      <c r="D261" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E261" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F261" s="43">
+        <v>120</v>
+      </c>
+      <c r="G261" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H261" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="262" ht="17" spans="1:8">
+      <c r="A262" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B262" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C262" s="9">
+        <v>100</v>
+      </c>
+      <c r="D262" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E262" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F262" s="40">
+        <v>1300</v>
+      </c>
+      <c r="G262" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H262" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="263" ht="17" spans="1:8">
+      <c r="A263" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B263" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C263" s="9">
+        <v>100</v>
+      </c>
+      <c r="D263" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E263" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F263" s="40">
+        <v>1300</v>
+      </c>
+      <c r="G263" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H263" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="264" ht="17" spans="1:8">
+      <c r="A264" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B264" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C264" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D264" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E264" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F264" s="12">
+        <v>0</v>
+      </c>
+      <c r="G264" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H264" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="265" ht="17" spans="1:8">
+      <c r="A265" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B265" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C265" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D265" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E265" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F265" s="40">
+        <v>400</v>
+      </c>
+      <c r="G265" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H265" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="266" ht="17" spans="1:8">
+      <c r="A266" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B266" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C266" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D266" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E266" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F266" s="40">
+        <v>400</v>
+      </c>
+      <c r="G266" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H266" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="267" ht="17" spans="1:8">
+      <c r="A267" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B267" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C267" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D267" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E267" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F267" s="20">
+        <v>0</v>
+      </c>
+      <c r="G267" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H267" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="268" ht="17" spans="1:8">
+      <c r="A268" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B268" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C268" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D268" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E268" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F268" s="40">
+        <v>700</v>
+      </c>
+      <c r="G268" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H268" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="269" ht="17" spans="1:8">
+      <c r="A269" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B269" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C269" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D269" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E269" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F269" s="40">
+        <v>700</v>
+      </c>
+      <c r="G269" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H269" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="270" ht="17" spans="1:8">
+      <c r="A270" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B270" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C270" s="21">
+        <v>990</v>
+      </c>
+      <c r="D270" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E270" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F270" s="43">
+        <v>100</v>
+      </c>
+      <c r="G270" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H270" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="271" ht="17" spans="1:8">
+      <c r="A271" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B271" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C271" s="21">
+        <v>990</v>
+      </c>
+      <c r="D271" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E271" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F271" s="40">
+        <v>235</v>
+      </c>
+      <c r="G271" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H271" s="11">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="272" ht="17" spans="1:8">
+      <c r="A272" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B272" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C272" s="21">
+        <v>990</v>
+      </c>
+      <c r="D272" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E272" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F272" s="40">
+        <v>1100</v>
+      </c>
+      <c r="G272" s="11">
+        <v>46233</v>
+      </c>
+      <c r="H272" s="11">
+        <v>46226</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H236" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="初中"/>
-      </filters>
-    </filterColumn>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H272" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <sortState ref="A2:F79">

</xml_diff>

<commit_message>
Update progress dashboard reports and documentation
</commit_message>
<xml_diff>
--- a/tongji_target.xlsx
+++ b/tongji_target.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$272</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$289</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="39">
   <si>
     <t>期次</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>暑_15</t>
+  </si>
+  <si>
+    <t>秋_2</t>
   </si>
 </sst>
 </file>
@@ -942,7 +945,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1193,7 +1196,23 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
@@ -1209,15 +1228,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
@@ -1764,8 +1775,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:H272"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:H289"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.3076923076923" style="2" customWidth="1"/>
@@ -1802,7 +1813,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="17.55" spans="1:8">
+    <row r="2" hidden="1" spans="1:8">
       <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
@@ -1828,7 +1839,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" hidden="1" spans="1:8">
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
@@ -1854,7 +1865,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" hidden="1" spans="1:8">
       <c r="A4" s="7" t="s">
         <v>8</v>
       </c>
@@ -1880,7 +1891,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="5" ht="17" spans="1:8">
+    <row r="5" ht="17" hidden="1" spans="1:8">
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
@@ -1906,7 +1917,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="6" ht="17" spans="1:8">
+    <row r="6" ht="17" hidden="1" spans="1:8">
       <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
@@ -1932,7 +1943,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="7" ht="17" spans="1:8">
+    <row r="7" ht="17" hidden="1" spans="1:8">
       <c r="A7" s="7" t="s">
         <v>8</v>
       </c>
@@ -1958,7 +1969,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" hidden="1" spans="1:8">
       <c r="A8" s="7" t="s">
         <v>8</v>
       </c>
@@ -1984,7 +1995,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" hidden="1" spans="1:8">
       <c r="A9" s="7" t="s">
         <v>8</v>
       </c>
@@ -2010,7 +2021,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" hidden="1" spans="1:8">
       <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
@@ -2036,7 +2047,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" hidden="1" spans="1:8">
       <c r="A11" s="7" t="s">
         <v>8</v>
       </c>
@@ -2062,7 +2073,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" hidden="1" spans="1:8">
       <c r="A12" s="7" t="s">
         <v>8</v>
       </c>
@@ -2088,7 +2099,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" hidden="1" spans="1:8">
       <c r="A13" s="7" t="s">
         <v>8</v>
       </c>
@@ -2114,7 +2125,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="14" ht="17" spans="1:8">
+    <row r="14" ht="17" hidden="1" spans="1:8">
       <c r="A14" s="7" t="s">
         <v>8</v>
       </c>
@@ -2140,7 +2151,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="15" ht="17" spans="1:8">
+    <row r="15" ht="17" hidden="1" spans="1:8">
       <c r="A15" s="7" t="s">
         <v>8</v>
       </c>
@@ -2166,7 +2177,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="16" ht="17" spans="1:8">
+    <row r="16" ht="17" hidden="1" spans="1:8">
       <c r="A16" s="7" t="s">
         <v>8</v>
       </c>
@@ -2192,7 +2203,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" hidden="1" spans="1:8">
       <c r="A17" s="7" t="s">
         <v>8</v>
       </c>
@@ -2218,7 +2229,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" hidden="1" spans="1:8">
       <c r="A18" s="7" t="s">
         <v>8</v>
       </c>
@@ -2244,7 +2255,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" hidden="1" spans="1:8">
       <c r="A19" s="7" t="s">
         <v>8</v>
       </c>
@@ -2270,7 +2281,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" hidden="1" spans="1:8">
       <c r="A20" s="7" t="s">
         <v>8</v>
       </c>
@@ -2296,7 +2307,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" hidden="1" spans="1:8">
       <c r="A21" s="7" t="s">
         <v>8</v>
       </c>
@@ -2322,7 +2333,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="22" ht="17" spans="1:8">
+    <row r="22" ht="17" hidden="1" spans="1:8">
       <c r="A22" s="16" t="s">
         <v>18</v>
       </c>
@@ -2348,7 +2359,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="23" ht="17" spans="1:8">
+    <row r="23" ht="17" hidden="1" spans="1:8">
       <c r="A23" s="16" t="s">
         <v>18</v>
       </c>
@@ -2374,7 +2385,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="24" ht="17" spans="1:8">
+    <row r="24" ht="17" hidden="1" spans="1:8">
       <c r="A24" s="16" t="s">
         <v>18</v>
       </c>
@@ -2400,7 +2411,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="25" ht="17" spans="1:8">
+    <row r="25" ht="17" hidden="1" spans="1:8">
       <c r="A25" s="16" t="s">
         <v>18</v>
       </c>
@@ -2426,7 +2437,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="26" ht="17" spans="1:8">
+    <row r="26" ht="17" hidden="1" spans="1:8">
       <c r="A26" s="16" t="s">
         <v>18</v>
       </c>
@@ -2452,7 +2463,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="27" ht="17" spans="1:8">
+    <row r="27" ht="17" hidden="1" spans="1:8">
       <c r="A27" s="16" t="s">
         <v>18</v>
       </c>
@@ -2478,7 +2489,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="28" ht="17" spans="1:8">
+    <row r="28" ht="17" hidden="1" spans="1:8">
       <c r="A28" s="16" t="s">
         <v>18</v>
       </c>
@@ -2504,7 +2515,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="29" ht="17" spans="1:8">
+    <row r="29" ht="17" hidden="1" spans="1:8">
       <c r="A29" s="16" t="s">
         <v>18</v>
       </c>
@@ -2530,7 +2541,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="30" ht="17" spans="1:8">
+    <row r="30" ht="17" hidden="1" spans="1:8">
       <c r="A30" s="16" t="s">
         <v>18</v>
       </c>
@@ -2556,7 +2567,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="31" ht="17" spans="1:8">
+    <row r="31" ht="17" hidden="1" spans="1:8">
       <c r="A31" s="16" t="s">
         <v>18</v>
       </c>
@@ -2582,7 +2593,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="32" ht="17" spans="1:8">
+    <row r="32" ht="17" hidden="1" spans="1:8">
       <c r="A32" s="16" t="s">
         <v>18</v>
       </c>
@@ -2608,7 +2619,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="33" ht="17" spans="1:8">
+    <row r="33" ht="17" hidden="1" spans="1:8">
       <c r="A33" s="16" t="s">
         <v>18</v>
       </c>
@@ -2634,7 +2645,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="34" ht="17" spans="1:8">
+    <row r="34" ht="17" hidden="1" spans="1:8">
       <c r="A34" s="16" t="s">
         <v>18</v>
       </c>
@@ -2660,7 +2671,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="35" ht="17" spans="1:8">
+    <row r="35" ht="17" hidden="1" spans="1:8">
       <c r="A35" s="16" t="s">
         <v>18</v>
       </c>
@@ -2686,7 +2697,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="36" ht="17" spans="1:8">
+    <row r="36" ht="17" hidden="1" spans="1:8">
       <c r="A36" s="16" t="s">
         <v>18</v>
       </c>
@@ -2712,7 +2723,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="37" ht="17" spans="1:8">
+    <row r="37" ht="17" hidden="1" spans="1:8">
       <c r="A37" s="16" t="s">
         <v>18</v>
       </c>
@@ -2738,7 +2749,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="38" ht="17" spans="1:8">
+    <row r="38" ht="17" hidden="1" spans="1:8">
       <c r="A38" s="16" t="s">
         <v>18</v>
       </c>
@@ -2764,7 +2775,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="39" ht="17" spans="1:8">
+    <row r="39" ht="17" hidden="1" spans="1:8">
       <c r="A39" s="16" t="s">
         <v>18</v>
       </c>
@@ -2790,7 +2801,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="40" ht="17" spans="1:8">
+    <row r="40" ht="17" hidden="1" spans="1:8">
       <c r="A40" s="16" t="s">
         <v>18</v>
       </c>
@@ -2816,7 +2827,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="41" ht="17" spans="1:8">
+    <row r="41" ht="17" hidden="1" spans="1:8">
       <c r="A41" s="16" t="s">
         <v>18</v>
       </c>
@@ -2842,7 +2853,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="42" ht="17" spans="1:8">
+    <row r="42" ht="17" hidden="1" spans="1:8">
       <c r="A42" s="16" t="s">
         <v>18</v>
       </c>
@@ -2868,7 +2879,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="43" ht="17" spans="1:8">
+    <row r="43" ht="17" hidden="1" spans="1:8">
       <c r="A43" s="16" t="s">
         <v>18</v>
       </c>
@@ -2894,7 +2905,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="44" ht="17" spans="1:8">
+    <row r="44" ht="17" hidden="1" spans="1:8">
       <c r="A44" s="16" t="s">
         <v>18</v>
       </c>
@@ -2920,7 +2931,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="45" ht="17" spans="1:8">
+    <row r="45" ht="17" hidden="1" spans="1:8">
       <c r="A45" s="16" t="s">
         <v>18</v>
       </c>
@@ -2946,7 +2957,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="46" ht="17" spans="1:8">
+    <row r="46" ht="17" hidden="1" spans="1:8">
       <c r="A46" s="16" t="s">
         <v>18</v>
       </c>
@@ -2972,7 +2983,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="47" ht="17" spans="1:8">
+    <row r="47" ht="17" hidden="1" spans="1:8">
       <c r="A47" s="16" t="s">
         <v>18</v>
       </c>
@@ -2998,7 +3009,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="48" ht="17" spans="1:8">
+    <row r="48" ht="17" hidden="1" spans="1:8">
       <c r="A48" s="16" t="s">
         <v>25</v>
       </c>
@@ -3024,7 +3035,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="49" ht="17" spans="1:8">
+    <row r="49" ht="17" hidden="1" spans="1:8">
       <c r="A49" s="16" t="s">
         <v>25</v>
       </c>
@@ -3050,7 +3061,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="50" ht="17" spans="1:8">
+    <row r="50" ht="17" hidden="1" spans="1:8">
       <c r="A50" s="16" t="s">
         <v>25</v>
       </c>
@@ -3076,7 +3087,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="51" ht="17" spans="1:8">
+    <row r="51" ht="17" hidden="1" spans="1:8">
       <c r="A51" s="16" t="s">
         <v>25</v>
       </c>
@@ -3102,7 +3113,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="52" ht="17" spans="1:8">
+    <row r="52" ht="17" hidden="1" spans="1:8">
       <c r="A52" s="16" t="s">
         <v>25</v>
       </c>
@@ -3128,7 +3139,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="53" ht="17" spans="1:8">
+    <row r="53" ht="17" hidden="1" spans="1:8">
       <c r="A53" s="16" t="s">
         <v>25</v>
       </c>
@@ -3154,7 +3165,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="54" ht="17" spans="1:8">
+    <row r="54" ht="17" hidden="1" spans="1:8">
       <c r="A54" s="16" t="s">
         <v>25</v>
       </c>
@@ -3180,7 +3191,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="55" ht="17" spans="1:8">
+    <row r="55" ht="17" hidden="1" spans="1:8">
       <c r="A55" s="16" t="s">
         <v>25</v>
       </c>
@@ -3206,7 +3217,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="56" ht="17" spans="1:8">
+    <row r="56" ht="17" hidden="1" spans="1:8">
       <c r="A56" s="16" t="s">
         <v>25</v>
       </c>
@@ -3232,7 +3243,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="57" ht="17" spans="1:8">
+    <row r="57" ht="17" hidden="1" spans="1:8">
       <c r="A57" s="16" t="s">
         <v>25</v>
       </c>
@@ -3258,7 +3269,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="58" ht="17" spans="1:8">
+    <row r="58" ht="17" hidden="1" spans="1:8">
       <c r="A58" s="16" t="s">
         <v>25</v>
       </c>
@@ -3284,7 +3295,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="59" ht="17" spans="1:8">
+    <row r="59" ht="17" hidden="1" spans="1:8">
       <c r="A59" s="16" t="s">
         <v>25</v>
       </c>
@@ -3310,7 +3321,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="60" ht="17" spans="1:8">
+    <row r="60" ht="17" hidden="1" spans="1:8">
       <c r="A60" s="16" t="s">
         <v>25</v>
       </c>
@@ -3336,7 +3347,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="61" ht="17" spans="1:8">
+    <row r="61" ht="17" hidden="1" spans="1:8">
       <c r="A61" s="16" t="s">
         <v>25</v>
       </c>
@@ -3362,7 +3373,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="62" ht="17" spans="1:8">
+    <row r="62" ht="17" hidden="1" spans="1:8">
       <c r="A62" s="16" t="s">
         <v>25</v>
       </c>
@@ -3388,7 +3399,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="63" ht="17" spans="1:8">
+    <row r="63" ht="17" hidden="1" spans="1:8">
       <c r="A63" s="16" t="s">
         <v>25</v>
       </c>
@@ -3414,7 +3425,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="64" ht="17" spans="1:8">
+    <row r="64" ht="17" hidden="1" spans="1:8">
       <c r="A64" s="16" t="s">
         <v>25</v>
       </c>
@@ -3440,7 +3451,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="65" ht="17" spans="1:8">
+    <row r="65" ht="17" hidden="1" spans="1:8">
       <c r="A65" s="16" t="s">
         <v>25</v>
       </c>
@@ -3466,7 +3477,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="66" ht="17" spans="1:8">
+    <row r="66" ht="17" hidden="1" spans="1:8">
       <c r="A66" s="16" t="s">
         <v>25</v>
       </c>
@@ -3492,7 +3503,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="67" ht="17" spans="1:8">
+    <row r="67" ht="17" hidden="1" spans="1:8">
       <c r="A67" s="16" t="s">
         <v>25</v>
       </c>
@@ -3518,7 +3529,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="68" ht="17" spans="1:8">
+    <row r="68" ht="17" hidden="1" spans="1:8">
       <c r="A68" s="16" t="s">
         <v>25</v>
       </c>
@@ -3544,7 +3555,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" hidden="1" spans="1:8">
       <c r="A69" s="7" t="s">
         <v>25</v>
       </c>
@@ -3570,7 +3581,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="70" spans="1:8">
+    <row r="70" hidden="1" spans="1:8">
       <c r="A70" s="7" t="s">
         <v>25</v>
       </c>
@@ -3596,7 +3607,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="71" spans="1:8">
+    <row r="71" hidden="1" spans="1:8">
       <c r="A71" s="7" t="s">
         <v>25</v>
       </c>
@@ -3622,7 +3633,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" hidden="1" spans="1:8">
       <c r="A72" s="7" t="s">
         <v>25</v>
       </c>
@@ -3648,7 +3659,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="73" spans="1:8">
+    <row r="73" hidden="1" spans="1:8">
       <c r="A73" s="7" t="s">
         <v>25</v>
       </c>
@@ -3674,7 +3685,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" hidden="1" spans="1:8">
       <c r="A74" s="7" t="s">
         <v>25</v>
       </c>
@@ -3700,7 +3711,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" hidden="1" spans="1:8">
       <c r="A75" s="7" t="s">
         <v>25</v>
       </c>
@@ -3726,7 +3737,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" hidden="1" spans="1:8">
       <c r="A76" s="7" t="s">
         <v>25</v>
       </c>
@@ -3752,7 +3763,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="77" spans="1:8">
+    <row r="77" hidden="1" spans="1:8">
       <c r="A77" s="7" t="s">
         <v>25</v>
       </c>
@@ -3778,7 +3789,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="78" ht="17" spans="1:8">
+    <row r="78" ht="17" hidden="1" spans="1:8">
       <c r="A78" s="7" t="s">
         <v>25</v>
       </c>
@@ -3804,7 +3815,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="79" ht="17" spans="1:8">
+    <row r="79" ht="17" hidden="1" spans="1:8">
       <c r="A79" s="7" t="s">
         <v>25</v>
       </c>
@@ -3830,7 +3841,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="80" ht="17" spans="1:8">
+    <row r="80" ht="17" hidden="1" spans="1:8">
       <c r="A80" s="7" t="s">
         <v>25</v>
       </c>
@@ -3856,7 +3867,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" hidden="1" spans="1:8">
       <c r="A81" s="7" t="s">
         <v>25</v>
       </c>
@@ -3882,7 +3893,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="82" spans="1:8">
+    <row r="82" hidden="1" spans="1:8">
       <c r="A82" s="7" t="s">
         <v>25</v>
       </c>
@@ -3908,7 +3919,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="83" spans="1:8">
+    <row r="83" hidden="1" spans="1:8">
       <c r="A83" s="7" t="s">
         <v>25</v>
       </c>
@@ -3934,7 +3945,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" hidden="1" spans="1:8">
       <c r="A84" s="7" t="s">
         <v>25</v>
       </c>
@@ -3960,7 +3971,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="85" spans="1:8">
+    <row r="85" hidden="1" spans="1:8">
       <c r="A85" s="7" t="s">
         <v>25</v>
       </c>
@@ -3986,7 +3997,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="86" ht="17" spans="1:8">
+    <row r="86" ht="17" hidden="1" spans="1:8">
       <c r="A86" s="16" t="s">
         <v>32</v>
       </c>
@@ -4012,7 +4023,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="87" ht="17" spans="1:8">
+    <row r="87" ht="17" hidden="1" spans="1:8">
       <c r="A87" s="16" t="s">
         <v>32</v>
       </c>
@@ -4038,7 +4049,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="88" ht="17" spans="1:8">
+    <row r="88" ht="17" hidden="1" spans="1:8">
       <c r="A88" s="16" t="s">
         <v>32</v>
       </c>
@@ -4064,7 +4075,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="89" ht="17" spans="1:8">
+    <row r="89" ht="17" hidden="1" spans="1:8">
       <c r="A89" s="16" t="s">
         <v>32</v>
       </c>
@@ -4090,7 +4101,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="90" ht="17" spans="1:8">
+    <row r="90" ht="17" hidden="1" spans="1:8">
       <c r="A90" s="16" t="s">
         <v>32</v>
       </c>
@@ -4116,7 +4127,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="91" ht="17" spans="1:8">
+    <row r="91" ht="17" hidden="1" spans="1:8">
       <c r="A91" s="16" t="s">
         <v>32</v>
       </c>
@@ -4142,7 +4153,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="92" ht="17" spans="1:8">
+    <row r="92" ht="17" hidden="1" spans="1:8">
       <c r="A92" s="16" t="s">
         <v>32</v>
       </c>
@@ -4168,7 +4179,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="93" ht="17" spans="1:8">
+    <row r="93" ht="17" hidden="1" spans="1:8">
       <c r="A93" s="16" t="s">
         <v>32</v>
       </c>
@@ -4194,7 +4205,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="94" ht="17" spans="1:8">
+    <row r="94" ht="17" hidden="1" spans="1:8">
       <c r="A94" s="16" t="s">
         <v>32</v>
       </c>
@@ -4220,7 +4231,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="95" ht="17" spans="1:8">
+    <row r="95" ht="17" hidden="1" spans="1:8">
       <c r="A95" s="16" t="s">
         <v>32</v>
       </c>
@@ -4246,7 +4257,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="96" ht="17" spans="1:8">
+    <row r="96" ht="17" hidden="1" spans="1:8">
       <c r="A96" s="16" t="s">
         <v>32</v>
       </c>
@@ -4272,7 +4283,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="97" ht="17" spans="1:8">
+    <row r="97" ht="17" hidden="1" spans="1:8">
       <c r="A97" s="16" t="s">
         <v>32</v>
       </c>
@@ -4298,7 +4309,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="98" ht="17" spans="1:8">
+    <row r="98" ht="17" hidden="1" spans="1:8">
       <c r="A98" s="16" t="s">
         <v>32</v>
       </c>
@@ -4324,7 +4335,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="99" ht="17" spans="1:8">
+    <row r="99" ht="17" hidden="1" spans="1:8">
       <c r="A99" s="16" t="s">
         <v>32</v>
       </c>
@@ -4350,7 +4361,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="100" ht="17" spans="1:8">
+    <row r="100" ht="17" hidden="1" spans="1:8">
       <c r="A100" s="16" t="s">
         <v>32</v>
       </c>
@@ -4376,7 +4387,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="101" ht="17" spans="1:8">
+    <row r="101" ht="17" hidden="1" spans="1:8">
       <c r="A101" s="16" t="s">
         <v>32</v>
       </c>
@@ -4402,7 +4413,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="102" ht="17" spans="1:8">
+    <row r="102" ht="17" hidden="1" spans="1:8">
       <c r="A102" s="16" t="s">
         <v>32</v>
       </c>
@@ -4428,7 +4439,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="103" ht="17" spans="1:8">
+    <row r="103" ht="17" hidden="1" spans="1:8">
       <c r="A103" s="16" t="s">
         <v>33</v>
       </c>
@@ -4454,7 +4465,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="104" ht="17" spans="1:8">
+    <row r="104" ht="17" hidden="1" spans="1:8">
       <c r="A104" s="16" t="s">
         <v>33</v>
       </c>
@@ -4480,7 +4491,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="105" ht="17" spans="1:8">
+    <row r="105" ht="17" hidden="1" spans="1:8">
       <c r="A105" s="16" t="s">
         <v>33</v>
       </c>
@@ -4506,7 +4517,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="106" ht="17" spans="1:8">
+    <row r="106" ht="17" hidden="1" spans="1:8">
       <c r="A106" s="16" t="s">
         <v>33</v>
       </c>
@@ -4532,7 +4543,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="107" ht="17" spans="1:8">
+    <row r="107" ht="17" hidden="1" spans="1:8">
       <c r="A107" s="16" t="s">
         <v>33</v>
       </c>
@@ -4558,7 +4569,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="108" ht="17" spans="1:8">
+    <row r="108" ht="17" hidden="1" spans="1:8">
       <c r="A108" s="16" t="s">
         <v>33</v>
       </c>
@@ -4584,7 +4595,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="109" ht="17" spans="1:8">
+    <row r="109" ht="17" hidden="1" spans="1:8">
       <c r="A109" s="16" t="s">
         <v>33</v>
       </c>
@@ -4610,7 +4621,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="110" ht="17" spans="1:8">
+    <row r="110" ht="17" hidden="1" spans="1:8">
       <c r="A110" s="16" t="s">
         <v>33</v>
       </c>
@@ -4636,7 +4647,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="111" ht="17" spans="1:8">
+    <row r="111" ht="17" hidden="1" spans="1:8">
       <c r="A111" s="16" t="s">
         <v>33</v>
       </c>
@@ -4662,7 +4673,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="112" ht="17" spans="1:8">
+    <row r="112" ht="17" hidden="1" spans="1:8">
       <c r="A112" s="16" t="s">
         <v>33</v>
       </c>
@@ -4688,7 +4699,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="113" ht="17" spans="1:8">
+    <row r="113" ht="17" hidden="1" spans="1:8">
       <c r="A113" s="16" t="s">
         <v>33</v>
       </c>
@@ -4714,7 +4725,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="114" ht="17" spans="1:8">
+    <row r="114" ht="17" hidden="1" spans="1:8">
       <c r="A114" s="16" t="s">
         <v>33</v>
       </c>
@@ -4740,7 +4751,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="115" ht="17" spans="1:8">
+    <row r="115" ht="17" hidden="1" spans="1:8">
       <c r="A115" s="16" t="s">
         <v>33</v>
       </c>
@@ -4766,7 +4777,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="116" ht="17" spans="1:8">
+    <row r="116" ht="17" hidden="1" spans="1:8">
       <c r="A116" s="16" t="s">
         <v>33</v>
       </c>
@@ -4792,7 +4803,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="117" ht="17" spans="1:8">
+    <row r="117" ht="17" hidden="1" spans="1:8">
       <c r="A117" s="16" t="s">
         <v>33</v>
       </c>
@@ -4818,7 +4829,7 @@
         <v>46205</v>
       </c>
     </row>
-    <row r="118" ht="17" spans="1:8">
+    <row r="118" ht="17" hidden="1" spans="1:8">
       <c r="A118" s="16" t="s">
         <v>8</v>
       </c>
@@ -4844,7 +4855,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="119" ht="17" spans="1:8">
+    <row r="119" ht="17" hidden="1" spans="1:8">
       <c r="A119" s="16" t="s">
         <v>8</v>
       </c>
@@ -4870,7 +4881,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="120" ht="17" spans="1:8">
+    <row r="120" ht="17" hidden="1" spans="1:8">
       <c r="A120" s="16" t="s">
         <v>8</v>
       </c>
@@ -4896,7 +4907,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="121" ht="17" spans="1:8">
+    <row r="121" ht="17" hidden="1" spans="1:8">
       <c r="A121" s="16" t="s">
         <v>8</v>
       </c>
@@ -4922,7 +4933,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="122" ht="17" spans="1:8">
+    <row r="122" ht="17" hidden="1" spans="1:8">
       <c r="A122" s="16" t="s">
         <v>8</v>
       </c>
@@ -4948,7 +4959,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="123" ht="17" spans="1:8">
+    <row r="123" ht="17" hidden="1" spans="1:8">
       <c r="A123" s="16" t="s">
         <v>8</v>
       </c>
@@ -4974,7 +4985,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="124" ht="17" spans="1:8">
+    <row r="124" ht="17" hidden="1" spans="1:8">
       <c r="A124" s="16" t="s">
         <v>8</v>
       </c>
@@ -5000,7 +5011,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="125" ht="17" spans="1:8">
+    <row r="125" ht="17" hidden="1" spans="1:8">
       <c r="A125" s="16" t="s">
         <v>8</v>
       </c>
@@ -5026,7 +5037,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="126" ht="17" spans="1:8">
+    <row r="126" ht="17" hidden="1" spans="1:8">
       <c r="A126" s="16" t="s">
         <v>8</v>
       </c>
@@ -5052,7 +5063,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="127" ht="17" spans="1:8">
+    <row r="127" ht="17" hidden="1" spans="1:8">
       <c r="A127" s="16" t="s">
         <v>8</v>
       </c>
@@ -5078,7 +5089,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="128" ht="17" spans="1:8">
+    <row r="128" ht="17" hidden="1" spans="1:8">
       <c r="A128" s="16" t="s">
         <v>8</v>
       </c>
@@ -5104,7 +5115,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="129" ht="17" spans="1:8">
+    <row r="129" ht="17" hidden="1" spans="1:8">
       <c r="A129" s="16" t="s">
         <v>8</v>
       </c>
@@ -5130,7 +5141,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="130" ht="17" spans="1:8">
+    <row r="130" ht="17" hidden="1" spans="1:8">
       <c r="A130" s="16" t="s">
         <v>8</v>
       </c>
@@ -5156,7 +5167,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="131" ht="17" spans="1:8">
+    <row r="131" ht="17" hidden="1" spans="1:8">
       <c r="A131" s="16" t="s">
         <v>8</v>
       </c>
@@ -5182,7 +5193,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="132" ht="17" spans="1:8">
+    <row r="132" ht="17" hidden="1" spans="1:8">
       <c r="A132" s="16" t="s">
         <v>8</v>
       </c>
@@ -5208,7 +5219,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="133" ht="17" spans="1:8">
+    <row r="133" ht="17" hidden="1" spans="1:8">
       <c r="A133" s="16" t="s">
         <v>8</v>
       </c>
@@ -5234,7 +5245,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="134" ht="17" spans="1:8">
+    <row r="134" ht="17" hidden="1" spans="1:8">
       <c r="A134" s="16" t="s">
         <v>8</v>
       </c>
@@ -5260,7 +5271,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="135" spans="1:8">
+    <row r="135" hidden="1" spans="1:8">
       <c r="A135" s="7" t="s">
         <v>33</v>
       </c>
@@ -5286,7 +5297,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="136" spans="1:8">
+    <row r="136" hidden="1" spans="1:8">
       <c r="A136" s="7" t="s">
         <v>33</v>
       </c>
@@ -5312,7 +5323,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="137" spans="1:8">
+    <row r="137" hidden="1" spans="1:8">
       <c r="A137" s="7" t="s">
         <v>33</v>
       </c>
@@ -5338,7 +5349,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="138" s="1" customFormat="1" spans="1:8">
+    <row r="138" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A138" s="7" t="s">
         <v>33</v>
       </c>
@@ -5364,7 +5375,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="139" s="1" customFormat="1" spans="1:8">
+    <row r="139" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A139" s="7" t="s">
         <v>33</v>
       </c>
@@ -5390,7 +5401,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="140" s="1" customFormat="1" spans="1:8">
+    <row r="140" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A140" s="7" t="s">
         <v>33</v>
       </c>
@@ -5416,7 +5427,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="141" s="1" customFormat="1" spans="1:8">
+    <row r="141" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A141" s="7" t="s">
         <v>33</v>
       </c>
@@ -5442,7 +5453,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="142" s="1" customFormat="1" spans="1:8">
+    <row r="142" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A142" s="7" t="s">
         <v>33</v>
       </c>
@@ -5468,7 +5479,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="143" s="1" customFormat="1" spans="1:8">
+    <row r="143" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A143" s="7" t="s">
         <v>33</v>
       </c>
@@ -5494,7 +5505,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="144" s="1" customFormat="1" ht="17" spans="1:8">
+    <row r="144" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A144" s="7" t="s">
         <v>33</v>
       </c>
@@ -5520,7 +5531,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="145" s="1" customFormat="1" ht="17" spans="1:8">
+    <row r="145" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A145" s="7" t="s">
         <v>33</v>
       </c>
@@ -5546,7 +5557,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="146" s="1" customFormat="1" ht="17" spans="1:8">
+    <row r="146" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A146" s="7" t="s">
         <v>33</v>
       </c>
@@ -5572,7 +5583,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="147" s="1" customFormat="1" spans="1:8">
+    <row r="147" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A147" s="7" t="s">
         <v>33</v>
       </c>
@@ -5598,7 +5609,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="148" spans="1:8">
+    <row r="148" hidden="1" spans="1:8">
       <c r="A148" s="7" t="s">
         <v>33</v>
       </c>
@@ -5624,7 +5635,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="149" spans="1:8">
+    <row r="149" hidden="1" spans="1:8">
       <c r="A149" s="7" t="s">
         <v>33</v>
       </c>
@@ -5650,7 +5661,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="150" spans="1:8">
+    <row r="150" hidden="1" spans="1:8">
       <c r="A150" s="7" t="s">
         <v>33</v>
       </c>
@@ -5676,7 +5687,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="151" spans="1:8">
+    <row r="151" hidden="1" spans="1:8">
       <c r="A151" s="7" t="s">
         <v>33</v>
       </c>
@@ -5702,7 +5713,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="152" ht="17" spans="1:8">
+    <row r="152" ht="17" hidden="1" spans="1:8">
       <c r="A152" s="16" t="s">
         <v>34</v>
       </c>
@@ -5728,7 +5739,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="153" ht="17" spans="1:8">
+    <row r="153" ht="17" hidden="1" spans="1:8">
       <c r="A153" s="16" t="s">
         <v>34</v>
       </c>
@@ -5754,7 +5765,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="154" ht="17" spans="1:8">
+    <row r="154" ht="17" hidden="1" spans="1:8">
       <c r="A154" s="16" t="s">
         <v>34</v>
       </c>
@@ -5780,7 +5791,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="155" ht="17" spans="1:8">
+    <row r="155" ht="17" hidden="1" spans="1:8">
       <c r="A155" s="16" t="s">
         <v>34</v>
       </c>
@@ -5806,7 +5817,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="156" ht="17" spans="1:8">
+    <row r="156" ht="17" hidden="1" spans="1:8">
       <c r="A156" s="16" t="s">
         <v>34</v>
       </c>
@@ -5832,7 +5843,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="157" ht="17" spans="1:8">
+    <row r="157" ht="17" hidden="1" spans="1:8">
       <c r="A157" s="16" t="s">
         <v>34</v>
       </c>
@@ -5858,7 +5869,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="158" ht="17" spans="1:8">
+    <row r="158" ht="17" hidden="1" spans="1:8">
       <c r="A158" s="16" t="s">
         <v>34</v>
       </c>
@@ -5884,7 +5895,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="159" ht="17" spans="1:8">
+    <row r="159" ht="17" hidden="1" spans="1:8">
       <c r="A159" s="16" t="s">
         <v>34</v>
       </c>
@@ -5910,7 +5921,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="160" ht="17" spans="1:8">
+    <row r="160" ht="17" hidden="1" spans="1:8">
       <c r="A160" s="16" t="s">
         <v>34</v>
       </c>
@@ -5936,7 +5947,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="161" ht="17" spans="1:8">
+    <row r="161" ht="17" hidden="1" spans="1:8">
       <c r="A161" s="16" t="s">
         <v>34</v>
       </c>
@@ -5962,7 +5973,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="162" ht="17" spans="1:8">
+    <row r="162" ht="17" hidden="1" spans="1:8">
       <c r="A162" s="16" t="s">
         <v>34</v>
       </c>
@@ -5988,7 +5999,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="163" ht="17" spans="1:8">
+    <row r="163" ht="17" hidden="1" spans="1:8">
       <c r="A163" s="16" t="s">
         <v>34</v>
       </c>
@@ -6014,7 +6025,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="164" ht="17" spans="1:8">
+    <row r="164" ht="17" hidden="1" spans="1:8">
       <c r="A164" s="16" t="s">
         <v>34</v>
       </c>
@@ -6040,7 +6051,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="165" ht="17" spans="1:8">
+    <row r="165" ht="17" hidden="1" spans="1:8">
       <c r="A165" s="16" t="s">
         <v>34</v>
       </c>
@@ -6066,7 +6077,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="166" ht="17" spans="1:8">
+    <row r="166" ht="17" hidden="1" spans="1:8">
       <c r="A166" s="16" t="s">
         <v>34</v>
       </c>
@@ -6092,7 +6103,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="167" spans="1:8">
+    <row r="167" hidden="1" spans="1:8">
       <c r="A167" s="7" t="s">
         <v>34</v>
       </c>
@@ -6118,7 +6129,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="168" spans="1:8">
+    <row r="168" hidden="1" spans="1:8">
       <c r="A168" s="7" t="s">
         <v>34</v>
       </c>
@@ -6144,7 +6155,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="169" spans="1:8">
+    <row r="169" hidden="1" spans="1:8">
       <c r="A169" s="7" t="s">
         <v>34</v>
       </c>
@@ -6170,7 +6181,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="170" spans="1:8">
+    <row r="170" hidden="1" spans="1:8">
       <c r="A170" s="7" t="s">
         <v>34</v>
       </c>
@@ -6196,7 +6207,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="171" spans="1:8">
+    <row r="171" hidden="1" spans="1:8">
       <c r="A171" s="7" t="s">
         <v>34</v>
       </c>
@@ -6222,7 +6233,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="172" spans="1:8">
+    <row r="172" hidden="1" spans="1:8">
       <c r="A172" s="7" t="s">
         <v>34</v>
       </c>
@@ -6248,7 +6259,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="173" spans="1:8">
+    <row r="173" hidden="1" spans="1:8">
       <c r="A173" s="7" t="s">
         <v>34</v>
       </c>
@@ -6274,7 +6285,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="174" spans="1:8">
+    <row r="174" hidden="1" spans="1:8">
       <c r="A174" s="7" t="s">
         <v>34</v>
       </c>
@@ -6300,7 +6311,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="175" spans="1:8">
+    <row r="175" hidden="1" spans="1:8">
       <c r="A175" s="7" t="s">
         <v>34</v>
       </c>
@@ -6326,7 +6337,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="176" ht="17" spans="1:8">
+    <row r="176" ht="17" hidden="1" spans="1:8">
       <c r="A176" s="7" t="s">
         <v>34</v>
       </c>
@@ -6352,7 +6363,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="177" ht="17" spans="1:8">
+    <row r="177" ht="17" hidden="1" spans="1:8">
       <c r="A177" s="7" t="s">
         <v>34</v>
       </c>
@@ -6378,7 +6389,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="178" ht="17" spans="1:8">
+    <row r="178" ht="17" hidden="1" spans="1:8">
       <c r="A178" s="7" t="s">
         <v>34</v>
       </c>
@@ -6404,7 +6415,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="179" spans="1:8">
+    <row r="179" hidden="1" spans="1:8">
       <c r="A179" s="7" t="s">
         <v>34</v>
       </c>
@@ -6430,7 +6441,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="180" spans="1:8">
+    <row r="180" hidden="1" spans="1:8">
       <c r="A180" s="7" t="s">
         <v>34</v>
       </c>
@@ -6456,7 +6467,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="181" spans="1:8">
+    <row r="181" hidden="1" spans="1:8">
       <c r="A181" s="7" t="s">
         <v>34</v>
       </c>
@@ -6482,7 +6493,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="182" spans="1:8">
+    <row r="182" hidden="1" spans="1:8">
       <c r="A182" s="7" t="s">
         <v>34</v>
       </c>
@@ -6508,7 +6519,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="183" spans="1:8">
+    <row r="183" hidden="1" spans="1:8">
       <c r="A183" s="7" t="s">
         <v>34</v>
       </c>
@@ -6534,7 +6545,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="184" ht="17" spans="1:8">
+    <row r="184" ht="17" hidden="1" spans="1:8">
       <c r="A184" s="16" t="s">
         <v>25</v>
       </c>
@@ -6560,7 +6571,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="185" ht="17" spans="1:8">
+    <row r="185" ht="17" hidden="1" spans="1:8">
       <c r="A185" s="16" t="s">
         <v>25</v>
       </c>
@@ -6586,7 +6597,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="186" ht="17" spans="1:8">
+    <row r="186" ht="17" hidden="1" spans="1:8">
       <c r="A186" s="16" t="s">
         <v>25</v>
       </c>
@@ -6612,7 +6623,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="187" ht="17" spans="1:8">
+    <row r="187" ht="17" hidden="1" spans="1:8">
       <c r="A187" s="16" t="s">
         <v>25</v>
       </c>
@@ -6638,7 +6649,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="188" ht="17" spans="1:8">
+    <row r="188" ht="17" hidden="1" spans="1:8">
       <c r="A188" s="16" t="s">
         <v>25</v>
       </c>
@@ -6664,7 +6675,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="189" ht="17" spans="1:8">
+    <row r="189" ht="17" hidden="1" spans="1:8">
       <c r="A189" s="16" t="s">
         <v>25</v>
       </c>
@@ -6690,7 +6701,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="190" ht="17" spans="1:8">
+    <row r="190" ht="17" hidden="1" spans="1:8">
       <c r="A190" s="16" t="s">
         <v>25</v>
       </c>
@@ -6716,7 +6727,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="191" ht="17" spans="1:8">
+    <row r="191" ht="17" hidden="1" spans="1:8">
       <c r="A191" s="16" t="s">
         <v>25</v>
       </c>
@@ -6742,7 +6753,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="192" ht="17" spans="1:8">
+    <row r="192" ht="17" hidden="1" spans="1:8">
       <c r="A192" s="16" t="s">
         <v>25</v>
       </c>
@@ -6768,7 +6779,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="193" ht="17" spans="1:8">
+    <row r="193" ht="17" hidden="1" spans="1:8">
       <c r="A193" s="16" t="s">
         <v>25</v>
       </c>
@@ -6794,7 +6805,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="194" ht="17" spans="1:8">
+    <row r="194" ht="17" hidden="1" spans="1:8">
       <c r="A194" s="16" t="s">
         <v>25</v>
       </c>
@@ -6820,7 +6831,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="195" ht="17" spans="1:8">
+    <row r="195" ht="17" hidden="1" spans="1:8">
       <c r="A195" s="16" t="s">
         <v>25</v>
       </c>
@@ -6846,7 +6857,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="196" ht="17" spans="1:8">
+    <row r="196" ht="17" hidden="1" spans="1:8">
       <c r="A196" s="16" t="s">
         <v>25</v>
       </c>
@@ -6872,7 +6883,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="197" ht="17" spans="1:8">
+    <row r="197" ht="17" hidden="1" spans="1:8">
       <c r="A197" s="16" t="s">
         <v>25</v>
       </c>
@@ -6898,7 +6909,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="198" ht="17" spans="1:8">
+    <row r="198" ht="17" hidden="1" spans="1:8">
       <c r="A198" s="16" t="s">
         <v>25</v>
       </c>
@@ -6924,7 +6935,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="199" ht="17" spans="1:8">
+    <row r="199" ht="17" hidden="1" spans="1:8">
       <c r="A199" s="16" t="s">
         <v>25</v>
       </c>
@@ -6950,7 +6961,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="200" ht="17" spans="1:8">
+    <row r="200" ht="17" hidden="1" spans="1:8">
       <c r="A200" s="16" t="s">
         <v>25</v>
       </c>
@@ -6976,7 +6987,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="201" ht="17" spans="1:8">
+    <row r="201" ht="17" hidden="1" spans="1:8">
       <c r="A201" s="16" t="s">
         <v>25</v>
       </c>
@@ -7002,7 +7013,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="202" ht="17" spans="1:8">
+    <row r="202" ht="17" hidden="1" spans="1:8">
       <c r="A202" s="16" t="s">
         <v>25</v>
       </c>
@@ -7028,7 +7039,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="203" ht="17" spans="1:8">
+    <row r="203" ht="17" hidden="1" spans="1:8">
       <c r="A203" s="16" t="s">
         <v>25</v>
       </c>
@@ -7054,7 +7065,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="204" ht="17" spans="1:8">
+    <row r="204" ht="17" hidden="1" spans="1:8">
       <c r="A204" s="16" t="s">
         <v>25</v>
       </c>
@@ -7080,7 +7091,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="205" ht="17" spans="1:8">
+    <row r="205" ht="17" hidden="1" spans="1:8">
       <c r="A205" s="16" t="s">
         <v>35</v>
       </c>
@@ -7106,7 +7117,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="206" ht="17" spans="1:8">
+    <row r="206" ht="17" hidden="1" spans="1:8">
       <c r="A206" s="16" t="s">
         <v>35</v>
       </c>
@@ -7132,7 +7143,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="207" ht="17" spans="1:8">
+    <row r="207" ht="17" hidden="1" spans="1:8">
       <c r="A207" s="16" t="s">
         <v>35</v>
       </c>
@@ -7158,7 +7169,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="208" ht="17" spans="1:8">
+    <row r="208" ht="17" hidden="1" spans="1:8">
       <c r="A208" s="16" t="s">
         <v>35</v>
       </c>
@@ -7184,7 +7195,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="209" ht="17" spans="1:8">
+    <row r="209" ht="17" hidden="1" spans="1:8">
       <c r="A209" s="16" t="s">
         <v>35</v>
       </c>
@@ -7210,7 +7221,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="210" ht="17" spans="1:8">
+    <row r="210" ht="17" hidden="1" spans="1:8">
       <c r="A210" s="16" t="s">
         <v>35</v>
       </c>
@@ -7236,7 +7247,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="211" ht="17" spans="1:8">
+    <row r="211" ht="17" hidden="1" spans="1:8">
       <c r="A211" s="16" t="s">
         <v>35</v>
       </c>
@@ -7262,7 +7273,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="212" ht="17" spans="1:8">
+    <row r="212" ht="17" hidden="1" spans="1:8">
       <c r="A212" s="16" t="s">
         <v>35</v>
       </c>
@@ -7288,7 +7299,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="213" ht="17" spans="1:8">
+    <row r="213" ht="17" hidden="1" spans="1:8">
       <c r="A213" s="16" t="s">
         <v>35</v>
       </c>
@@ -7314,7 +7325,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="214" ht="17" spans="1:8">
+    <row r="214" ht="17" hidden="1" spans="1:8">
       <c r="A214" s="16" t="s">
         <v>35</v>
       </c>
@@ -7340,7 +7351,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="215" ht="17" spans="1:8">
+    <row r="215" ht="17" hidden="1" spans="1:8">
       <c r="A215" s="16" t="s">
         <v>35</v>
       </c>
@@ -7366,7 +7377,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="216" ht="17" spans="1:8">
+    <row r="216" ht="17" hidden="1" spans="1:8">
       <c r="A216" s="16" t="s">
         <v>35</v>
       </c>
@@ -7392,7 +7403,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="217" ht="17" spans="1:8">
+    <row r="217" ht="17" hidden="1" spans="1:8">
       <c r="A217" s="16" t="s">
         <v>35</v>
       </c>
@@ -7418,7 +7429,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="218" ht="17" spans="1:8">
+    <row r="218" ht="17" hidden="1" spans="1:8">
       <c r="A218" s="16" t="s">
         <v>35</v>
       </c>
@@ -7444,7 +7455,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="219" ht="17" spans="1:8">
+    <row r="219" ht="17" hidden="1" spans="1:8">
       <c r="A219" s="16" t="s">
         <v>35</v>
       </c>
@@ -7470,7 +7481,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="220" spans="1:8">
+    <row r="220" hidden="1" spans="1:8">
       <c r="A220" s="7" t="s">
         <v>36</v>
       </c>
@@ -7496,7 +7507,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="221" spans="1:8">
+    <row r="221" hidden="1" spans="1:8">
       <c r="A221" s="7" t="s">
         <v>36</v>
       </c>
@@ -7522,7 +7533,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="222" spans="1:8">
+    <row r="222" hidden="1" spans="1:8">
       <c r="A222" s="7" t="s">
         <v>36</v>
       </c>
@@ -7548,7 +7559,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="223" spans="1:8">
+    <row r="223" hidden="1" spans="1:8">
       <c r="A223" s="7" t="s">
         <v>36</v>
       </c>
@@ -7574,7 +7585,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="224" spans="1:8">
+    <row r="224" hidden="1" spans="1:8">
       <c r="A224" s="7" t="s">
         <v>36</v>
       </c>
@@ -7600,7 +7611,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="225" spans="1:8">
+    <row r="225" hidden="1" spans="1:8">
       <c r="A225" s="7" t="s">
         <v>36</v>
       </c>
@@ -7626,7 +7637,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="226" spans="1:8">
+    <row r="226" hidden="1" spans="1:8">
       <c r="A226" s="7" t="s">
         <v>36</v>
       </c>
@@ -7652,7 +7663,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="227" spans="1:8">
+    <row r="227" hidden="1" spans="1:8">
       <c r="A227" s="7" t="s">
         <v>36</v>
       </c>
@@ -7678,7 +7689,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="228" spans="1:8">
+    <row r="228" hidden="1" spans="1:8">
       <c r="A228" s="7" t="s">
         <v>36</v>
       </c>
@@ -7704,7 +7715,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="229" ht="17" spans="1:8">
+    <row r="229" ht="17" hidden="1" spans="1:8">
       <c r="A229" s="7" t="s">
         <v>36</v>
       </c>
@@ -7730,7 +7741,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="230" ht="17" spans="1:8">
+    <row r="230" ht="17" hidden="1" spans="1:8">
       <c r="A230" s="7" t="s">
         <v>36</v>
       </c>
@@ -7756,7 +7767,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="231" ht="17" spans="1:8">
+    <row r="231" ht="17" hidden="1" spans="1:8">
       <c r="A231" s="7" t="s">
         <v>36</v>
       </c>
@@ -7782,7 +7793,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="232" spans="1:8">
+    <row r="232" hidden="1" spans="1:8">
       <c r="A232" s="7" t="s">
         <v>36</v>
       </c>
@@ -7808,7 +7819,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="233" spans="1:8">
+    <row r="233" hidden="1" spans="1:8">
       <c r="A233" s="7" t="s">
         <v>36</v>
       </c>
@@ -7834,7 +7845,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="234" spans="1:8">
+    <row r="234" hidden="1" spans="1:8">
       <c r="A234" s="7" t="s">
         <v>36</v>
       </c>
@@ -7860,7 +7871,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="235" spans="1:8">
+    <row r="235" hidden="1" spans="1:8">
       <c r="A235" s="7" t="s">
         <v>36</v>
       </c>
@@ -7886,7 +7897,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="236" spans="1:8">
+    <row r="236" hidden="1" spans="1:8">
       <c r="A236" s="7" t="s">
         <v>36</v>
       </c>
@@ -7912,7 +7923,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="237" ht="17" spans="1:8">
+    <row r="237" ht="17" hidden="1" spans="1:8">
       <c r="A237" s="16" t="s">
         <v>33</v>
       </c>
@@ -7928,7 +7939,7 @@
       <c r="E237" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F237" s="40">
+      <c r="F237" s="37">
         <v>120</v>
       </c>
       <c r="G237" s="11">
@@ -7938,7 +7949,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="238" ht="17" spans="1:8">
+    <row r="238" ht="17" hidden="1" spans="1:8">
       <c r="A238" s="16" t="s">
         <v>33</v>
       </c>
@@ -7954,7 +7965,7 @@
       <c r="E238" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F238" s="41">
+      <c r="F238" s="33">
         <v>200</v>
       </c>
       <c r="G238" s="11">
@@ -7964,7 +7975,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="239" ht="17" spans="1:8">
+    <row r="239" ht="17" hidden="1" spans="1:8">
       <c r="A239" s="16" t="s">
         <v>33</v>
       </c>
@@ -7980,7 +7991,7 @@
       <c r="E239" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F239" s="41">
+      <c r="F239" s="33">
         <v>350</v>
       </c>
       <c r="G239" s="11">
@@ -7990,7 +8001,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="240" ht="17" spans="1:8">
+    <row r="240" ht="17" hidden="1" spans="1:8">
       <c r="A240" s="16" t="s">
         <v>33</v>
       </c>
@@ -8006,7 +8017,7 @@
       <c r="E240" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F240" s="41">
+      <c r="F240" s="33">
         <v>400</v>
       </c>
       <c r="G240" s="11">
@@ -8016,7 +8027,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="241" ht="17" spans="1:8">
+    <row r="241" ht="17" hidden="1" spans="1:8">
       <c r="A241" s="16" t="s">
         <v>33</v>
       </c>
@@ -8032,7 +8043,7 @@
       <c r="E241" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F241" s="41">
+      <c r="F241" s="33">
         <v>550</v>
       </c>
       <c r="G241" s="11">
@@ -8042,7 +8053,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="242" ht="17" spans="1:8">
+    <row r="242" ht="17" hidden="1" spans="1:8">
       <c r="A242" s="16" t="s">
         <v>33</v>
       </c>
@@ -8058,7 +8069,7 @@
       <c r="E242" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F242" s="41">
+      <c r="F242" s="33">
         <v>100</v>
       </c>
       <c r="G242" s="11">
@@ -8068,7 +8079,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="243" ht="17" spans="1:8">
+    <row r="243" ht="17" hidden="1" spans="1:8">
       <c r="A243" s="16" t="s">
         <v>33</v>
       </c>
@@ -8084,7 +8095,7 @@
       <c r="E243" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F243" s="41">
+      <c r="F243" s="33">
         <v>320</v>
       </c>
       <c r="G243" s="11">
@@ -8094,7 +8105,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="244" ht="17" spans="1:8">
+    <row r="244" ht="17" hidden="1" spans="1:8">
       <c r="A244" s="16" t="s">
         <v>33</v>
       </c>
@@ -8110,7 +8121,7 @@
       <c r="E244" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F244" s="41">
+      <c r="F244" s="33">
         <v>240</v>
       </c>
       <c r="G244" s="11">
@@ -8120,7 +8131,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="245" ht="17" spans="1:8">
+    <row r="245" ht="17" hidden="1" spans="1:8">
       <c r="A245" s="16" t="s">
         <v>33</v>
       </c>
@@ -8136,7 +8147,7 @@
       <c r="E245" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F245" s="41">
+      <c r="F245" s="33">
         <v>240</v>
       </c>
       <c r="G245" s="11">
@@ -8146,7 +8157,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="246" ht="17" spans="1:8">
+    <row r="246" ht="17" hidden="1" spans="1:8">
       <c r="A246" s="16" t="s">
         <v>33</v>
       </c>
@@ -8162,7 +8173,7 @@
       <c r="E246" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F246" s="40">
+      <c r="F246" s="37">
         <v>50</v>
       </c>
       <c r="G246" s="11">
@@ -8172,7 +8183,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="247" ht="17" spans="1:8">
+    <row r="247" ht="17" hidden="1" spans="1:8">
       <c r="A247" s="16" t="s">
         <v>33</v>
       </c>
@@ -8188,7 +8199,7 @@
       <c r="E247" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F247" s="40">
+      <c r="F247" s="37">
         <v>200</v>
       </c>
       <c r="G247" s="11">
@@ -8198,7 +8209,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="248" ht="17" spans="1:8">
+    <row r="248" ht="17" hidden="1" spans="1:8">
       <c r="A248" s="16" t="s">
         <v>33</v>
       </c>
@@ -8214,7 +8225,7 @@
       <c r="E248" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F248" s="40">
+      <c r="F248" s="37">
         <v>200</v>
       </c>
       <c r="G248" s="11">
@@ -8224,7 +8235,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="249" ht="17" spans="1:8">
+    <row r="249" ht="17" hidden="1" spans="1:8">
       <c r="A249" s="16" t="s">
         <v>33</v>
       </c>
@@ -8240,7 +8251,7 @@
       <c r="E249" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F249" s="40">
+      <c r="F249" s="37">
         <v>200</v>
       </c>
       <c r="G249" s="11">
@@ -8250,7 +8261,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="250" ht="17" spans="1:8">
+    <row r="250" ht="17" hidden="1" spans="1:8">
       <c r="A250" s="16" t="s">
         <v>33</v>
       </c>
@@ -8266,7 +8277,7 @@
       <c r="E250" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F250" s="41">
+      <c r="F250" s="33">
         <v>2050</v>
       </c>
       <c r="G250" s="11">
@@ -8276,7 +8287,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="251" ht="17" spans="1:8">
+    <row r="251" ht="17" hidden="1" spans="1:8">
       <c r="A251" s="16" t="s">
         <v>33</v>
       </c>
@@ -8292,7 +8303,7 @@
       <c r="E251" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F251" s="41">
+      <c r="F251" s="33">
         <v>2050</v>
       </c>
       <c r="G251" s="11">
@@ -8302,7 +8313,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="252" ht="17" spans="1:8">
+    <row r="252" ht="17" hidden="1" spans="1:8">
       <c r="A252" s="16" t="s">
         <v>33</v>
       </c>
@@ -8318,7 +8329,7 @@
       <c r="E252" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F252" s="41">
+      <c r="F252" s="33">
         <v>2050</v>
       </c>
       <c r="G252" s="11">
@@ -8328,7 +8339,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="253" ht="17" spans="1:8">
+    <row r="253" ht="17" hidden="1" spans="1:8">
       <c r="A253" s="16" t="s">
         <v>33</v>
       </c>
@@ -8344,7 +8355,7 @@
       <c r="E253" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F253" s="41">
+      <c r="F253" s="33">
         <v>2050</v>
       </c>
       <c r="G253" s="11">
@@ -8354,7 +8365,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="254" ht="17" spans="1:8">
+    <row r="254" ht="17" hidden="1" spans="1:8">
       <c r="A254" s="16" t="s">
         <v>33</v>
       </c>
@@ -8370,7 +8381,7 @@
       <c r="E254" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F254" s="42">
+      <c r="F254" s="40">
         <v>200</v>
       </c>
       <c r="G254" s="11">
@@ -8380,7 +8391,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="255" ht="17" spans="1:8">
+    <row r="255" ht="17" hidden="1" spans="1:8">
       <c r="A255" s="16" t="s">
         <v>33</v>
       </c>
@@ -8396,7 +8407,7 @@
       <c r="E255" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F255" s="42">
+      <c r="F255" s="40">
         <v>200</v>
       </c>
       <c r="G255" s="11">
@@ -8406,7 +8417,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="256" ht="17" spans="1:8">
+    <row r="256" ht="17" hidden="1" spans="1:8">
       <c r="A256" s="16" t="s">
         <v>33</v>
       </c>
@@ -8422,7 +8433,7 @@
       <c r="E256" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F256" s="42">
+      <c r="F256" s="40">
         <v>200</v>
       </c>
       <c r="G256" s="11">
@@ -8432,7 +8443,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="257" ht="17" spans="1:8">
+    <row r="257" ht="17" hidden="1" spans="1:8">
       <c r="A257" s="16" t="s">
         <v>33</v>
       </c>
@@ -8448,7 +8459,7 @@
       <c r="E257" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F257" s="42">
+      <c r="F257" s="40">
         <v>200</v>
       </c>
       <c r="G257" s="11">
@@ -8458,7 +8469,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="258" ht="17" spans="1:8">
+    <row r="258" ht="17" hidden="1" spans="1:8">
       <c r="A258" s="16" t="s">
         <v>37</v>
       </c>
@@ -8474,7 +8485,7 @@
       <c r="E258" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F258" s="40">
+      <c r="F258" s="37">
         <v>150</v>
       </c>
       <c r="G258" s="11">
@@ -8484,7 +8495,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="259" ht="17" spans="1:8">
+    <row r="259" ht="17" hidden="1" spans="1:8">
       <c r="A259" s="16" t="s">
         <v>37</v>
       </c>
@@ -8500,7 +8511,7 @@
       <c r="E259" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F259" s="40">
+      <c r="F259" s="37">
         <v>300</v>
       </c>
       <c r="G259" s="11">
@@ -8510,7 +8521,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="260" ht="17" spans="1:8">
+    <row r="260" ht="17" hidden="1" spans="1:8">
       <c r="A260" s="16" t="s">
         <v>37</v>
       </c>
@@ -8526,7 +8537,7 @@
       <c r="E260" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F260" s="40">
+      <c r="F260" s="37">
         <v>300</v>
       </c>
       <c r="G260" s="11">
@@ -8536,7 +8547,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="261" ht="17" spans="1:8">
+    <row r="261" ht="17" hidden="1" spans="1:8">
       <c r="A261" s="16" t="s">
         <v>37</v>
       </c>
@@ -8552,7 +8563,7 @@
       <c r="E261" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F261" s="43">
+      <c r="F261" s="38">
         <v>120</v>
       </c>
       <c r="G261" s="11">
@@ -8562,7 +8573,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="262" ht="17" spans="1:8">
+    <row r="262" ht="17" hidden="1" spans="1:8">
       <c r="A262" s="16" t="s">
         <v>37</v>
       </c>
@@ -8578,7 +8589,7 @@
       <c r="E262" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F262" s="40">
+      <c r="F262" s="37">
         <v>1300</v>
       </c>
       <c r="G262" s="11">
@@ -8588,7 +8599,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="263" ht="17" spans="1:8">
+    <row r="263" ht="17" hidden="1" spans="1:8">
       <c r="A263" s="16" t="s">
         <v>37</v>
       </c>
@@ -8604,7 +8615,7 @@
       <c r="E263" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F263" s="40">
+      <c r="F263" s="37">
         <v>1300</v>
       </c>
       <c r="G263" s="11">
@@ -8614,7 +8625,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="264" ht="17" spans="1:8">
+    <row r="264" ht="17" hidden="1" spans="1:8">
       <c r="A264" s="16" t="s">
         <v>37</v>
       </c>
@@ -8640,7 +8651,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="265" ht="17" spans="1:8">
+    <row r="265" ht="17" hidden="1" spans="1:8">
       <c r="A265" s="16" t="s">
         <v>37</v>
       </c>
@@ -8656,7 +8667,7 @@
       <c r="E265" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F265" s="40">
+      <c r="F265" s="37">
         <v>400</v>
       </c>
       <c r="G265" s="11">
@@ -8666,7 +8677,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="266" ht="17" spans="1:8">
+    <row r="266" ht="17" hidden="1" spans="1:8">
       <c r="A266" s="16" t="s">
         <v>37</v>
       </c>
@@ -8682,7 +8693,7 @@
       <c r="E266" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F266" s="40">
+      <c r="F266" s="37">
         <v>400</v>
       </c>
       <c r="G266" s="11">
@@ -8692,7 +8703,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="267" ht="17" spans="1:8">
+    <row r="267" ht="17" hidden="1" spans="1:8">
       <c r="A267" s="16" t="s">
         <v>37</v>
       </c>
@@ -8718,7 +8729,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="268" ht="17" spans="1:8">
+    <row r="268" ht="17" hidden="1" spans="1:8">
       <c r="A268" s="16" t="s">
         <v>37</v>
       </c>
@@ -8734,7 +8745,7 @@
       <c r="E268" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F268" s="40">
+      <c r="F268" s="37">
         <v>700</v>
       </c>
       <c r="G268" s="11">
@@ -8744,7 +8755,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="269" ht="17" spans="1:8">
+    <row r="269" ht="17" hidden="1" spans="1:8">
       <c r="A269" s="16" t="s">
         <v>37</v>
       </c>
@@ -8760,7 +8771,7 @@
       <c r="E269" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F269" s="40">
+      <c r="F269" s="37">
         <v>700</v>
       </c>
       <c r="G269" s="11">
@@ -8770,7 +8781,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="270" ht="17" spans="1:8">
+    <row r="270" ht="17" hidden="1" spans="1:8">
       <c r="A270" s="16" t="s">
         <v>37</v>
       </c>
@@ -8786,7 +8797,7 @@
       <c r="E270" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F270" s="43">
+      <c r="F270" s="38">
         <v>100</v>
       </c>
       <c r="G270" s="11">
@@ -8796,7 +8807,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="271" ht="17" spans="1:8">
+    <row r="271" ht="17" hidden="1" spans="1:8">
       <c r="A271" s="16" t="s">
         <v>37</v>
       </c>
@@ -8812,7 +8823,7 @@
       <c r="E271" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F271" s="40">
+      <c r="F271" s="37">
         <v>235</v>
       </c>
       <c r="G271" s="11">
@@ -8822,7 +8833,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="272" ht="17" spans="1:8">
+    <row r="272" ht="17" hidden="1" spans="1:8">
       <c r="A272" s="16" t="s">
         <v>37</v>
       </c>
@@ -8838,7 +8849,7 @@
       <c r="E272" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F272" s="40">
+      <c r="F272" s="37">
         <v>1100</v>
       </c>
       <c r="G272" s="11">
@@ -8848,8 +8859,460 @@
         <v>46226</v>
       </c>
     </row>
+    <row r="273" ht="17.55" spans="1:8">
+      <c r="A273" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B273" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C273" s="8">
+        <v>0</v>
+      </c>
+      <c r="D273" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E273" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F273" s="41">
+        <v>150</v>
+      </c>
+      <c r="G273" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H273" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="274" spans="1:8">
+      <c r="A274" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B274" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C274" s="9">
+        <v>0</v>
+      </c>
+      <c r="D274" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E274" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F274" s="41">
+        <v>350</v>
+      </c>
+      <c r="G274" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H274" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="275" spans="1:8">
+      <c r="A275" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B275" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C275" s="9">
+        <v>0</v>
+      </c>
+      <c r="D275" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E275" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F275" s="41">
+        <v>350</v>
+      </c>
+      <c r="G275" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H275" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="276" spans="1:8">
+      <c r="A276" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B276" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C276" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D276" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E276" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F276" s="42">
+        <v>300</v>
+      </c>
+      <c r="G276" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H276" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="277" spans="1:8">
+      <c r="A277" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B277" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C277" s="9">
+        <v>990</v>
+      </c>
+      <c r="D277" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E277" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F277" s="42">
+        <v>1100</v>
+      </c>
+      <c r="G277" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H277" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="278" spans="1:8">
+      <c r="A278" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B278" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C278" s="9">
+        <v>990</v>
+      </c>
+      <c r="D278" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E278" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F278" s="42">
+        <v>1100</v>
+      </c>
+      <c r="G278" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H278" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="279" spans="1:8">
+      <c r="A279" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B279" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C279" s="9">
+        <v>990</v>
+      </c>
+      <c r="D279" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E279" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F279" s="42">
+        <v>100</v>
+      </c>
+      <c r="G279" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H279" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="280" spans="1:8">
+      <c r="A280" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B280" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C280" s="9">
+        <v>990</v>
+      </c>
+      <c r="D280" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E280" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F280" s="42">
+        <v>550</v>
+      </c>
+      <c r="G280" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H280" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="281" spans="1:8">
+      <c r="A281" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B281" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C281" s="9">
+        <v>990</v>
+      </c>
+      <c r="D281" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E281" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F281" s="42">
+        <v>550</v>
+      </c>
+      <c r="G281" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H281" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="282" ht="17" spans="1:8">
+      <c r="A282" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B282" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C282" s="9">
+        <v>990</v>
+      </c>
+      <c r="D282" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E282" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F282" s="43">
+        <v>50</v>
+      </c>
+      <c r="G282" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H282" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="283" ht="17" spans="1:8">
+      <c r="A283" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B283" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C283" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D283" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E283" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F283" s="43">
+        <v>300</v>
+      </c>
+      <c r="G283" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H283" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="284" ht="17" spans="1:8">
+      <c r="A284" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B284" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C284" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D284" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E284" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F284" s="43">
+        <v>410</v>
+      </c>
+      <c r="G284" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H284" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="285" spans="1:8">
+      <c r="A285" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B285" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C285" s="9">
+        <v>100</v>
+      </c>
+      <c r="D285" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E285" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F285" s="44">
+        <v>650</v>
+      </c>
+      <c r="G285" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H285" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="286" spans="1:8">
+      <c r="A286" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B286" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C286" s="9">
+        <v>100</v>
+      </c>
+      <c r="D286" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E286" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F286" s="44">
+        <v>800</v>
+      </c>
+      <c r="G286" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H286" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="287" spans="1:8">
+      <c r="A287" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B287" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C287" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D287" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E287" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F287" s="44">
+        <v>450</v>
+      </c>
+      <c r="G287" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H287" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="288" spans="1:8">
+      <c r="A288" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B288" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C288" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D288" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E288" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F288" s="42">
+        <v>450</v>
+      </c>
+      <c r="G288" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H288" s="11">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="289" spans="1:8">
+      <c r="A289" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B289" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C289" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D289" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E289" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F289" s="44">
+        <v>450</v>
+      </c>
+      <c r="G289" s="11">
+        <v>46239</v>
+      </c>
+      <c r="H289" s="11">
+        <v>46232</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H272" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H289" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="秋_2"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="3">
+      <filters>
+        <filter val="初中"/>
+      </filters>
+    </filterColumn>
     <extLst/>
   </autoFilter>
   <sortState ref="A2:F79">

</xml_diff>

<commit_message>
Publish dashboard sorting and latest data
</commit_message>
<xml_diff>
--- a/tongji_target.xlsx
+++ b/tongji_target.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$289</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$321</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1288" uniqueCount="40">
   <si>
     <t>期次</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>秋_2</t>
+  </si>
+  <si>
+    <t>暑_16</t>
   </si>
 </sst>
 </file>
@@ -945,7 +948,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -959,7 +962,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1204,37 +1207,8 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
     </xf>
   </cellXfs>
   <cellStyles count="50">
@@ -1776,7 +1750,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H289"/>
+  <dimension ref="A1:H321"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.3076923076923" style="2" customWidth="1"/>
@@ -8859,7 +8833,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="273" ht="17.55" spans="1:8">
+    <row r="273" spans="1:8">
       <c r="A273" s="7" t="s">
         <v>38</v>
       </c>
@@ -8875,7 +8849,7 @@
       <c r="E273" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F273" s="41">
+      <c r="F273" s="31">
         <v>150</v>
       </c>
       <c r="G273" s="11">
@@ -8901,7 +8875,7 @@
       <c r="E274" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F274" s="41">
+      <c r="F274" s="31">
         <v>350</v>
       </c>
       <c r="G274" s="11">
@@ -8927,7 +8901,7 @@
       <c r="E275" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F275" s="41">
+      <c r="F275" s="31">
         <v>350</v>
       </c>
       <c r="G275" s="11">
@@ -8953,7 +8927,7 @@
       <c r="E276" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F276" s="42">
+      <c r="F276" s="32">
         <v>300</v>
       </c>
       <c r="G276" s="11">
@@ -8979,7 +8953,7 @@
       <c r="E277" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F277" s="42">
+      <c r="F277" s="32">
         <v>1100</v>
       </c>
       <c r="G277" s="11">
@@ -9005,7 +8979,7 @@
       <c r="E278" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F278" s="42">
+      <c r="F278" s="32">
         <v>1100</v>
       </c>
       <c r="G278" s="11">
@@ -9031,7 +9005,7 @@
       <c r="E279" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F279" s="42">
+      <c r="F279" s="32">
         <v>100</v>
       </c>
       <c r="G279" s="11">
@@ -9057,7 +9031,7 @@
       <c r="E280" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F280" s="42">
+      <c r="F280" s="32">
         <v>550</v>
       </c>
       <c r="G280" s="11">
@@ -9083,7 +9057,7 @@
       <c r="E281" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F281" s="42">
+      <c r="F281" s="32">
         <v>550</v>
       </c>
       <c r="G281" s="11">
@@ -9101,7 +9075,7 @@
         <v>16</v>
       </c>
       <c r="C282" s="9">
-        <v>990</v>
+        <v>1880</v>
       </c>
       <c r="D282" s="8" t="s">
         <v>10</v>
@@ -9109,7 +9083,7 @@
       <c r="E282" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F282" s="43">
+      <c r="F282" s="33">
         <v>50</v>
       </c>
       <c r="G282" s="11">
@@ -9135,7 +9109,7 @@
       <c r="E283" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F283" s="43">
+      <c r="F283" s="33">
         <v>300</v>
       </c>
       <c r="G283" s="11">
@@ -9161,7 +9135,7 @@
       <c r="E284" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F284" s="43">
+      <c r="F284" s="33">
         <v>410</v>
       </c>
       <c r="G284" s="11">
@@ -9187,7 +9161,7 @@
       <c r="E285" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F285" s="44">
+      <c r="F285" s="34">
         <v>650</v>
       </c>
       <c r="G285" s="11">
@@ -9213,7 +9187,7 @@
       <c r="E286" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F286" s="44">
+      <c r="F286" s="34">
         <v>800</v>
       </c>
       <c r="G286" s="11">
@@ -9239,7 +9213,7 @@
       <c r="E287" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F287" s="44">
+      <c r="F287" s="34">
         <v>450</v>
       </c>
       <c r="G287" s="11">
@@ -9265,7 +9239,7 @@
       <c r="E288" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F288" s="42">
+      <c r="F288" s="32">
         <v>450</v>
       </c>
       <c r="G288" s="11">
@@ -9291,7 +9265,7 @@
       <c r="E289" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F289" s="44">
+      <c r="F289" s="34">
         <v>450</v>
       </c>
       <c r="G289" s="11">
@@ -9301,8 +9275,840 @@
         <v>46232</v>
       </c>
     </row>
+    <row r="290" ht="17" hidden="1" spans="1:8">
+      <c r="A290" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B290" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C290" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D290" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E290" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F290" s="37">
+        <v>120</v>
+      </c>
+      <c r="G290" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H290" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="291" ht="17" hidden="1" spans="1:8">
+      <c r="A291" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B291" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C291" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D291" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E291" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F291" s="33">
+        <v>150</v>
+      </c>
+      <c r="G291" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H291" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="292" ht="17" hidden="1" spans="1:8">
+      <c r="A292" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B292" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C292" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D292" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E292" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F292" s="33">
+        <v>350</v>
+      </c>
+      <c r="G292" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H292" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="293" ht="17" hidden="1" spans="1:8">
+      <c r="A293" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B293" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C293" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D293" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E293" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F293" s="33">
+        <v>330</v>
+      </c>
+      <c r="G293" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H293" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="294" ht="17" hidden="1" spans="1:8">
+      <c r="A294" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B294" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C294" s="9">
+        <v>2880</v>
+      </c>
+      <c r="D294" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E294" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F294" s="33">
+        <v>400</v>
+      </c>
+      <c r="G294" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H294" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="295" ht="17" hidden="1" spans="1:8">
+      <c r="A295" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B295" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C295" s="9">
+        <v>990</v>
+      </c>
+      <c r="D295" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E295" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F295" s="33">
+        <v>100</v>
+      </c>
+      <c r="G295" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H295" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="296" ht="17" hidden="1" spans="1:8">
+      <c r="A296" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B296" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C296" s="9">
+        <v>990</v>
+      </c>
+      <c r="D296" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E296" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F296" s="33">
+        <v>320</v>
+      </c>
+      <c r="G296" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H296" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="297" ht="17" hidden="1" spans="1:8">
+      <c r="A297" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B297" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C297" s="9">
+        <v>990</v>
+      </c>
+      <c r="D297" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E297" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F297" s="33">
+        <v>240</v>
+      </c>
+      <c r="G297" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H297" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="298" ht="17" hidden="1" spans="1:8">
+      <c r="A298" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B298" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C298" s="9">
+        <v>990</v>
+      </c>
+      <c r="D298" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E298" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F298" s="33">
+        <v>240</v>
+      </c>
+      <c r="G298" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H298" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="299" ht="17" hidden="1" spans="1:8">
+      <c r="A299" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B299" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C299" s="9">
+        <v>0</v>
+      </c>
+      <c r="D299" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E299" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F299" s="37">
+        <v>60</v>
+      </c>
+      <c r="G299" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H299" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="300" ht="17" hidden="1" spans="1:8">
+      <c r="A300" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B300" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C300" s="9">
+        <v>0</v>
+      </c>
+      <c r="D300" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E300" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F300" s="37">
+        <v>180</v>
+      </c>
+      <c r="G300" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H300" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="301" ht="17" hidden="1" spans="1:8">
+      <c r="A301" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B301" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C301" s="9">
+        <v>0</v>
+      </c>
+      <c r="D301" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E301" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F301" s="37">
+        <v>180</v>
+      </c>
+      <c r="G301" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H301" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="302" ht="17" hidden="1" spans="1:8">
+      <c r="A302" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B302" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C302" s="9">
+        <v>0</v>
+      </c>
+      <c r="D302" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E302" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F302" s="37">
+        <v>180</v>
+      </c>
+      <c r="G302" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H302" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="303" ht="17" hidden="1" spans="1:8">
+      <c r="A303" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B303" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C303" s="9">
+        <v>100</v>
+      </c>
+      <c r="D303" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E303" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F303" s="33">
+        <v>2500</v>
+      </c>
+      <c r="G303" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H303" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="304" ht="17" hidden="1" spans="1:8">
+      <c r="A304" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B304" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C304" s="9">
+        <v>100</v>
+      </c>
+      <c r="D304" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E304" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F304" s="33">
+        <v>2500</v>
+      </c>
+      <c r="G304" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H304" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="305" ht="17" hidden="1" spans="1:8">
+      <c r="A305" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B305" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C305" s="9">
+        <v>100</v>
+      </c>
+      <c r="D305" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E305" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F305" s="33">
+        <v>1950</v>
+      </c>
+      <c r="G305" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H305" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="306" ht="17" hidden="1" spans="1:8">
+      <c r="A306" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B306" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C306" s="9">
+        <v>100</v>
+      </c>
+      <c r="D306" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E306" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F306" s="33">
+        <v>1850</v>
+      </c>
+      <c r="G306" s="41">
+        <v>46239</v>
+      </c>
+      <c r="H306" s="41">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="307" ht="17" hidden="1" spans="1:8">
+      <c r="A307" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B307" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C307" s="9">
+        <v>0</v>
+      </c>
+      <c r="D307" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E307" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F307" s="37">
+        <v>100</v>
+      </c>
+      <c r="G307" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H307" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="308" ht="17" hidden="1" spans="1:8">
+      <c r="A308" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B308" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C308" s="9">
+        <v>0</v>
+      </c>
+      <c r="D308" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E308" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F308" s="37">
+        <v>200</v>
+      </c>
+      <c r="G308" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H308" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="309" ht="17" hidden="1" spans="1:8">
+      <c r="A309" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B309" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C309" s="9">
+        <v>0</v>
+      </c>
+      <c r="D309" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E309" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F309" s="37">
+        <v>250</v>
+      </c>
+      <c r="G309" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H309" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="310" ht="17" hidden="1" spans="1:8">
+      <c r="A310" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B310" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C310" s="9">
+        <v>100</v>
+      </c>
+      <c r="D310" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E310" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F310" s="38">
+        <v>125</v>
+      </c>
+      <c r="G310" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H310" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="311" ht="17" hidden="1" spans="1:8">
+      <c r="A311" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B311" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C311" s="9">
+        <v>100</v>
+      </c>
+      <c r="D311" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E311" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F311" s="37">
+        <v>800</v>
+      </c>
+      <c r="G311" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H311" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="312" ht="17" hidden="1" spans="1:8">
+      <c r="A312" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B312" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C312" s="9">
+        <v>100</v>
+      </c>
+      <c r="D312" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E312" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F312" s="37">
+        <v>1200</v>
+      </c>
+      <c r="G312" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H312" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="313" ht="17" hidden="1" spans="1:8">
+      <c r="A313" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B313" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C313" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D313" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E313" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F313" s="12">
+        <v>0</v>
+      </c>
+      <c r="G313" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H313" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="314" ht="17" hidden="1" spans="1:8">
+      <c r="A314" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B314" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C314" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D314" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E314" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F314" s="37">
+        <v>450</v>
+      </c>
+      <c r="G314" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H314" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="315" ht="17" hidden="1" spans="1:8">
+      <c r="A315" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B315" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C315" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D315" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E315" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F315" s="37">
+        <v>600</v>
+      </c>
+      <c r="G315" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H315" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="316" ht="17" hidden="1" spans="1:8">
+      <c r="A316" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B316" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C316" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D316" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E316" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F316" s="20">
+        <v>0</v>
+      </c>
+      <c r="G316" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H316" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="317" ht="17" hidden="1" spans="1:8">
+      <c r="A317" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B317" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C317" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D317" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E317" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F317" s="37">
+        <v>800</v>
+      </c>
+      <c r="G317" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H317" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="318" ht="17" hidden="1" spans="1:8">
+      <c r="A318" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B318" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C318" s="9">
+        <v>1880</v>
+      </c>
+      <c r="D318" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E318" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F318" s="37">
+        <v>900</v>
+      </c>
+      <c r="G318" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H318" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="319" ht="17" hidden="1" spans="1:8">
+      <c r="A319" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B319" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C319" s="21">
+        <v>990</v>
+      </c>
+      <c r="D319" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E319" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F319" s="38">
+        <v>100</v>
+      </c>
+      <c r="G319" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H319" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="320" ht="17" hidden="1" spans="1:8">
+      <c r="A320" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B320" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C320" s="21">
+        <v>990</v>
+      </c>
+      <c r="D320" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E320" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F320" s="37">
+        <v>400</v>
+      </c>
+      <c r="G320" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H320" s="11">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="321" ht="17" hidden="1" spans="1:8">
+      <c r="A321" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B321" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C321" s="21">
+        <v>990</v>
+      </c>
+      <c r="D321" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E321" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F321" s="37">
+        <v>1100</v>
+      </c>
+      <c r="G321" s="11">
+        <v>46240</v>
+      </c>
+      <c r="H321" s="11">
+        <v>46233</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H289" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H321" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
       <filters>
         <filter val="秋_2"/>

</xml_diff>

<commit_message>
Fix order date daily current filtering
</commit_message>
<xml_diff>
--- a/tongji_target.xlsx
+++ b/tongji_target.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="11740"/>
+    <workbookView windowWidth="28000" windowHeight="11140"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$397</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$446</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1592" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1788" uniqueCount="44">
   <si>
     <t>期次</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t>秋_4</t>
+  </si>
+  <si>
+    <t>秋_5</t>
   </si>
 </sst>
 </file>
@@ -982,7 +985,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1329,6 +1332,62 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
     </xf>
   </cellXfs>
   <cellStyles count="50">
@@ -1870,7 +1929,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H397"/>
+  <dimension ref="A1:H446"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.3076923076923" style="3" customWidth="1"/>
@@ -1908,7 +1967,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" customFormat="1" ht="17.55" spans="1:8">
+    <row r="2" customFormat="1" hidden="1" spans="1:8">
       <c r="A2" s="8" t="s">
         <v>8</v>
       </c>
@@ -1934,7 +1993,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="3" customFormat="1" spans="1:8">
+    <row r="3" customFormat="1" hidden="1" spans="1:8">
       <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
@@ -1960,7 +2019,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="4" customFormat="1" spans="1:8">
+    <row r="4" customFormat="1" hidden="1" spans="1:8">
       <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
@@ -1986,7 +2045,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="5" customFormat="1" ht="17" spans="1:8">
+    <row r="5" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A5" s="8" t="s">
         <v>8</v>
       </c>
@@ -2012,7 +2071,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="6" customFormat="1" ht="17" spans="1:8">
+    <row r="6" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A6" s="8" t="s">
         <v>8</v>
       </c>
@@ -2038,7 +2097,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="7" customFormat="1" ht="17" spans="1:8">
+    <row r="7" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A7" s="8" t="s">
         <v>8</v>
       </c>
@@ -2064,7 +2123,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="8" customFormat="1" spans="1:8">
+    <row r="8" customFormat="1" hidden="1" spans="1:8">
       <c r="A8" s="8" t="s">
         <v>8</v>
       </c>
@@ -2090,7 +2149,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="9" customFormat="1" spans="1:8">
+    <row r="9" customFormat="1" hidden="1" spans="1:8">
       <c r="A9" s="8" t="s">
         <v>8</v>
       </c>
@@ -2116,7 +2175,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="10" customFormat="1" spans="1:8">
+    <row r="10" customFormat="1" hidden="1" spans="1:8">
       <c r="A10" s="8" t="s">
         <v>8</v>
       </c>
@@ -2142,7 +2201,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="11" customFormat="1" spans="1:8">
+    <row r="11" customFormat="1" hidden="1" spans="1:8">
       <c r="A11" s="8" t="s">
         <v>8</v>
       </c>
@@ -2168,7 +2227,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="12" customFormat="1" spans="1:8">
+    <row r="12" customFormat="1" hidden="1" spans="1:8">
       <c r="A12" s="8" t="s">
         <v>8</v>
       </c>
@@ -2194,7 +2253,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="13" customFormat="1" spans="1:8">
+    <row r="13" customFormat="1" hidden="1" spans="1:8">
       <c r="A13" s="8" t="s">
         <v>8</v>
       </c>
@@ -2220,7 +2279,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="14" customFormat="1" ht="17" spans="1:8">
+    <row r="14" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A14" s="8" t="s">
         <v>8</v>
       </c>
@@ -2246,7 +2305,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="15" customFormat="1" ht="17" spans="1:8">
+    <row r="15" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A15" s="8" t="s">
         <v>8</v>
       </c>
@@ -2272,7 +2331,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="16" customFormat="1" ht="17" spans="1:8">
+    <row r="16" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A16" s="8" t="s">
         <v>8</v>
       </c>
@@ -2298,7 +2357,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="17" customFormat="1" spans="1:8">
+    <row r="17" customFormat="1" hidden="1" spans="1:8">
       <c r="A17" s="8" t="s">
         <v>8</v>
       </c>
@@ -2324,7 +2383,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="18" customFormat="1" spans="1:8">
+    <row r="18" customFormat="1" hidden="1" spans="1:8">
       <c r="A18" s="8" t="s">
         <v>8</v>
       </c>
@@ -2350,7 +2409,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="19" customFormat="1" spans="1:8">
+    <row r="19" customFormat="1" hidden="1" spans="1:8">
       <c r="A19" s="8" t="s">
         <v>8</v>
       </c>
@@ -2376,7 +2435,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="20" customFormat="1" spans="1:8">
+    <row r="20" customFormat="1" hidden="1" spans="1:8">
       <c r="A20" s="8" t="s">
         <v>8</v>
       </c>
@@ -2402,7 +2461,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="21" customFormat="1" spans="1:8">
+    <row r="21" customFormat="1" hidden="1" spans="1:8">
       <c r="A21" s="8" t="s">
         <v>8</v>
       </c>
@@ -3650,7 +3709,7 @@
         <v>46198</v>
       </c>
     </row>
-    <row r="69" customFormat="1" spans="1:8">
+    <row r="69" customFormat="1" hidden="1" spans="1:8">
       <c r="A69" s="8" t="s">
         <v>25</v>
       </c>
@@ -3676,7 +3735,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="70" customFormat="1" spans="1:8">
+    <row r="70" customFormat="1" hidden="1" spans="1:8">
       <c r="A70" s="8" t="s">
         <v>25</v>
       </c>
@@ -3702,7 +3761,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="71" customFormat="1" spans="1:8">
+    <row r="71" customFormat="1" hidden="1" spans="1:8">
       <c r="A71" s="8" t="s">
         <v>25</v>
       </c>
@@ -3728,7 +3787,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="72" customFormat="1" spans="1:8">
+    <row r="72" customFormat="1" hidden="1" spans="1:8">
       <c r="A72" s="8" t="s">
         <v>25</v>
       </c>
@@ -3754,7 +3813,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="73" customFormat="1" spans="1:8">
+    <row r="73" customFormat="1" hidden="1" spans="1:8">
       <c r="A73" s="8" t="s">
         <v>25</v>
       </c>
@@ -3780,7 +3839,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="74" customFormat="1" spans="1:8">
+    <row r="74" customFormat="1" hidden="1" spans="1:8">
       <c r="A74" s="8" t="s">
         <v>25</v>
       </c>
@@ -3806,7 +3865,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="75" customFormat="1" spans="1:8">
+    <row r="75" customFormat="1" hidden="1" spans="1:8">
       <c r="A75" s="8" t="s">
         <v>25</v>
       </c>
@@ -3832,7 +3891,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="76" customFormat="1" spans="1:8">
+    <row r="76" customFormat="1" hidden="1" spans="1:8">
       <c r="A76" s="8" t="s">
         <v>25</v>
       </c>
@@ -3858,7 +3917,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="77" customFormat="1" spans="1:8">
+    <row r="77" customFormat="1" hidden="1" spans="1:8">
       <c r="A77" s="8" t="s">
         <v>25</v>
       </c>
@@ -3884,7 +3943,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="78" customFormat="1" ht="17" spans="1:8">
+    <row r="78" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A78" s="8" t="s">
         <v>25</v>
       </c>
@@ -3910,7 +3969,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="79" customFormat="1" ht="17" spans="1:8">
+    <row r="79" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A79" s="8" t="s">
         <v>25</v>
       </c>
@@ -3936,7 +3995,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="80" customFormat="1" ht="17" spans="1:8">
+    <row r="80" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A80" s="8" t="s">
         <v>25</v>
       </c>
@@ -3962,7 +4021,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="81" customFormat="1" spans="1:8">
+    <row r="81" customFormat="1" hidden="1" spans="1:8">
       <c r="A81" s="8" t="s">
         <v>25</v>
       </c>
@@ -3988,7 +4047,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="82" customFormat="1" spans="1:8">
+    <row r="82" customFormat="1" hidden="1" spans="1:8">
       <c r="A82" s="8" t="s">
         <v>25</v>
       </c>
@@ -4014,7 +4073,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="83" customFormat="1" spans="1:8">
+    <row r="83" customFormat="1" hidden="1" spans="1:8">
       <c r="A83" s="8" t="s">
         <v>25</v>
       </c>
@@ -4040,7 +4099,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="84" customFormat="1" spans="1:8">
+    <row r="84" customFormat="1" hidden="1" spans="1:8">
       <c r="A84" s="8" t="s">
         <v>25</v>
       </c>
@@ -4066,7 +4125,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="85" customFormat="1" spans="1:8">
+    <row r="85" customFormat="1" hidden="1" spans="1:8">
       <c r="A85" s="8" t="s">
         <v>25</v>
       </c>
@@ -5366,7 +5425,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="135" customFormat="1" spans="1:8">
+    <row r="135" customFormat="1" hidden="1" spans="1:8">
       <c r="A135" s="8" t="s">
         <v>33</v>
       </c>
@@ -5392,7 +5451,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="136" customFormat="1" spans="1:8">
+    <row r="136" customFormat="1" hidden="1" spans="1:8">
       <c r="A136" s="8" t="s">
         <v>33</v>
       </c>
@@ -5418,7 +5477,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="137" customFormat="1" spans="1:8">
+    <row r="137" customFormat="1" hidden="1" spans="1:8">
       <c r="A137" s="8" t="s">
         <v>33</v>
       </c>
@@ -5444,7 +5503,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="138" s="2" customFormat="1" spans="1:8">
+    <row r="138" s="2" customFormat="1" hidden="1" spans="1:8">
       <c r="A138" s="8" t="s">
         <v>33</v>
       </c>
@@ -5470,7 +5529,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="139" s="2" customFormat="1" spans="1:8">
+    <row r="139" s="2" customFormat="1" hidden="1" spans="1:8">
       <c r="A139" s="8" t="s">
         <v>33</v>
       </c>
@@ -5496,7 +5555,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="140" s="2" customFormat="1" spans="1:8">
+    <row r="140" s="2" customFormat="1" hidden="1" spans="1:8">
       <c r="A140" s="8" t="s">
         <v>33</v>
       </c>
@@ -5522,7 +5581,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="141" s="2" customFormat="1" spans="1:8">
+    <row r="141" s="2" customFormat="1" hidden="1" spans="1:8">
       <c r="A141" s="8" t="s">
         <v>33</v>
       </c>
@@ -5548,7 +5607,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="142" s="2" customFormat="1" spans="1:8">
+    <row r="142" s="2" customFormat="1" hidden="1" spans="1:8">
       <c r="A142" s="8" t="s">
         <v>33</v>
       </c>
@@ -5574,7 +5633,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="143" s="2" customFormat="1" spans="1:8">
+    <row r="143" s="2" customFormat="1" hidden="1" spans="1:8">
       <c r="A143" s="8" t="s">
         <v>33</v>
       </c>
@@ -5600,7 +5659,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="144" s="2" customFormat="1" ht="17" spans="1:8">
+    <row r="144" s="2" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A144" s="8" t="s">
         <v>33</v>
       </c>
@@ -5626,7 +5685,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="145" s="2" customFormat="1" ht="17" spans="1:8">
+    <row r="145" s="2" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A145" s="8" t="s">
         <v>33</v>
       </c>
@@ -5652,7 +5711,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="146" s="2" customFormat="1" ht="17" spans="1:8">
+    <row r="146" s="2" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A146" s="8" t="s">
         <v>33</v>
       </c>
@@ -5678,7 +5737,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="147" s="2" customFormat="1" spans="1:8">
+    <row r="147" s="2" customFormat="1" hidden="1" spans="1:8">
       <c r="A147" s="8" t="s">
         <v>33</v>
       </c>
@@ -5704,7 +5763,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="148" customFormat="1" spans="1:8">
+    <row r="148" customFormat="1" hidden="1" spans="1:8">
       <c r="A148" s="8" t="s">
         <v>33</v>
       </c>
@@ -5730,7 +5789,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="149" customFormat="1" spans="1:8">
+    <row r="149" customFormat="1" hidden="1" spans="1:8">
       <c r="A149" s="8" t="s">
         <v>33</v>
       </c>
@@ -5756,7 +5815,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="150" customFormat="1" spans="1:8">
+    <row r="150" customFormat="1" hidden="1" spans="1:8">
       <c r="A150" s="8" t="s">
         <v>33</v>
       </c>
@@ -5782,7 +5841,7 @@
         <v>46211</v>
       </c>
     </row>
-    <row r="151" customFormat="1" spans="1:8">
+    <row r="151" customFormat="1" hidden="1" spans="1:8">
       <c r="A151" s="8" t="s">
         <v>33</v>
       </c>
@@ -6198,7 +6257,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="167" customFormat="1" spans="1:8">
+    <row r="167" customFormat="1" hidden="1" spans="1:8">
       <c r="A167" s="8" t="s">
         <v>34</v>
       </c>
@@ -6224,7 +6283,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="168" customFormat="1" spans="1:8">
+    <row r="168" customFormat="1" hidden="1" spans="1:8">
       <c r="A168" s="8" t="s">
         <v>34</v>
       </c>
@@ -6250,7 +6309,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="169" customFormat="1" spans="1:8">
+    <row r="169" customFormat="1" hidden="1" spans="1:8">
       <c r="A169" s="8" t="s">
         <v>34</v>
       </c>
@@ -6276,7 +6335,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="170" customFormat="1" spans="1:8">
+    <row r="170" customFormat="1" hidden="1" spans="1:8">
       <c r="A170" s="8" t="s">
         <v>34</v>
       </c>
@@ -6302,7 +6361,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="171" customFormat="1" spans="1:8">
+    <row r="171" customFormat="1" hidden="1" spans="1:8">
       <c r="A171" s="8" t="s">
         <v>34</v>
       </c>
@@ -6328,7 +6387,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="172" customFormat="1" spans="1:8">
+    <row r="172" customFormat="1" hidden="1" spans="1:8">
       <c r="A172" s="8" t="s">
         <v>34</v>
       </c>
@@ -6354,7 +6413,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="173" customFormat="1" spans="1:8">
+    <row r="173" customFormat="1" hidden="1" spans="1:8">
       <c r="A173" s="8" t="s">
         <v>34</v>
       </c>
@@ -6380,7 +6439,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="174" customFormat="1" spans="1:8">
+    <row r="174" customFormat="1" hidden="1" spans="1:8">
       <c r="A174" s="8" t="s">
         <v>34</v>
       </c>
@@ -6406,7 +6465,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="175" customFormat="1" spans="1:8">
+    <row r="175" customFormat="1" hidden="1" spans="1:8">
       <c r="A175" s="8" t="s">
         <v>34</v>
       </c>
@@ -6432,7 +6491,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="176" customFormat="1" ht="17" spans="1:8">
+    <row r="176" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A176" s="8" t="s">
         <v>34</v>
       </c>
@@ -6458,7 +6517,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="177" customFormat="1" ht="17" spans="1:8">
+    <row r="177" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A177" s="8" t="s">
         <v>34</v>
       </c>
@@ -6484,7 +6543,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="178" customFormat="1" ht="17" spans="1:8">
+    <row r="178" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A178" s="8" t="s">
         <v>34</v>
       </c>
@@ -6510,7 +6569,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="179" customFormat="1" spans="1:8">
+    <row r="179" customFormat="1" hidden="1" spans="1:8">
       <c r="A179" s="8" t="s">
         <v>34</v>
       </c>
@@ -6536,7 +6595,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="180" customFormat="1" spans="1:8">
+    <row r="180" customFormat="1" hidden="1" spans="1:8">
       <c r="A180" s="8" t="s">
         <v>34</v>
       </c>
@@ -6562,7 +6621,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="181" customFormat="1" spans="1:8">
+    <row r="181" customFormat="1" hidden="1" spans="1:8">
       <c r="A181" s="8" t="s">
         <v>34</v>
       </c>
@@ -6588,7 +6647,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="182" customFormat="1" spans="1:8">
+    <row r="182" customFormat="1" hidden="1" spans="1:8">
       <c r="A182" s="8" t="s">
         <v>34</v>
       </c>
@@ -6614,7 +6673,7 @@
         <v>46218</v>
       </c>
     </row>
-    <row r="183" customFormat="1" spans="1:8">
+    <row r="183" customFormat="1" hidden="1" spans="1:8">
       <c r="A183" s="8" t="s">
         <v>34</v>
       </c>
@@ -7576,7 +7635,7 @@
         <v>46219</v>
       </c>
     </row>
-    <row r="220" customFormat="1" spans="1:8">
+    <row r="220" customFormat="1" hidden="1" spans="1:8">
       <c r="A220" s="8" t="s">
         <v>36</v>
       </c>
@@ -7602,7 +7661,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="221" customFormat="1" spans="1:8">
+    <row r="221" customFormat="1" hidden="1" spans="1:8">
       <c r="A221" s="8" t="s">
         <v>36</v>
       </c>
@@ -7628,7 +7687,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="222" customFormat="1" spans="1:8">
+    <row r="222" customFormat="1" hidden="1" spans="1:8">
       <c r="A222" s="8" t="s">
         <v>36</v>
       </c>
@@ -7654,7 +7713,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="223" customFormat="1" spans="1:8">
+    <row r="223" customFormat="1" hidden="1" spans="1:8">
       <c r="A223" s="8" t="s">
         <v>36</v>
       </c>
@@ -7680,7 +7739,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="224" customFormat="1" spans="1:8">
+    <row r="224" customFormat="1" hidden="1" spans="1:8">
       <c r="A224" s="8" t="s">
         <v>36</v>
       </c>
@@ -7706,7 +7765,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="225" customFormat="1" spans="1:8">
+    <row r="225" customFormat="1" hidden="1" spans="1:8">
       <c r="A225" s="8" t="s">
         <v>36</v>
       </c>
@@ -7732,7 +7791,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="226" customFormat="1" spans="1:8">
+    <row r="226" customFormat="1" hidden="1" spans="1:8">
       <c r="A226" s="8" t="s">
         <v>36</v>
       </c>
@@ -7758,7 +7817,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="227" customFormat="1" spans="1:8">
+    <row r="227" customFormat="1" hidden="1" spans="1:8">
       <c r="A227" s="8" t="s">
         <v>36</v>
       </c>
@@ -7784,7 +7843,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="228" customFormat="1" spans="1:8">
+    <row r="228" customFormat="1" hidden="1" spans="1:8">
       <c r="A228" s="8" t="s">
         <v>36</v>
       </c>
@@ -7810,7 +7869,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="229" customFormat="1" ht="17" spans="1:8">
+    <row r="229" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A229" s="8" t="s">
         <v>36</v>
       </c>
@@ -7836,7 +7895,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="230" customFormat="1" ht="17" spans="1:8">
+    <row r="230" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A230" s="8" t="s">
         <v>36</v>
       </c>
@@ -7862,7 +7921,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="231" customFormat="1" ht="17" spans="1:8">
+    <row r="231" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A231" s="8" t="s">
         <v>36</v>
       </c>
@@ -7888,7 +7947,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="232" customFormat="1" spans="1:8">
+    <row r="232" customFormat="1" hidden="1" spans="1:8">
       <c r="A232" s="8" t="s">
         <v>36</v>
       </c>
@@ -7914,7 +7973,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="233" customFormat="1" spans="1:8">
+    <row r="233" customFormat="1" hidden="1" spans="1:8">
       <c r="A233" s="8" t="s">
         <v>36</v>
       </c>
@@ -7940,7 +7999,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="234" customFormat="1" spans="1:8">
+    <row r="234" customFormat="1" hidden="1" spans="1:8">
       <c r="A234" s="8" t="s">
         <v>36</v>
       </c>
@@ -7966,7 +8025,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="235" customFormat="1" spans="1:8">
+    <row r="235" customFormat="1" hidden="1" spans="1:8">
       <c r="A235" s="8" t="s">
         <v>36</v>
       </c>
@@ -7992,7 +8051,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="236" customFormat="1" spans="1:8">
+    <row r="236" customFormat="1" hidden="1" spans="1:8">
       <c r="A236" s="8" t="s">
         <v>36</v>
       </c>
@@ -8954,7 +9013,7 @@
         <v>46226</v>
       </c>
     </row>
-    <row r="273" customFormat="1" spans="1:8">
+    <row r="273" customFormat="1" hidden="1" spans="1:8">
       <c r="A273" s="8" t="s">
         <v>38</v>
       </c>
@@ -8980,7 +9039,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="274" customFormat="1" spans="1:8">
+    <row r="274" customFormat="1" hidden="1" spans="1:8">
       <c r="A274" s="8" t="s">
         <v>38</v>
       </c>
@@ -9006,7 +9065,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="275" customFormat="1" spans="1:8">
+    <row r="275" customFormat="1" hidden="1" spans="1:8">
       <c r="A275" s="8" t="s">
         <v>38</v>
       </c>
@@ -9032,7 +9091,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="276" customFormat="1" spans="1:8">
+    <row r="276" customFormat="1" hidden="1" spans="1:8">
       <c r="A276" s="8" t="s">
         <v>38</v>
       </c>
@@ -9058,7 +9117,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="277" customFormat="1" spans="1:8">
+    <row r="277" customFormat="1" hidden="1" spans="1:8">
       <c r="A277" s="8" t="s">
         <v>38</v>
       </c>
@@ -9084,7 +9143,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="278" customFormat="1" spans="1:8">
+    <row r="278" customFormat="1" hidden="1" spans="1:8">
       <c r="A278" s="8" t="s">
         <v>38</v>
       </c>
@@ -9110,7 +9169,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="279" customFormat="1" spans="1:8">
+    <row r="279" customFormat="1" hidden="1" spans="1:8">
       <c r="A279" s="8" t="s">
         <v>38</v>
       </c>
@@ -9136,7 +9195,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="280" customFormat="1" spans="1:8">
+    <row r="280" customFormat="1" hidden="1" spans="1:8">
       <c r="A280" s="8" t="s">
         <v>38</v>
       </c>
@@ -9162,7 +9221,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="281" customFormat="1" spans="1:8">
+    <row r="281" customFormat="1" hidden="1" spans="1:8">
       <c r="A281" s="8" t="s">
         <v>38</v>
       </c>
@@ -9188,7 +9247,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="282" customFormat="1" ht="17" spans="1:8">
+    <row r="282" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A282" s="8" t="s">
         <v>38</v>
       </c>
@@ -9214,7 +9273,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="283" customFormat="1" ht="17" spans="1:8">
+    <row r="283" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A283" s="8" t="s">
         <v>38</v>
       </c>
@@ -9240,7 +9299,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="284" customFormat="1" ht="17" spans="1:8">
+    <row r="284" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A284" s="8" t="s">
         <v>38</v>
       </c>
@@ -9266,7 +9325,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="285" customFormat="1" spans="1:8">
+    <row r="285" customFormat="1" hidden="1" spans="1:8">
       <c r="A285" s="8" t="s">
         <v>38</v>
       </c>
@@ -9292,7 +9351,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="286" customFormat="1" spans="1:8">
+    <row r="286" customFormat="1" hidden="1" spans="1:8">
       <c r="A286" s="8" t="s">
         <v>38</v>
       </c>
@@ -9318,7 +9377,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="287" customFormat="1" spans="1:8">
+    <row r="287" customFormat="1" hidden="1" spans="1:8">
       <c r="A287" s="8" t="s">
         <v>38</v>
       </c>
@@ -9344,7 +9403,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="288" customFormat="1" spans="1:8">
+    <row r="288" customFormat="1" hidden="1" spans="1:8">
       <c r="A288" s="8" t="s">
         <v>38</v>
       </c>
@@ -9370,7 +9429,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="289" customFormat="1" spans="1:8">
+    <row r="289" customFormat="1" hidden="1" spans="1:8">
       <c r="A289" s="8" t="s">
         <v>38</v>
       </c>
@@ -10228,7 +10287,7 @@
         <v>46233</v>
       </c>
     </row>
-    <row r="322" s="1" customFormat="1" spans="1:8">
+    <row r="322" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A322" s="8" t="s">
         <v>40</v>
       </c>
@@ -10254,7 +10313,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="323" s="1" customFormat="1" spans="1:8">
+    <row r="323" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A323" s="8" t="s">
         <v>40</v>
       </c>
@@ -10280,7 +10339,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="324" s="1" customFormat="1" spans="1:8">
+    <row r="324" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A324" s="8" t="s">
         <v>40</v>
       </c>
@@ -10306,7 +10365,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="325" s="1" customFormat="1" spans="1:8">
+    <row r="325" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A325" s="8" t="s">
         <v>40</v>
       </c>
@@ -10332,7 +10391,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="326" s="1" customFormat="1" spans="1:8">
+    <row r="326" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A326" s="8" t="s">
         <v>40</v>
       </c>
@@ -10358,7 +10417,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="327" s="1" customFormat="1" spans="1:8">
+    <row r="327" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A327" s="8" t="s">
         <v>40</v>
       </c>
@@ -10384,7 +10443,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="328" s="1" customFormat="1" ht="17" spans="1:8">
+    <row r="328" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A328" s="8" t="s">
         <v>40</v>
       </c>
@@ -10410,7 +10469,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="329" s="1" customFormat="1" ht="17" spans="1:8">
+    <row r="329" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A329" s="8" t="s">
         <v>40</v>
       </c>
@@ -10436,7 +10495,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="330" s="1" customFormat="1" ht="17" spans="1:8">
+    <row r="330" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A330" s="8" t="s">
         <v>40</v>
       </c>
@@ -10462,7 +10521,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="331" s="1" customFormat="1" spans="1:8">
+    <row r="331" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A331" s="8" t="s">
         <v>40</v>
       </c>
@@ -10488,7 +10547,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="332" s="1" customFormat="1" spans="1:8">
+    <row r="332" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A332" s="8" t="s">
         <v>40</v>
       </c>
@@ -10514,7 +10573,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="333" s="1" customFormat="1" spans="1:8">
+    <row r="333" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A333" s="8" t="s">
         <v>40</v>
       </c>
@@ -10540,7 +10599,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="334" s="1" customFormat="1" ht="17" spans="1:8">
+    <row r="334" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A334" s="8" t="s">
         <v>40</v>
       </c>
@@ -10566,7 +10625,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="335" s="1" customFormat="1" ht="17" spans="1:8">
+    <row r="335" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A335" s="8" t="s">
         <v>40</v>
       </c>
@@ -10592,7 +10651,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="336" s="1" customFormat="1" ht="17" spans="1:8">
+    <row r="336" s="1" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A336" s="8" t="s">
         <v>40</v>
       </c>
@@ -10618,7 +10677,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="337" s="1" customFormat="1" spans="1:8">
+    <row r="337" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A337" s="8" t="s">
         <v>40</v>
       </c>
@@ -10644,7 +10703,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="338" s="1" customFormat="1" spans="1:8">
+    <row r="338" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A338" s="8" t="s">
         <v>40</v>
       </c>
@@ -10670,7 +10729,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="339" s="1" customFormat="1" spans="1:8">
+    <row r="339" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A339" s="8" t="s">
         <v>40</v>
       </c>
@@ -10696,7 +10755,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="340" s="1" customFormat="1" spans="1:8">
+    <row r="340" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A340" s="8" t="s">
         <v>40</v>
       </c>
@@ -10722,7 +10781,7 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="341" s="1" customFormat="1" spans="1:8">
+    <row r="341" s="1" customFormat="1" hidden="1" spans="1:8">
       <c r="A341" s="8" t="s">
         <v>40</v>
       </c>
@@ -11684,7 +11743,7 @@
         <v>46240</v>
       </c>
     </row>
-    <row r="378" spans="1:8">
+    <row r="378" hidden="1" spans="1:8">
       <c r="A378" s="8" t="s">
         <v>42</v>
       </c>
@@ -11710,7 +11769,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="379" spans="1:8">
+    <row r="379" hidden="1" spans="1:8">
       <c r="A379" s="8" t="s">
         <v>42</v>
       </c>
@@ -11736,7 +11795,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="380" spans="1:8">
+    <row r="380" hidden="1" spans="1:8">
       <c r="A380" s="8" t="s">
         <v>42</v>
       </c>
@@ -11762,7 +11821,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="381" ht="17" spans="1:8">
+    <row r="381" ht="17" hidden="1" spans="1:8">
       <c r="A381" s="8" t="s">
         <v>42</v>
       </c>
@@ -11788,7 +11847,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="382" ht="17" spans="1:8">
+    <row r="382" ht="17" hidden="1" spans="1:8">
       <c r="A382" s="8" t="s">
         <v>42</v>
       </c>
@@ -11814,7 +11873,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="383" ht="17" spans="1:8">
+    <row r="383" ht="17" hidden="1" spans="1:8">
       <c r="A383" s="8" t="s">
         <v>42</v>
       </c>
@@ -11840,7 +11899,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="384" ht="17" spans="1:8">
+    <row r="384" ht="17" hidden="1" spans="1:8">
       <c r="A384" s="8" t="s">
         <v>42</v>
       </c>
@@ -11866,7 +11925,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="385" ht="17" spans="1:8">
+    <row r="385" ht="17" hidden="1" spans="1:8">
       <c r="A385" s="8" t="s">
         <v>42</v>
       </c>
@@ -11892,7 +11951,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="386" ht="17" spans="1:8">
+    <row r="386" ht="17" hidden="1" spans="1:8">
       <c r="A386" s="8" t="s">
         <v>42</v>
       </c>
@@ -11918,7 +11977,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="387" spans="1:8">
+    <row r="387" hidden="1" spans="1:8">
       <c r="A387" s="8" t="s">
         <v>42</v>
       </c>
@@ -11944,7 +12003,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="388" ht="17" spans="1:8">
+    <row r="388" ht="17" hidden="1" spans="1:8">
       <c r="A388" s="8" t="s">
         <v>42</v>
       </c>
@@ -11970,7 +12029,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="389" ht="17" spans="1:8">
+    <row r="389" ht="17" hidden="1" spans="1:8">
       <c r="A389" s="8" t="s">
         <v>42</v>
       </c>
@@ -11996,7 +12055,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="390" ht="17" spans="1:8">
+    <row r="390" ht="17" hidden="1" spans="1:8">
       <c r="A390" s="8" t="s">
         <v>42</v>
       </c>
@@ -12022,7 +12081,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="391" ht="17" spans="1:8">
+    <row r="391" ht="17" hidden="1" spans="1:8">
       <c r="A391" s="8" t="s">
         <v>42</v>
       </c>
@@ -12048,7 +12107,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="392" ht="17" spans="1:8">
+    <row r="392" ht="17" hidden="1" spans="1:8">
       <c r="A392" s="8" t="s">
         <v>42</v>
       </c>
@@ -12074,7 +12133,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="393" spans="1:8">
+    <row r="393" hidden="1" spans="1:8">
       <c r="A393" s="8" t="s">
         <v>42</v>
       </c>
@@ -12088,10 +12147,10 @@
         <v>10</v>
       </c>
       <c r="E393" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F393" s="53">
-        <v>1300</v>
+        <v>800</v>
       </c>
       <c r="G393" s="42">
         <v>46252</v>
@@ -12100,7 +12159,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="394" spans="1:8">
+    <row r="394" hidden="1" spans="1:8">
       <c r="A394" s="8" t="s">
         <v>42</v>
       </c>
@@ -12114,10 +12173,10 @@
         <v>10</v>
       </c>
       <c r="E394" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F394" s="53">
-        <v>1550</v>
+        <v>1300</v>
       </c>
       <c r="G394" s="42">
         <v>46252</v>
@@ -12126,7 +12185,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="395" spans="1:8">
+    <row r="395" hidden="1" spans="1:8">
       <c r="A395" s="8" t="s">
         <v>42</v>
       </c>
@@ -12134,16 +12193,16 @@
         <v>17</v>
       </c>
       <c r="C395" s="10">
-        <v>1880</v>
+        <v>100</v>
       </c>
       <c r="D395" s="9" t="s">
         <v>10</v>
       </c>
       <c r="E395" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F395" s="35">
-        <v>550</v>
+        <v>13</v>
+      </c>
+      <c r="F395" s="53">
+        <v>1550</v>
       </c>
       <c r="G395" s="42">
         <v>46252</v>
@@ -12152,7 +12211,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="396" spans="1:8">
+    <row r="396" hidden="1" spans="1:8">
       <c r="A396" s="8" t="s">
         <v>42</v>
       </c>
@@ -12160,16 +12219,16 @@
         <v>17</v>
       </c>
       <c r="C396" s="10">
-        <v>2880</v>
+        <v>1880</v>
       </c>
       <c r="D396" s="9" t="s">
         <v>10</v>
       </c>
       <c r="E396" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F396" s="33">
-        <v>600</v>
+        <v>11</v>
+      </c>
+      <c r="F396" s="35">
+        <v>550</v>
       </c>
       <c r="G396" s="42">
         <v>46252</v>
@@ -12178,7 +12237,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="397" spans="1:8">
+    <row r="397" hidden="1" spans="1:8">
       <c r="A397" s="8" t="s">
         <v>42</v>
       </c>
@@ -12192,10 +12251,10 @@
         <v>10</v>
       </c>
       <c r="E397" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F397" s="33">
-        <v>650</v>
+        <v>600</v>
       </c>
       <c r="G397" s="42">
         <v>46252</v>
@@ -12204,8 +12263,1287 @@
         <v>46246</v>
       </c>
     </row>
+    <row r="398" hidden="1" spans="1:8">
+      <c r="A398" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B398" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C398" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D398" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E398" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F398" s="33">
+        <v>650</v>
+      </c>
+      <c r="G398" s="42">
+        <v>46252</v>
+      </c>
+      <c r="H398" s="42">
+        <v>46246</v>
+      </c>
+    </row>
+    <row r="399" ht="17" hidden="1" spans="1:8">
+      <c r="A399" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B399" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C399" s="10">
+        <v>0</v>
+      </c>
+      <c r="D399" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E399" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F399" s="46">
+        <v>110</v>
+      </c>
+      <c r="G399" s="42">
+        <v>46254</v>
+      </c>
+      <c r="H399" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="400" ht="17" hidden="1" spans="1:8">
+      <c r="A400" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B400" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C400" s="10">
+        <v>0</v>
+      </c>
+      <c r="D400" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E400" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F400" s="46">
+        <v>900</v>
+      </c>
+      <c r="G400" s="42">
+        <v>46254</v>
+      </c>
+      <c r="H400" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="401" ht="17" hidden="1" spans="1:8">
+      <c r="A401" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B401" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C401" s="10">
+        <v>0</v>
+      </c>
+      <c r="D401" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E401" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F401" s="46">
+        <v>426</v>
+      </c>
+      <c r="G401" s="42">
+        <v>46254</v>
+      </c>
+      <c r="H401" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="402" ht="17" hidden="1" spans="1:8">
+      <c r="A402" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B402" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C402" s="10">
+        <v>100</v>
+      </c>
+      <c r="D402" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E402" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F402" s="54">
+        <v>203</v>
+      </c>
+      <c r="G402" s="42">
+        <v>46254</v>
+      </c>
+      <c r="H402" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="403" ht="17" hidden="1" spans="1:8">
+      <c r="A403" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B403" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C403" s="10">
+        <v>100</v>
+      </c>
+      <c r="D403" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E403" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F403" s="54">
+        <v>2300</v>
+      </c>
+      <c r="G403" s="42">
+        <v>46254</v>
+      </c>
+      <c r="H403" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="404" ht="17" hidden="1" spans="1:8">
+      <c r="A404" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B404" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C404" s="10">
+        <v>100</v>
+      </c>
+      <c r="D404" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E404" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F404" s="54">
+        <v>1750</v>
+      </c>
+      <c r="G404" s="42">
+        <v>46254</v>
+      </c>
+      <c r="H404" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="405" ht="17" hidden="1" spans="1:8">
+      <c r="A405" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B405" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C405" s="22">
+        <v>990</v>
+      </c>
+      <c r="D405" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E405" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F405" s="21">
+        <v>0</v>
+      </c>
+      <c r="G405" s="42">
+        <v>46254</v>
+      </c>
+      <c r="H405" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="406" ht="17" hidden="1" spans="1:8">
+      <c r="A406" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B406" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C406" s="22">
+        <v>990</v>
+      </c>
+      <c r="D406" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E406" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F406" s="46">
+        <v>1091</v>
+      </c>
+      <c r="G406" s="42">
+        <v>46254</v>
+      </c>
+      <c r="H406" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="407" ht="17" hidden="1" spans="1:8">
+      <c r="A407" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B407" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C407" s="22">
+        <v>990</v>
+      </c>
+      <c r="D407" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E407" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F407" s="46">
+        <v>1050</v>
+      </c>
+      <c r="G407" s="42">
+        <v>46254</v>
+      </c>
+      <c r="H407" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="408" ht="17" hidden="1" spans="1:8">
+      <c r="A408" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B408" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C408" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D408" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E408" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F408" s="50">
+        <v>90</v>
+      </c>
+      <c r="G408" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H408" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="409" ht="17" hidden="1" spans="1:8">
+      <c r="A409" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B409" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C409" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D409" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E409" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F409" s="51">
+        <v>230</v>
+      </c>
+      <c r="G409" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H409" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="410" ht="17" hidden="1" spans="1:8">
+      <c r="A410" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B410" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C410" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D410" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E410" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F410" s="51">
+        <v>310</v>
+      </c>
+      <c r="G410" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H410" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="411" ht="17" hidden="1" spans="1:8">
+      <c r="A411" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B411" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C411" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D411" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E411" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F411" s="51">
+        <v>320</v>
+      </c>
+      <c r="G411" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H411" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="412" ht="17" hidden="1" spans="1:8">
+      <c r="A412" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B412" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C412" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D412" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E412" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F412" s="51">
+        <v>350</v>
+      </c>
+      <c r="G412" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H412" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="413" ht="17" hidden="1" spans="1:8">
+      <c r="A413" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B413" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C413" s="10">
+        <v>990</v>
+      </c>
+      <c r="D413" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E413" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F413" s="34">
+        <v>40</v>
+      </c>
+      <c r="G413" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H413" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="414" ht="17" hidden="1" spans="1:8">
+      <c r="A414" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B414" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C414" s="10">
+        <v>990</v>
+      </c>
+      <c r="D414" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E414" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F414" s="34">
+        <v>300</v>
+      </c>
+      <c r="G414" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H414" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="415" ht="17" hidden="1" spans="1:8">
+      <c r="A415" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B415" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C415" s="10">
+        <v>990</v>
+      </c>
+      <c r="D415" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E415" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F415" s="34">
+        <v>230</v>
+      </c>
+      <c r="G415" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H415" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="416" ht="17" hidden="1" spans="1:8">
+      <c r="A416" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B416" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C416" s="10">
+        <v>990</v>
+      </c>
+      <c r="D416" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E416" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F416" s="34">
+        <v>230</v>
+      </c>
+      <c r="G416" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H416" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="417" ht="17" hidden="1" spans="1:8">
+      <c r="A417" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B417" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C417" s="10">
+        <v>0</v>
+      </c>
+      <c r="D417" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E417" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F417" s="38">
+        <v>60</v>
+      </c>
+      <c r="G417" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H417" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="418" ht="17" hidden="1" spans="1:8">
+      <c r="A418" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B418" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C418" s="10">
+        <v>0</v>
+      </c>
+      <c r="D418" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E418" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F418" s="38">
+        <v>180</v>
+      </c>
+      <c r="G418" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H418" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="419" ht="17" hidden="1" spans="1:8">
+      <c r="A419" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B419" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C419" s="10">
+        <v>0</v>
+      </c>
+      <c r="D419" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E419" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F419" s="38">
+        <v>180</v>
+      </c>
+      <c r="G419" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H419" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="420" ht="17" hidden="1" spans="1:8">
+      <c r="A420" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B420" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C420" s="10">
+        <v>0</v>
+      </c>
+      <c r="D420" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E420" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F420" s="38">
+        <v>180</v>
+      </c>
+      <c r="G420" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H420" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="421" ht="17" hidden="1" spans="1:8">
+      <c r="A421" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B421" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C421" s="10">
+        <v>100</v>
+      </c>
+      <c r="D421" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E421" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F421" s="51">
+        <v>1675</v>
+      </c>
+      <c r="G421" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H421" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="422" ht="17" hidden="1" spans="1:8">
+      <c r="A422" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B422" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C422" s="10">
+        <v>100</v>
+      </c>
+      <c r="D422" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E422" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F422" s="51">
+        <v>1875</v>
+      </c>
+      <c r="G422" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H422" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="423" ht="17" hidden="1" spans="1:8">
+      <c r="A423" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B423" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C423" s="10">
+        <v>100</v>
+      </c>
+      <c r="D423" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E423" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F423" s="51">
+        <v>1725</v>
+      </c>
+      <c r="G423" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H423" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="424" ht="17" hidden="1" spans="1:8">
+      <c r="A424" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B424" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C424" s="10">
+        <v>100</v>
+      </c>
+      <c r="D424" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E424" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F424" s="51">
+        <v>1825</v>
+      </c>
+      <c r="G424" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H424" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="425" ht="17" hidden="1" spans="1:8">
+      <c r="A425" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B425" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C425" s="10">
+        <v>990</v>
+      </c>
+      <c r="D425" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E425" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F425" s="41">
+        <v>75</v>
+      </c>
+      <c r="G425" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H425" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="426" ht="17" hidden="1" spans="1:8">
+      <c r="A426" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B426" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C426" s="10">
+        <v>990</v>
+      </c>
+      <c r="D426" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E426" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F426" s="41">
+        <v>75</v>
+      </c>
+      <c r="G426" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H426" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="427" ht="17" hidden="1" spans="1:8">
+      <c r="A427" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B427" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C427" s="10">
+        <v>990</v>
+      </c>
+      <c r="D427" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E427" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F427" s="41">
+        <v>75</v>
+      </c>
+      <c r="G427" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H427" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="428" ht="17" hidden="1" spans="1:8">
+      <c r="A428" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B428" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C428" s="10">
+        <v>990</v>
+      </c>
+      <c r="D428" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E428" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F428" s="41">
+        <v>75</v>
+      </c>
+      <c r="G428" s="42">
+        <v>46253</v>
+      </c>
+      <c r="H428" s="42">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="429" ht="17.55" spans="1:8">
+      <c r="A429" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B429" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C429" s="9">
+        <v>0</v>
+      </c>
+      <c r="D429" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E429" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F429" s="55">
+        <v>200</v>
+      </c>
+      <c r="G429" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H429" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="430" spans="1:8">
+      <c r="A430" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B430" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C430" s="10">
+        <v>0</v>
+      </c>
+      <c r="D430" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E430" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F430" s="55">
+        <v>400</v>
+      </c>
+      <c r="G430" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H430" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="431" spans="1:8">
+      <c r="A431" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B431" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C431" s="10">
+        <v>0</v>
+      </c>
+      <c r="D431" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E431" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F431" s="55">
+        <v>400</v>
+      </c>
+      <c r="G431" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H431" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="432" spans="1:8">
+      <c r="A432" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B432" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C432" s="10">
+        <v>1880</v>
+      </c>
+      <c r="D432" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E432" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F432" s="56">
+        <v>150</v>
+      </c>
+      <c r="G432" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H432" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="433" spans="1:8">
+      <c r="A433" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B433" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C433" s="10">
+        <v>990</v>
+      </c>
+      <c r="D433" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E433" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F433" s="56">
+        <v>700</v>
+      </c>
+      <c r="G433" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H433" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="434" spans="1:8">
+      <c r="A434" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B434" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C434" s="10">
+        <v>990</v>
+      </c>
+      <c r="D434" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E434" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F434" s="56">
+        <v>700</v>
+      </c>
+      <c r="G434" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H434" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="435" spans="1:8">
+      <c r="A435" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B435" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="C435" s="10">
+        <v>100</v>
+      </c>
+      <c r="D435" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E435" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F435" s="56">
+        <v>100</v>
+      </c>
+      <c r="G435" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H435" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="436" spans="1:8">
+      <c r="A436" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B436" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="C436" s="10">
+        <v>100</v>
+      </c>
+      <c r="D436" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E436" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F436" s="56">
+        <v>200</v>
+      </c>
+      <c r="G436" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H436" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="437" spans="1:8">
+      <c r="A437" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B437" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="C437" s="10">
+        <v>100</v>
+      </c>
+      <c r="D437" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E437" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F437" s="56">
+        <v>200</v>
+      </c>
+      <c r="G437" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H437" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="438" ht="17" spans="1:8">
+      <c r="A438" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B438" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C438" s="10">
+        <v>990</v>
+      </c>
+      <c r="D438" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E438" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F438" s="57">
+        <v>200</v>
+      </c>
+      <c r="G438" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H438" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="439" ht="17" spans="1:8">
+      <c r="A439" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B439" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C439" s="10">
+        <v>990</v>
+      </c>
+      <c r="D439" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E439" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F439" s="58">
+        <v>700</v>
+      </c>
+      <c r="G439" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H439" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="440" ht="17" spans="1:8">
+      <c r="A440" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B440" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C440" s="10">
+        <v>990</v>
+      </c>
+      <c r="D440" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E440" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F440" s="58">
+        <v>700</v>
+      </c>
+      <c r="G440" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H440" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="441" ht="17" spans="1:8">
+      <c r="A441" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B441" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C441" s="10">
+        <v>100</v>
+      </c>
+      <c r="D441" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E441" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F441" s="59">
+        <v>750</v>
+      </c>
+      <c r="G441" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H441" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="442" ht="17" spans="1:8">
+      <c r="A442" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B442" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C442" s="10">
+        <v>100</v>
+      </c>
+      <c r="D442" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E442" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F442" s="59">
+        <v>1000</v>
+      </c>
+      <c r="G442" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H442" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="443" ht="17" spans="1:8">
+      <c r="A443" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B443" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C443" s="10">
+        <v>100</v>
+      </c>
+      <c r="D443" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E443" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F443" s="59">
+        <v>1000</v>
+      </c>
+      <c r="G443" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H443" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="444" spans="1:8">
+      <c r="A444" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B444" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C444" s="10">
+        <v>1880</v>
+      </c>
+      <c r="D444" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E444" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F444" s="60">
+        <v>600</v>
+      </c>
+      <c r="G444" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H444" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="445" spans="1:8">
+      <c r="A445" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B445" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C445" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D445" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E445" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F445" s="33">
+        <v>550</v>
+      </c>
+      <c r="G445" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H445" s="42">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="446" spans="1:8">
+      <c r="A446" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B446" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C446" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D446" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E446" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F446" s="33">
+        <v>550</v>
+      </c>
+      <c r="G446" s="42">
+        <v>46259</v>
+      </c>
+      <c r="H446" s="42">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H397" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H446" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="秋_5"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="3">
       <filters>
         <filter val="初中"/>

</xml_diff>

<commit_message>
Add zipin report publishing support
</commit_message>
<xml_diff>
--- a/tongji_target.xlsx
+++ b/tongji_target.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="11140"/>
+    <workbookView windowWidth="28000" windowHeight="11740"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$490</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$532</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1964" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2144" uniqueCount="52">
   <si>
     <t>期次</t>
   </si>
@@ -174,6 +174,18 @@
   </si>
   <si>
     <t>暑_9</t>
+  </si>
+  <si>
+    <t>秋_6</t>
+  </si>
+  <si>
+    <t>暑_17</t>
+  </si>
+  <si>
+    <t>自拼</t>
+  </si>
+  <si>
+    <t>一年级</t>
   </si>
 </sst>
 </file>
@@ -1017,7 +1029,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1545,6 +1557,70 @@
       </extLst>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
@@ -2092,7 +2168,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H490"/>
+  <dimension ref="A1:H535"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.3076923076923" style="3" customWidth="1"/>
@@ -5926,7 +6002,7 @@
         <v>46246</v>
       </c>
     </row>
-    <row r="148" customFormat="1" ht="17.55" spans="1:8">
+    <row r="148" customFormat="1" hidden="1" spans="1:8">
       <c r="A148" s="8" t="s">
         <v>27</v>
       </c>
@@ -5952,7 +6028,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="149" customFormat="1" spans="1:8">
+    <row r="149" customFormat="1" hidden="1" spans="1:8">
       <c r="A149" s="8" t="s">
         <v>27</v>
       </c>
@@ -5978,7 +6054,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="150" customFormat="1" spans="1:8">
+    <row r="150" customFormat="1" hidden="1" spans="1:8">
       <c r="A150" s="8" t="s">
         <v>27</v>
       </c>
@@ -6004,7 +6080,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="151" customFormat="1" spans="1:8">
+    <row r="151" customFormat="1" hidden="1" spans="1:8">
       <c r="A151" s="8" t="s">
         <v>27</v>
       </c>
@@ -6030,7 +6106,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="152" customFormat="1" spans="1:8">
+    <row r="152" customFormat="1" hidden="1" spans="1:8">
       <c r="A152" s="17" t="s">
         <v>27</v>
       </c>
@@ -6056,7 +6132,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="153" customFormat="1" spans="1:8">
+    <row r="153" customFormat="1" hidden="1" spans="1:8">
       <c r="A153" s="17" t="s">
         <v>27</v>
       </c>
@@ -6082,7 +6158,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="154" customFormat="1" ht="17" spans="1:8">
+    <row r="154" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A154" s="17" t="s">
         <v>27</v>
       </c>
@@ -6108,7 +6184,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="155" customFormat="1" ht="17" spans="1:8">
+    <row r="155" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A155" s="17" t="s">
         <v>27</v>
       </c>
@@ -6134,7 +6210,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="156" customFormat="1" ht="17" spans="1:8">
+    <row r="156" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A156" s="17" t="s">
         <v>27</v>
       </c>
@@ -6160,7 +6236,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="157" customFormat="1" ht="17" spans="1:8">
+    <row r="157" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A157" s="17" t="s">
         <v>27</v>
       </c>
@@ -6186,7 +6262,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="158" customFormat="1" ht="17" spans="1:8">
+    <row r="158" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A158" s="17" t="s">
         <v>27</v>
       </c>
@@ -6212,7 +6288,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="159" customFormat="1" ht="17" spans="1:8">
+    <row r="159" customFormat="1" ht="17" hidden="1" spans="1:8">
       <c r="A159" s="17" t="s">
         <v>27</v>
       </c>
@@ -6238,7 +6314,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="160" customFormat="1" spans="1:8">
+    <row r="160" customFormat="1" hidden="1" spans="1:8">
       <c r="A160" s="17" t="s">
         <v>27</v>
       </c>
@@ -6264,7 +6340,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="161" customFormat="1" spans="1:8">
+    <row r="161" customFormat="1" hidden="1" spans="1:8">
       <c r="A161" s="17" t="s">
         <v>27</v>
       </c>
@@ -6290,7 +6366,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="162" customFormat="1" spans="1:8">
+    <row r="162" customFormat="1" hidden="1" spans="1:8">
       <c r="A162" s="17" t="s">
         <v>27</v>
       </c>
@@ -6316,7 +6392,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="163" customFormat="1" spans="1:8">
+    <row r="163" customFormat="1" hidden="1" spans="1:8">
       <c r="A163" s="17" t="s">
         <v>27</v>
       </c>
@@ -6342,7 +6418,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="164" customFormat="1" spans="1:8">
+    <row r="164" customFormat="1" hidden="1" spans="1:8">
       <c r="A164" s="17" t="s">
         <v>27</v>
       </c>
@@ -6368,7 +6444,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="165" customFormat="1" spans="1:8">
+    <row r="165" customFormat="1" hidden="1" spans="1:8">
       <c r="A165" s="17" t="s">
         <v>27</v>
       </c>
@@ -14766,7 +14842,7 @@
         <v>46254</v>
       </c>
     </row>
-    <row r="488" ht="17" spans="1:8">
+    <row r="488" ht="17" hidden="1" spans="1:8">
       <c r="A488" s="17" t="s">
         <v>27</v>
       </c>
@@ -14792,7 +14868,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="489" ht="17" spans="1:8">
+    <row r="489" ht="17" hidden="1" spans="1:8">
       <c r="A489" s="17" t="s">
         <v>27</v>
       </c>
@@ -14818,7 +14894,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="490" ht="17" spans="1:8">
+    <row r="490" ht="17" hidden="1" spans="1:8">
       <c r="A490" s="17" t="s">
         <v>27</v>
       </c>
@@ -14844,21 +14920,1188 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="491" hidden="1" spans="1:8">
+      <c r="A491" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B491" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C491" s="10">
+        <v>0</v>
+      </c>
+      <c r="D491" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E491" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F491" s="78">
+        <v>200</v>
+      </c>
+      <c r="G491" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H491" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="492" hidden="1" spans="1:8">
+      <c r="A492" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B492" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C492" s="10">
+        <v>0</v>
+      </c>
+      <c r="D492" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E492" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F492" s="78">
+        <v>400</v>
+      </c>
+      <c r="G492" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H492" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="493" hidden="1" spans="1:8">
+      <c r="A493" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B493" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C493" s="10">
+        <v>0</v>
+      </c>
+      <c r="D493" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E493" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F493" s="78">
+        <v>400</v>
+      </c>
+      <c r="G493" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H493" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="494" ht="17" hidden="1" spans="1:8">
+      <c r="A494" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B494" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C494" s="10">
+        <v>1880</v>
+      </c>
+      <c r="D494" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E494" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F494" s="79">
+        <v>200</v>
+      </c>
+      <c r="G494" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H494" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="495" ht="17" hidden="1" spans="1:8">
+      <c r="A495" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B495" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C495" s="10">
+        <v>990</v>
+      </c>
+      <c r="D495" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E495" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F495" s="79">
+        <v>700</v>
+      </c>
+      <c r="G495" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H495" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="496" ht="17" hidden="1" spans="1:8">
+      <c r="A496" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B496" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C496" s="10">
+        <v>990</v>
+      </c>
+      <c r="D496" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E496" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F496" s="79">
+        <v>700</v>
+      </c>
+      <c r="G496" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H496" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="497" ht="17" hidden="1" spans="1:8">
+      <c r="A497" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B497" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C497" s="10">
+        <v>100</v>
+      </c>
+      <c r="D497" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E497" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F497" s="79">
+        <v>450</v>
+      </c>
+      <c r="G497" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H497" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="498" ht="17" hidden="1" spans="1:8">
+      <c r="A498" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B498" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C498" s="10">
+        <v>100</v>
+      </c>
+      <c r="D498" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E498" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F498" s="79">
+        <v>1000</v>
+      </c>
+      <c r="G498" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H498" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="499" ht="17" hidden="1" spans="1:8">
+      <c r="A499" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B499" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C499" s="10">
+        <v>100</v>
+      </c>
+      <c r="D499" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E499" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F499" s="79">
+        <v>1000</v>
+      </c>
+      <c r="G499" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H499" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="500" ht="17" hidden="1" spans="1:8">
+      <c r="A500" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B500" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C500" s="10">
+        <v>990</v>
+      </c>
+      <c r="D500" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E500" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F500" s="80">
+        <v>200</v>
+      </c>
+      <c r="G500" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H500" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="501" ht="17" hidden="1" spans="1:8">
+      <c r="A501" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B501" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C501" s="10">
+        <v>990</v>
+      </c>
+      <c r="D501" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E501" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F501" s="81">
+        <v>500</v>
+      </c>
+      <c r="G501" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H501" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="502" ht="17" hidden="1" spans="1:8">
+      <c r="A502" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B502" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C502" s="10">
+        <v>990</v>
+      </c>
+      <c r="D502" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E502" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F502" s="81">
+        <v>500</v>
+      </c>
+      <c r="G502" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H502" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="503" hidden="1" spans="1:8">
+      <c r="A503" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B503" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C503" s="10">
+        <v>100</v>
+      </c>
+      <c r="D503" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E503" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F503" s="82">
+        <v>650</v>
+      </c>
+      <c r="G503" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H503" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="504" hidden="1" spans="1:8">
+      <c r="A504" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B504" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C504" s="10">
+        <v>100</v>
+      </c>
+      <c r="D504" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E504" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F504" s="82">
+        <v>550</v>
+      </c>
+      <c r="G504" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H504" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="505" hidden="1" spans="1:8">
+      <c r="A505" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B505" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C505" s="10">
+        <v>100</v>
+      </c>
+      <c r="D505" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E505" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F505" s="82">
+        <v>550</v>
+      </c>
+      <c r="G505" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H505" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="506" hidden="1" spans="1:8">
+      <c r="A506" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B506" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C506" s="10">
+        <v>1880</v>
+      </c>
+      <c r="D506" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E506" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F506" s="41">
+        <v>450</v>
+      </c>
+      <c r="G506" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H506" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="507" hidden="1" spans="1:8">
+      <c r="A507" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B507" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C507" s="32">
+        <v>2880</v>
+      </c>
+      <c r="D507" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E507" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F507" s="83">
+        <v>300</v>
+      </c>
+      <c r="G507" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H507" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="508" hidden="1" spans="1:8">
+      <c r="A508" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B508" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C508" s="32">
+        <v>2880</v>
+      </c>
+      <c r="D508" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E508" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F508" s="83">
+        <v>450</v>
+      </c>
+      <c r="G508" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H508" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="509" ht="17" hidden="1" spans="1:8">
+      <c r="A509" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B509" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C509" s="10">
+        <v>100</v>
+      </c>
+      <c r="D509" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E509" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F509" s="84">
+        <v>200</v>
+      </c>
+      <c r="G509" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H509" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="510" ht="17" hidden="1" spans="1:8">
+      <c r="A510" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B510" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C510" s="10">
+        <v>100</v>
+      </c>
+      <c r="D510" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E510" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F510" s="84">
+        <v>150</v>
+      </c>
+      <c r="G510" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H510" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="511" ht="17" hidden="1" spans="1:8">
+      <c r="A511" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B511" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C511" s="10">
+        <v>100</v>
+      </c>
+      <c r="D511" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E511" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F511" s="84">
+        <v>150</v>
+      </c>
+      <c r="G511" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H511" s="43">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="512" ht="17.75" spans="1:8">
+      <c r="A512" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B512" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C512" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D512" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E512" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="F512" s="80">
+        <v>100</v>
+      </c>
+      <c r="G512" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H512" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="513" ht="17" spans="1:8">
+      <c r="A513" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B513" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C513" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D513" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E513" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F513" s="81">
+        <v>250</v>
+      </c>
+      <c r="G513" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H513" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="514" ht="17" spans="1:8">
+      <c r="A514" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B514" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C514" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D514" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E514" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F514" s="81">
+        <v>250</v>
+      </c>
+      <c r="G514" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H514" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="515" ht="17" spans="1:8">
+      <c r="A515" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B515" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C515" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D515" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E515" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F515" s="81">
+        <v>250</v>
+      </c>
+      <c r="G515" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H515" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="516" ht="17" spans="1:8">
+      <c r="A516" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B516" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C516" s="10">
+        <v>2880</v>
+      </c>
+      <c r="D516" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E516" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F516" s="81">
+        <v>250</v>
+      </c>
+      <c r="G516" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H516" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="517" ht="17" spans="1:8">
+      <c r="A517" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B517" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C517" s="10">
+        <v>990</v>
+      </c>
+      <c r="D517" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E517" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F517" s="85">
+        <v>40</v>
+      </c>
+      <c r="G517" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H517" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="518" ht="17" spans="1:8">
+      <c r="A518" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B518" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C518" s="10">
+        <v>990</v>
+      </c>
+      <c r="D518" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E518" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F518" s="85">
+        <v>300</v>
+      </c>
+      <c r="G518" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H518" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="519" ht="17" spans="1:8">
+      <c r="A519" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B519" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C519" s="10">
+        <v>990</v>
+      </c>
+      <c r="D519" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E519" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F519" s="85">
+        <v>230</v>
+      </c>
+      <c r="G519" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H519" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="520" ht="17" spans="1:8">
+      <c r="A520" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B520" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C520" s="10">
+        <v>990</v>
+      </c>
+      <c r="D520" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E520" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F520" s="85">
+        <v>230</v>
+      </c>
+      <c r="G520" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H520" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="521" ht="17" spans="1:8">
+      <c r="A521" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B521" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C521" s="10">
+        <v>0</v>
+      </c>
+      <c r="D521" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E521" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F521" s="84">
+        <v>90</v>
+      </c>
+      <c r="G521" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H521" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="522" ht="17" spans="1:8">
+      <c r="A522" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B522" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C522" s="10">
+        <v>0</v>
+      </c>
+      <c r="D522" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E522" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F522" s="84">
+        <v>200</v>
+      </c>
+      <c r="G522" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H522" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="523" ht="17" spans="1:8">
+      <c r="A523" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B523" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C523" s="10">
+        <v>0</v>
+      </c>
+      <c r="D523" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E523" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F523" s="84">
+        <v>180</v>
+      </c>
+      <c r="G523" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H523" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="524" ht="17" spans="1:8">
+      <c r="A524" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B524" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C524" s="10">
+        <v>0</v>
+      </c>
+      <c r="D524" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E524" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F524" s="84">
+        <v>180</v>
+      </c>
+      <c r="G524" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H524" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="525" ht="17" spans="1:8">
+      <c r="A525" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B525" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C525" s="10">
+        <v>100</v>
+      </c>
+      <c r="D525" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E525" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F525" s="85">
+        <v>900</v>
+      </c>
+      <c r="G525" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H525" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="526" ht="17" spans="1:8">
+      <c r="A526" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B526" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C526" s="10">
+        <v>100</v>
+      </c>
+      <c r="D526" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E526" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F526" s="85">
+        <v>1100</v>
+      </c>
+      <c r="G526" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H526" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="527" ht="17" spans="1:8">
+      <c r="A527" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B527" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C527" s="10">
+        <v>100</v>
+      </c>
+      <c r="D527" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E527" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F527" s="85">
+        <v>900</v>
+      </c>
+      <c r="G527" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H527" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="528" ht="17" spans="1:8">
+      <c r="A528" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B528" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C528" s="10">
+        <v>100</v>
+      </c>
+      <c r="D528" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E528" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F528" s="85">
+        <v>1000</v>
+      </c>
+      <c r="G528" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H528" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="529" ht="17" spans="1:8">
+      <c r="A529" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B529" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C529" s="10">
+        <v>990</v>
+      </c>
+      <c r="D529" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E529" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F529" s="80">
+        <v>100</v>
+      </c>
+      <c r="G529" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H529" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="530" ht="17" spans="1:8">
+      <c r="A530" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B530" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C530" s="10">
+        <v>990</v>
+      </c>
+      <c r="D530" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E530" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F530" s="80">
+        <v>100</v>
+      </c>
+      <c r="G530" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H530" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="531" ht="17" spans="1:8">
+      <c r="A531" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B531" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C531" s="10">
+        <v>990</v>
+      </c>
+      <c r="D531" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E531" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F531" s="80">
+        <v>100</v>
+      </c>
+      <c r="G531" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H531" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="532" ht="17" spans="1:8">
+      <c r="A532" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B532" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C532" s="10">
+        <v>990</v>
+      </c>
+      <c r="D532" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E532" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F532" s="80">
+        <v>100</v>
+      </c>
+      <c r="G532" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H532" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="533" ht="17" spans="1:8">
+      <c r="A533" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B533" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C533" s="10">
+        <v>990</v>
+      </c>
+      <c r="D533" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E533" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F533" s="79">
+        <v>700</v>
+      </c>
+      <c r="G533" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H533" s="43">
+        <v>46259</v>
+      </c>
+    </row>
+    <row r="534" ht="17" spans="1:8">
+      <c r="A534" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B534" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C534" s="10">
+        <v>990</v>
+      </c>
+      <c r="D534" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E534" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F534" s="79">
+        <v>200</v>
+      </c>
+      <c r="G534" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H534" s="43">
+        <v>46259</v>
+      </c>
+    </row>
+    <row r="535" ht="17" spans="1:8">
+      <c r="A535" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B535" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C535" s="10">
+        <v>990</v>
+      </c>
+      <c r="D535" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E535" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F535" s="79">
+        <v>100</v>
+      </c>
+      <c r="G535" s="43">
+        <v>46266</v>
+      </c>
+      <c r="H535" s="43">
+        <v>46259</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H490" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H532" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
       <filters>
-        <filter val="秋_5"/>
+        <filter val="暑_17"/>
       </filters>
     </filterColumn>
     <filterColumn colId="3">
       <filters>
-        <filter val="初中"/>
+        <filter val="小学"/>
       </filters>
     </filterColumn>
-    <sortState ref="A1:H490">
-      <sortCondition ref="D1"/>
-    </sortState>
     <extLst/>
   </autoFilter>
   <sortState ref="A2:F79">

</xml_diff>

<commit_message>
Update dashboard filters and data
</commit_message>
<xml_diff>
--- a/tongji_target.xlsx
+++ b/tongji_target.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$532</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$552</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2144" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2224" uniqueCount="52">
   <si>
     <t>期次</t>
   </si>
@@ -1029,7 +1029,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1628,6 +1628,22 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2168,7 +2184,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H535"/>
+  <dimension ref="A1:H555"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.3076923076923" style="3" customWidth="1"/>
@@ -15466,7 +15482,7 @@
         <v>46260</v>
       </c>
     </row>
-    <row r="512" ht="17.75" spans="1:8">
+    <row r="512" ht="17" hidden="1" spans="1:8">
       <c r="A512" s="17" t="s">
         <v>49</v>
       </c>
@@ -15492,7 +15508,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="513" ht="17" spans="1:8">
+    <row r="513" ht="17" hidden="1" spans="1:8">
       <c r="A513" s="17" t="s">
         <v>49</v>
       </c>
@@ -15518,7 +15534,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="514" ht="17" spans="1:8">
+    <row r="514" ht="17" hidden="1" spans="1:8">
       <c r="A514" s="17" t="s">
         <v>49</v>
       </c>
@@ -15544,7 +15560,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="515" ht="17" spans="1:8">
+    <row r="515" ht="17" hidden="1" spans="1:8">
       <c r="A515" s="17" t="s">
         <v>49</v>
       </c>
@@ -15570,7 +15586,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="516" ht="17" spans="1:8">
+    <row r="516" ht="17" hidden="1" spans="1:8">
       <c r="A516" s="17" t="s">
         <v>49</v>
       </c>
@@ -15596,7 +15612,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="517" ht="17" spans="1:8">
+    <row r="517" ht="17" hidden="1" spans="1:8">
       <c r="A517" s="17" t="s">
         <v>49</v>
       </c>
@@ -15622,7 +15638,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="518" ht="17" spans="1:8">
+    <row r="518" ht="17" hidden="1" spans="1:8">
       <c r="A518" s="17" t="s">
         <v>49</v>
       </c>
@@ -15648,7 +15664,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="519" ht="17" spans="1:8">
+    <row r="519" ht="17" hidden="1" spans="1:8">
       <c r="A519" s="17" t="s">
         <v>49</v>
       </c>
@@ -15674,7 +15690,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="520" ht="17" spans="1:8">
+    <row r="520" ht="17" hidden="1" spans="1:8">
       <c r="A520" s="17" t="s">
         <v>49</v>
       </c>
@@ -15700,7 +15716,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="521" ht="17" spans="1:8">
+    <row r="521" ht="17" hidden="1" spans="1:8">
       <c r="A521" s="17" t="s">
         <v>49</v>
       </c>
@@ -15726,7 +15742,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="522" ht="17" spans="1:8">
+    <row r="522" ht="17" hidden="1" spans="1:8">
       <c r="A522" s="17" t="s">
         <v>49</v>
       </c>
@@ -15752,7 +15768,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="523" ht="17" spans="1:8">
+    <row r="523" ht="17" hidden="1" spans="1:8">
       <c r="A523" s="17" t="s">
         <v>49</v>
       </c>
@@ -15778,7 +15794,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="524" ht="17" spans="1:8">
+    <row r="524" ht="17" hidden="1" spans="1:8">
       <c r="A524" s="17" t="s">
         <v>49</v>
       </c>
@@ -15804,7 +15820,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="525" ht="17" spans="1:8">
+    <row r="525" ht="17" hidden="1" spans="1:8">
       <c r="A525" s="17" t="s">
         <v>49</v>
       </c>
@@ -15830,7 +15846,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="526" ht="17" spans="1:8">
+    <row r="526" ht="17" hidden="1" spans="1:8">
       <c r="A526" s="17" t="s">
         <v>49</v>
       </c>
@@ -15856,7 +15872,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="527" ht="17" spans="1:8">
+    <row r="527" ht="17" hidden="1" spans="1:8">
       <c r="A527" s="17" t="s">
         <v>49</v>
       </c>
@@ -15882,7 +15898,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="528" ht="17" spans="1:8">
+    <row r="528" ht="17" hidden="1" spans="1:8">
       <c r="A528" s="17" t="s">
         <v>49</v>
       </c>
@@ -15908,7 +15924,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="529" ht="17" spans="1:8">
+    <row r="529" ht="17" hidden="1" spans="1:8">
       <c r="A529" s="17" t="s">
         <v>49</v>
       </c>
@@ -15934,7 +15950,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="530" ht="17" spans="1:8">
+    <row r="530" ht="17" hidden="1" spans="1:8">
       <c r="A530" s="17" t="s">
         <v>49</v>
       </c>
@@ -15960,7 +15976,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="531" ht="17" spans="1:8">
+    <row r="531" ht="17" hidden="1" spans="1:8">
       <c r="A531" s="17" t="s">
         <v>49</v>
       </c>
@@ -15986,7 +16002,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="532" ht="17" spans="1:8">
+    <row r="532" ht="17" hidden="1" spans="1:8">
       <c r="A532" s="17" t="s">
         <v>49</v>
       </c>
@@ -16012,7 +16028,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="533" ht="17" spans="1:8">
+    <row r="533" ht="17" hidden="1" spans="1:8">
       <c r="A533" s="17" t="s">
         <v>49</v>
       </c>
@@ -16038,7 +16054,7 @@
         <v>46259</v>
       </c>
     </row>
-    <row r="534" ht="17" spans="1:8">
+    <row r="534" ht="17" hidden="1" spans="1:8">
       <c r="A534" s="17" t="s">
         <v>49</v>
       </c>
@@ -16064,7 +16080,7 @@
         <v>46259</v>
       </c>
     </row>
-    <row r="535" ht="17" spans="1:8">
+    <row r="535" ht="17" hidden="1" spans="1:8">
       <c r="A535" s="17" t="s">
         <v>49</v>
       </c>
@@ -16090,16 +16106,536 @@
         <v>46259</v>
       </c>
     </row>
+    <row r="536" ht="17.75" spans="1:8">
+      <c r="A536" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B536" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C536" s="10">
+        <v>0</v>
+      </c>
+      <c r="D536" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E536" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F536" s="86">
+        <v>140</v>
+      </c>
+      <c r="G536" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H536" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="537" ht="17" spans="1:8">
+      <c r="A537" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B537" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C537" s="10">
+        <v>0</v>
+      </c>
+      <c r="D537" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E537" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F537" s="86">
+        <v>500</v>
+      </c>
+      <c r="G537" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H537" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="538" ht="17" spans="1:8">
+      <c r="A538" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B538" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C538" s="10">
+        <v>0</v>
+      </c>
+      <c r="D538" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E538" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F538" s="86">
+        <v>600</v>
+      </c>
+      <c r="G538" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H538" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="539" ht="17" spans="1:8">
+      <c r="A539" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B539" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C539" s="10">
+        <v>100</v>
+      </c>
+      <c r="D539" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E539" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F539" s="86">
+        <v>125</v>
+      </c>
+      <c r="G539" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H539" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="540" ht="17" spans="1:8">
+      <c r="A540" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B540" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C540" s="10">
+        <v>100</v>
+      </c>
+      <c r="D540" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E540" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F540" s="86">
+        <v>1500</v>
+      </c>
+      <c r="G540" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H540" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="541" ht="17" spans="1:8">
+      <c r="A541" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B541" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C541" s="10">
+        <v>100</v>
+      </c>
+      <c r="D541" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E541" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F541" s="86">
+        <v>1200</v>
+      </c>
+      <c r="G541" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H541" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="542" ht="17" spans="1:8">
+      <c r="A542" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B542" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C542" s="10">
+        <v>100</v>
+      </c>
+      <c r="D542" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E542" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F542" s="86">
+        <v>100</v>
+      </c>
+      <c r="G542" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H542" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="543" ht="17" spans="1:8">
+      <c r="A543" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B543" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C543" s="10">
+        <v>100</v>
+      </c>
+      <c r="D543" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E543" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F543" s="86">
+        <v>370</v>
+      </c>
+      <c r="G543" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H543" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="544" ht="17" spans="1:8">
+      <c r="A544" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B544" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C544" s="10">
+        <v>100</v>
+      </c>
+      <c r="D544" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E544" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F544" s="86">
+        <v>100</v>
+      </c>
+      <c r="G544" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H544" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="545" ht="17" spans="1:8">
+      <c r="A545" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B545" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C545" s="10">
+        <v>990</v>
+      </c>
+      <c r="D545" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E545" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F545" s="15">
+        <v>0</v>
+      </c>
+      <c r="G545" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H545" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="546" ht="17" spans="1:8">
+      <c r="A546" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B546" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C546" s="10">
+        <v>990</v>
+      </c>
+      <c r="D546" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E546" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F546" s="86">
+        <v>500</v>
+      </c>
+      <c r="G546" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H546" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="547" ht="17" spans="1:8">
+      <c r="A547" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B547" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C547" s="10">
+        <v>990</v>
+      </c>
+      <c r="D547" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E547" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F547" s="86">
+        <v>600</v>
+      </c>
+      <c r="G547" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H547" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="548" ht="17" spans="1:8">
+      <c r="A548" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B548" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C548" s="10">
+        <v>0</v>
+      </c>
+      <c r="D548" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E548" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F548" s="87">
+        <v>100</v>
+      </c>
+      <c r="G548" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H548" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="549" ht="17" spans="1:8">
+      <c r="A549" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B549" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C549" s="10">
+        <v>0</v>
+      </c>
+      <c r="D549" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E549" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F549" s="87">
+        <v>100</v>
+      </c>
+      <c r="G549" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H549" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="550" ht="17" spans="1:8">
+      <c r="A550" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B550" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C550" s="10">
+        <v>0</v>
+      </c>
+      <c r="D550" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E550" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F550" s="87">
+        <v>100</v>
+      </c>
+      <c r="G550" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H550" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="551" ht="17" spans="1:8">
+      <c r="A551" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B551" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C551" s="10">
+        <v>1880</v>
+      </c>
+      <c r="D551" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E551" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F551" s="86">
+        <v>650</v>
+      </c>
+      <c r="G551" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H551" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="552" ht="17" spans="1:8">
+      <c r="A552" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B552" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C552" s="10">
+        <v>1880</v>
+      </c>
+      <c r="D552" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E552" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F552" s="86">
+        <v>550</v>
+      </c>
+      <c r="G552" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H552" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="553" ht="17" spans="1:8">
+      <c r="A553" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B553" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C553" s="10">
+        <v>100</v>
+      </c>
+      <c r="D553" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E553" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F553" s="15">
+        <v>0</v>
+      </c>
+      <c r="G553" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H553" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="554" ht="17" spans="1:8">
+      <c r="A554" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B554" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C554" s="10">
+        <v>100</v>
+      </c>
+      <c r="D554" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E554" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F554" s="86">
+        <v>200</v>
+      </c>
+      <c r="G554" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H554" s="43">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="555" ht="17" spans="1:8">
+      <c r="A555" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B555" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C555" s="10">
+        <v>100</v>
+      </c>
+      <c r="D555" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E555" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F555" s="86">
+        <v>300</v>
+      </c>
+      <c r="G555" s="43">
+        <v>46267</v>
+      </c>
+      <c r="H555" s="43">
+        <v>46261</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H532" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H552" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
       <filters>
-        <filter val="暑_17"/>
+        <filter val="秋_4"/>
       </filters>
     </filterColumn>
     <filterColumn colId="3">
       <filters>
-        <filter val="小学"/>
+        <filter val="高中"/>
       </filters>
     </filterColumn>
     <extLst/>

</xml_diff>